<commit_message>
feat: integrate microcredit 0.9.4 updates
</commit_message>
<xml_diff>
--- a/assets/modelo_consulta_lote.xlsx
+++ b/assets/modelo_consulta_lote.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultas" sheetId="1" r:id="R384b169ef2f740f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" r:id="R75c0191f12d04e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultas" sheetId="1" r:id="R33e1b5d7b903427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" r:id="Rb3cf97369ee24a52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -69,14 +69,39 @@
         <x:fgColor rgb="FFEDF5F1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF165C41"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFB7DEE8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF5F1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF3DB7E9"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -109,6 +134,49 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -331,8 +399,10 @@
     <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="49" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -346,9 +416,15 @@
         <x:v>PROPRIETARIO_POSSUIDOR</x:v>
       </x:c>
       <x:c r="D1" s="7" t="str">
+        <x:v>FONTE_RECURSOS</x:v>
+      </x:c>
+      <x:c r="E1" s="7" t="str">
+        <x:v>LINHA_CREDITO</x:v>
+      </x:c>
+      <x:c r="F1" s="21" t="str">
         <x:v>REFERENCIA_INTERNA</x:v>
       </x:c>
-      <x:c r="E1" s="7" t="str">
+      <x:c r="G1" s="21" t="str">
         <x:v>OBSERVACAO</x:v>
       </x:c>
     </x:row>
@@ -358,6 +434,8 @@
       <x:c r="C2" s="9" t="str"/>
       <x:c r="D2" s="9" t="str"/>
       <x:c r="E2" s="9" t="str"/>
+      <x:c r="F2" s="25"/>
+      <x:c r="G2" s="25"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8"/>
@@ -365,6 +443,8 @@
       <x:c r="C3" s="9"/>
       <x:c r="D3" s="9"/>
       <x:c r="E3" s="9"/>
+      <x:c r="F3" s="29"/>
+      <x:c r="G3" s="29"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="8"/>
@@ -372,6 +452,8 @@
       <x:c r="C4" s="9"/>
       <x:c r="D4" s="9"/>
       <x:c r="E4" s="9"/>
+      <x:c r="F4" s="25"/>
+      <x:c r="G4" s="25"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8"/>
@@ -379,6 +461,8 @@
       <x:c r="C5" s="9"/>
       <x:c r="D5" s="9"/>
       <x:c r="E5" s="9"/>
+      <x:c r="F5" s="29"/>
+      <x:c r="G5" s="29"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8"/>
@@ -386,6 +470,8 @@
       <x:c r="C6" s="9"/>
       <x:c r="D6" s="9"/>
       <x:c r="E6" s="9"/>
+      <x:c r="F6" s="25"/>
+      <x:c r="G6" s="25"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="8"/>
@@ -393,6 +479,8 @@
       <x:c r="C7" s="9"/>
       <x:c r="D7" s="9"/>
       <x:c r="E7" s="9"/>
+      <x:c r="F7" s="29"/>
+      <x:c r="G7" s="29"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="8"/>
@@ -400,6 +488,8 @@
       <x:c r="C8" s="9"/>
       <x:c r="D8" s="9"/>
       <x:c r="E8" s="9"/>
+      <x:c r="F8" s="25"/>
+      <x:c r="G8" s="25"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="8"/>
@@ -407,6 +497,8 @@
       <x:c r="C9" s="9"/>
       <x:c r="D9" s="9"/>
       <x:c r="E9" s="9"/>
+      <x:c r="F9" s="29"/>
+      <x:c r="G9" s="29"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8"/>
@@ -414,6 +506,8 @@
       <x:c r="C10" s="9"/>
       <x:c r="D10" s="9"/>
       <x:c r="E10" s="9"/>
+      <x:c r="F10" s="25"/>
+      <x:c r="G10" s="25"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8"/>
@@ -421,6 +515,8 @@
       <x:c r="C11" s="9"/>
       <x:c r="D11" s="9"/>
       <x:c r="E11" s="9"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8"/>
@@ -428,6 +524,8 @@
       <x:c r="C12" s="9"/>
       <x:c r="D12" s="9"/>
       <x:c r="E12" s="9"/>
+      <x:c r="F12" s="25"/>
+      <x:c r="G12" s="25"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8"/>
@@ -435,6 +533,8 @@
       <x:c r="C13" s="9"/>
       <x:c r="D13" s="9"/>
       <x:c r="E13" s="9"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8"/>
@@ -442,6 +542,8 @@
       <x:c r="C14" s="9"/>
       <x:c r="D14" s="9"/>
       <x:c r="E14" s="9"/>
+      <x:c r="F14" s="25"/>
+      <x:c r="G14" s="25"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8"/>
@@ -449,6 +551,8 @@
       <x:c r="C15" s="9"/>
       <x:c r="D15" s="9"/>
       <x:c r="E15" s="9"/>
+      <x:c r="F15" s="29"/>
+      <x:c r="G15" s="29"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8"/>
@@ -456,6 +560,8 @@
       <x:c r="C16" s="9"/>
       <x:c r="D16" s="9"/>
       <x:c r="E16" s="9"/>
+      <x:c r="F16" s="25"/>
+      <x:c r="G16" s="25"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8"/>
@@ -463,6 +569,8 @@
       <x:c r="C17" s="9"/>
       <x:c r="D17" s="9"/>
       <x:c r="E17" s="9"/>
+      <x:c r="F17" s="29"/>
+      <x:c r="G17" s="29"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8"/>
@@ -470,6 +578,8 @@
       <x:c r="C18" s="9"/>
       <x:c r="D18" s="9"/>
       <x:c r="E18" s="9"/>
+      <x:c r="F18" s="25"/>
+      <x:c r="G18" s="25"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8"/>
@@ -477,6 +587,8 @@
       <x:c r="C19" s="9"/>
       <x:c r="D19" s="9"/>
       <x:c r="E19" s="9"/>
+      <x:c r="F19" s="29"/>
+      <x:c r="G19" s="29"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8"/>
@@ -484,6 +596,8 @@
       <x:c r="C20" s="9"/>
       <x:c r="D20" s="9"/>
       <x:c r="E20" s="9"/>
+      <x:c r="F20" s="25"/>
+      <x:c r="G20" s="25"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="8"/>
@@ -491,6 +605,8 @@
       <x:c r="C21" s="9"/>
       <x:c r="D21" s="9"/>
       <x:c r="E21" s="9"/>
+      <x:c r="F21" s="29"/>
+      <x:c r="G21" s="29"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="8"/>
@@ -498,6 +614,8 @@
       <x:c r="C22" s="9"/>
       <x:c r="D22" s="9"/>
       <x:c r="E22" s="9"/>
+      <x:c r="F22" s="25"/>
+      <x:c r="G22" s="25"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="8"/>
@@ -505,6 +623,8 @@
       <x:c r="C23" s="9"/>
       <x:c r="D23" s="9"/>
       <x:c r="E23" s="9"/>
+      <x:c r="F23" s="29"/>
+      <x:c r="G23" s="29"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="8"/>
@@ -512,6 +632,8 @@
       <x:c r="C24" s="9"/>
       <x:c r="D24" s="9"/>
       <x:c r="E24" s="9"/>
+      <x:c r="F24" s="25"/>
+      <x:c r="G24" s="25"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="8"/>
@@ -519,6 +641,8 @@
       <x:c r="C25" s="9"/>
       <x:c r="D25" s="9"/>
       <x:c r="E25" s="9"/>
+      <x:c r="F25" s="29"/>
+      <x:c r="G25" s="29"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="8"/>
@@ -526,6 +650,8 @@
       <x:c r="C26" s="9"/>
       <x:c r="D26" s="9"/>
       <x:c r="E26" s="9"/>
+      <x:c r="F26" s="25"/>
+      <x:c r="G26" s="25"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="8"/>
@@ -533,6 +659,8 @@
       <x:c r="C27" s="9"/>
       <x:c r="D27" s="9"/>
       <x:c r="E27" s="9"/>
+      <x:c r="F27" s="29"/>
+      <x:c r="G27" s="29"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="8"/>
@@ -540,6 +668,8 @@
       <x:c r="C28" s="9"/>
       <x:c r="D28" s="9"/>
       <x:c r="E28" s="9"/>
+      <x:c r="F28" s="25"/>
+      <x:c r="G28" s="25"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="8"/>
@@ -547,6 +677,8 @@
       <x:c r="C29" s="9"/>
       <x:c r="D29" s="9"/>
       <x:c r="E29" s="9"/>
+      <x:c r="F29" s="29"/>
+      <x:c r="G29" s="29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="8"/>
@@ -554,6 +686,8 @@
       <x:c r="C30" s="9"/>
       <x:c r="D30" s="9"/>
       <x:c r="E30" s="9"/>
+      <x:c r="F30" s="25"/>
+      <x:c r="G30" s="25"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="8"/>
@@ -561,6 +695,8 @@
       <x:c r="C31" s="9"/>
       <x:c r="D31" s="9"/>
       <x:c r="E31" s="9"/>
+      <x:c r="F31" s="29"/>
+      <x:c r="G31" s="29"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="8"/>
@@ -568,6 +704,8 @@
       <x:c r="C32" s="9"/>
       <x:c r="D32" s="9"/>
       <x:c r="E32" s="9"/>
+      <x:c r="F32" s="25"/>
+      <x:c r="G32" s="25"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="8"/>
@@ -575,6 +713,8 @@
       <x:c r="C33" s="9"/>
       <x:c r="D33" s="9"/>
       <x:c r="E33" s="9"/>
+      <x:c r="F33" s="29"/>
+      <x:c r="G33" s="29"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="8"/>
@@ -582,6 +722,8 @@
       <x:c r="C34" s="9"/>
       <x:c r="D34" s="9"/>
       <x:c r="E34" s="9"/>
+      <x:c r="F34" s="25"/>
+      <x:c r="G34" s="25"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="8"/>
@@ -589,6 +731,8 @@
       <x:c r="C35" s="9"/>
       <x:c r="D35" s="9"/>
       <x:c r="E35" s="9"/>
+      <x:c r="F35" s="29"/>
+      <x:c r="G35" s="29"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="8"/>
@@ -596,6 +740,8 @@
       <x:c r="C36" s="9"/>
       <x:c r="D36" s="9"/>
       <x:c r="E36" s="9"/>
+      <x:c r="F36" s="25"/>
+      <x:c r="G36" s="25"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="8"/>
@@ -603,6 +749,8 @@
       <x:c r="C37" s="9"/>
       <x:c r="D37" s="9"/>
       <x:c r="E37" s="9"/>
+      <x:c r="F37" s="29"/>
+      <x:c r="G37" s="29"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="8"/>
@@ -610,6 +758,8 @@
       <x:c r="C38" s="9"/>
       <x:c r="D38" s="9"/>
       <x:c r="E38" s="9"/>
+      <x:c r="F38" s="25"/>
+      <x:c r="G38" s="25"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="8"/>
@@ -617,6 +767,8 @@
       <x:c r="C39" s="9"/>
       <x:c r="D39" s="9"/>
       <x:c r="E39" s="9"/>
+      <x:c r="F39" s="29"/>
+      <x:c r="G39" s="29"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="8"/>
@@ -624,6 +776,8 @@
       <x:c r="C40" s="9"/>
       <x:c r="D40" s="9"/>
       <x:c r="E40" s="9"/>
+      <x:c r="F40" s="25"/>
+      <x:c r="G40" s="25"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="8"/>
@@ -631,6 +785,8 @@
       <x:c r="C41" s="9"/>
       <x:c r="D41" s="9"/>
       <x:c r="E41" s="9"/>
+      <x:c r="F41" s="29"/>
+      <x:c r="G41" s="29"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="8"/>
@@ -638,6 +794,8 @@
       <x:c r="C42" s="9"/>
       <x:c r="D42" s="9"/>
       <x:c r="E42" s="9"/>
+      <x:c r="F42" s="25"/>
+      <x:c r="G42" s="25"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="8"/>
@@ -645,6 +803,8 @@
       <x:c r="C43" s="9"/>
       <x:c r="D43" s="9"/>
       <x:c r="E43" s="9"/>
+      <x:c r="F43" s="29"/>
+      <x:c r="G43" s="29"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="8"/>
@@ -652,6 +812,8 @@
       <x:c r="C44" s="9"/>
       <x:c r="D44" s="9"/>
       <x:c r="E44" s="9"/>
+      <x:c r="F44" s="25"/>
+      <x:c r="G44" s="25"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="8"/>
@@ -659,6 +821,8 @@
       <x:c r="C45" s="9"/>
       <x:c r="D45" s="9"/>
       <x:c r="E45" s="9"/>
+      <x:c r="F45" s="29"/>
+      <x:c r="G45" s="29"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="8"/>
@@ -666,6 +830,8 @@
       <x:c r="C46" s="9"/>
       <x:c r="D46" s="9"/>
       <x:c r="E46" s="9"/>
+      <x:c r="F46" s="25"/>
+      <x:c r="G46" s="25"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="8"/>
@@ -673,6 +839,8 @@
       <x:c r="C47" s="9"/>
       <x:c r="D47" s="9"/>
       <x:c r="E47" s="9"/>
+      <x:c r="F47" s="29"/>
+      <x:c r="G47" s="29"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="8"/>
@@ -680,6 +848,8 @@
       <x:c r="C48" s="9"/>
       <x:c r="D48" s="9"/>
       <x:c r="E48" s="9"/>
+      <x:c r="F48" s="25"/>
+      <x:c r="G48" s="25"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="8"/>
@@ -687,6 +857,8 @@
       <x:c r="C49" s="9"/>
       <x:c r="D49" s="9"/>
       <x:c r="E49" s="9"/>
+      <x:c r="F49" s="29"/>
+      <x:c r="G49" s="29"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="8"/>
@@ -694,6 +866,8 @@
       <x:c r="C50" s="9"/>
       <x:c r="D50" s="9"/>
       <x:c r="E50" s="9"/>
+      <x:c r="F50" s="25"/>
+      <x:c r="G50" s="25"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="8"/>
@@ -701,6 +875,8 @@
       <x:c r="C51" s="9"/>
       <x:c r="D51" s="9"/>
       <x:c r="E51" s="9"/>
+      <x:c r="F51" s="29"/>
+      <x:c r="G51" s="29"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="8"/>
@@ -708,6 +884,8 @@
       <x:c r="C52" s="9"/>
       <x:c r="D52" s="9"/>
       <x:c r="E52" s="9"/>
+      <x:c r="F52" s="25"/>
+      <x:c r="G52" s="25"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="8"/>
@@ -715,6 +893,8 @@
       <x:c r="C53" s="9"/>
       <x:c r="D53" s="9"/>
       <x:c r="E53" s="9"/>
+      <x:c r="F53" s="29"/>
+      <x:c r="G53" s="29"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="8"/>
@@ -722,6 +902,8 @@
       <x:c r="C54" s="9"/>
       <x:c r="D54" s="9"/>
       <x:c r="E54" s="9"/>
+      <x:c r="F54" s="25"/>
+      <x:c r="G54" s="25"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="8"/>
@@ -729,6 +911,8 @@
       <x:c r="C55" s="9"/>
       <x:c r="D55" s="9"/>
       <x:c r="E55" s="9"/>
+      <x:c r="F55" s="29"/>
+      <x:c r="G55" s="29"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="8"/>
@@ -736,6 +920,8 @@
       <x:c r="C56" s="9"/>
       <x:c r="D56" s="9"/>
       <x:c r="E56" s="9"/>
+      <x:c r="F56" s="25"/>
+      <x:c r="G56" s="25"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="8"/>
@@ -743,6 +929,8 @@
       <x:c r="C57" s="9"/>
       <x:c r="D57" s="9"/>
       <x:c r="E57" s="9"/>
+      <x:c r="F57" s="29"/>
+      <x:c r="G57" s="29"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="8"/>
@@ -750,6 +938,8 @@
       <x:c r="C58" s="9"/>
       <x:c r="D58" s="9"/>
       <x:c r="E58" s="9"/>
+      <x:c r="F58" s="25"/>
+      <x:c r="G58" s="25"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="8"/>
@@ -757,6 +947,8 @@
       <x:c r="C59" s="9"/>
       <x:c r="D59" s="9"/>
       <x:c r="E59" s="9"/>
+      <x:c r="F59" s="29"/>
+      <x:c r="G59" s="29"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="8"/>
@@ -764,6 +956,8 @@
       <x:c r="C60" s="9"/>
       <x:c r="D60" s="9"/>
       <x:c r="E60" s="9"/>
+      <x:c r="F60" s="25"/>
+      <x:c r="G60" s="25"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="8"/>
@@ -771,6 +965,8 @@
       <x:c r="C61" s="9"/>
       <x:c r="D61" s="9"/>
       <x:c r="E61" s="9"/>
+      <x:c r="F61" s="29"/>
+      <x:c r="G61" s="29"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="8"/>
@@ -778,6 +974,8 @@
       <x:c r="C62" s="9"/>
       <x:c r="D62" s="9"/>
       <x:c r="E62" s="9"/>
+      <x:c r="F62" s="25"/>
+      <x:c r="G62" s="25"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="8"/>
@@ -785,6 +983,8 @@
       <x:c r="C63" s="9"/>
       <x:c r="D63" s="9"/>
       <x:c r="E63" s="9"/>
+      <x:c r="F63" s="29"/>
+      <x:c r="G63" s="29"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="8"/>
@@ -792,6 +992,8 @@
       <x:c r="C64" s="9"/>
       <x:c r="D64" s="9"/>
       <x:c r="E64" s="9"/>
+      <x:c r="F64" s="25"/>
+      <x:c r="G64" s="25"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="8"/>
@@ -799,6 +1001,8 @@
       <x:c r="C65" s="9"/>
       <x:c r="D65" s="9"/>
       <x:c r="E65" s="9"/>
+      <x:c r="F65" s="29"/>
+      <x:c r="G65" s="29"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="8"/>
@@ -806,6 +1010,8 @@
       <x:c r="C66" s="9"/>
       <x:c r="D66" s="9"/>
       <x:c r="E66" s="9"/>
+      <x:c r="F66" s="25"/>
+      <x:c r="G66" s="25"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="8"/>
@@ -813,6 +1019,8 @@
       <x:c r="C67" s="9"/>
       <x:c r="D67" s="9"/>
       <x:c r="E67" s="9"/>
+      <x:c r="F67" s="29"/>
+      <x:c r="G67" s="29"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="8"/>
@@ -820,6 +1028,8 @@
       <x:c r="C68" s="9"/>
       <x:c r="D68" s="9"/>
       <x:c r="E68" s="9"/>
+      <x:c r="F68" s="25"/>
+      <x:c r="G68" s="25"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="8"/>
@@ -827,6 +1037,8 @@
       <x:c r="C69" s="9"/>
       <x:c r="D69" s="9"/>
       <x:c r="E69" s="9"/>
+      <x:c r="F69" s="29"/>
+      <x:c r="G69" s="29"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="8"/>
@@ -834,6 +1046,8 @@
       <x:c r="C70" s="9"/>
       <x:c r="D70" s="9"/>
       <x:c r="E70" s="9"/>
+      <x:c r="F70" s="25"/>
+      <x:c r="G70" s="25"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="8"/>
@@ -841,6 +1055,8 @@
       <x:c r="C71" s="9"/>
       <x:c r="D71" s="9"/>
       <x:c r="E71" s="9"/>
+      <x:c r="F71" s="29"/>
+      <x:c r="G71" s="29"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="8"/>
@@ -848,6 +1064,8 @@
       <x:c r="C72" s="9"/>
       <x:c r="D72" s="9"/>
       <x:c r="E72" s="9"/>
+      <x:c r="F72" s="25"/>
+      <x:c r="G72" s="25"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="8"/>
@@ -855,6 +1073,8 @@
       <x:c r="C73" s="9"/>
       <x:c r="D73" s="9"/>
       <x:c r="E73" s="9"/>
+      <x:c r="F73" s="29"/>
+      <x:c r="G73" s="29"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="8"/>
@@ -862,6 +1082,8 @@
       <x:c r="C74" s="9"/>
       <x:c r="D74" s="9"/>
       <x:c r="E74" s="9"/>
+      <x:c r="F74" s="25"/>
+      <x:c r="G74" s="25"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="8"/>
@@ -869,6 +1091,8 @@
       <x:c r="C75" s="9"/>
       <x:c r="D75" s="9"/>
       <x:c r="E75" s="9"/>
+      <x:c r="F75" s="29"/>
+      <x:c r="G75" s="29"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="8"/>
@@ -876,6 +1100,8 @@
       <x:c r="C76" s="9"/>
       <x:c r="D76" s="9"/>
       <x:c r="E76" s="9"/>
+      <x:c r="F76" s="25"/>
+      <x:c r="G76" s="25"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="8"/>
@@ -883,6 +1109,8 @@
       <x:c r="C77" s="9"/>
       <x:c r="D77" s="9"/>
       <x:c r="E77" s="9"/>
+      <x:c r="F77" s="29"/>
+      <x:c r="G77" s="29"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="8"/>
@@ -890,6 +1118,8 @@
       <x:c r="C78" s="9"/>
       <x:c r="D78" s="9"/>
       <x:c r="E78" s="9"/>
+      <x:c r="F78" s="25"/>
+      <x:c r="G78" s="25"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="8"/>
@@ -897,6 +1127,8 @@
       <x:c r="C79" s="9"/>
       <x:c r="D79" s="9"/>
       <x:c r="E79" s="9"/>
+      <x:c r="F79" s="29"/>
+      <x:c r="G79" s="29"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="8"/>
@@ -904,6 +1136,8 @@
       <x:c r="C80" s="9"/>
       <x:c r="D80" s="9"/>
       <x:c r="E80" s="9"/>
+      <x:c r="F80" s="25"/>
+      <x:c r="G80" s="25"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="8"/>
@@ -911,6 +1145,8 @@
       <x:c r="C81" s="9"/>
       <x:c r="D81" s="9"/>
       <x:c r="E81" s="9"/>
+      <x:c r="F81" s="29"/>
+      <x:c r="G81" s="29"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="8"/>
@@ -918,6 +1154,8 @@
       <x:c r="C82" s="9"/>
       <x:c r="D82" s="9"/>
       <x:c r="E82" s="9"/>
+      <x:c r="F82" s="25"/>
+      <x:c r="G82" s="25"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="8"/>
@@ -925,6 +1163,8 @@
       <x:c r="C83" s="9"/>
       <x:c r="D83" s="9"/>
       <x:c r="E83" s="9"/>
+      <x:c r="F83" s="29"/>
+      <x:c r="G83" s="29"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="8"/>
@@ -932,6 +1172,8 @@
       <x:c r="C84" s="9"/>
       <x:c r="D84" s="9"/>
       <x:c r="E84" s="9"/>
+      <x:c r="F84" s="25"/>
+      <x:c r="G84" s="25"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="8"/>
@@ -939,6 +1181,8 @@
       <x:c r="C85" s="9"/>
       <x:c r="D85" s="9"/>
       <x:c r="E85" s="9"/>
+      <x:c r="F85" s="29"/>
+      <x:c r="G85" s="29"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="8"/>
@@ -946,6 +1190,8 @@
       <x:c r="C86" s="9"/>
       <x:c r="D86" s="9"/>
       <x:c r="E86" s="9"/>
+      <x:c r="F86" s="25"/>
+      <x:c r="G86" s="25"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="8"/>
@@ -953,6 +1199,8 @@
       <x:c r="C87" s="9"/>
       <x:c r="D87" s="9"/>
       <x:c r="E87" s="9"/>
+      <x:c r="F87" s="29"/>
+      <x:c r="G87" s="29"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="8"/>
@@ -960,6 +1208,8 @@
       <x:c r="C88" s="9"/>
       <x:c r="D88" s="9"/>
       <x:c r="E88" s="9"/>
+      <x:c r="F88" s="25"/>
+      <x:c r="G88" s="25"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="8"/>
@@ -967,6 +1217,8 @@
       <x:c r="C89" s="9"/>
       <x:c r="D89" s="9"/>
       <x:c r="E89" s="9"/>
+      <x:c r="F89" s="29"/>
+      <x:c r="G89" s="29"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="8"/>
@@ -974,6 +1226,8 @@
       <x:c r="C90" s="9"/>
       <x:c r="D90" s="9"/>
       <x:c r="E90" s="9"/>
+      <x:c r="F90" s="25"/>
+      <x:c r="G90" s="25"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="8"/>
@@ -981,6 +1235,8 @@
       <x:c r="C91" s="9"/>
       <x:c r="D91" s="9"/>
       <x:c r="E91" s="9"/>
+      <x:c r="F91" s="29"/>
+      <x:c r="G91" s="29"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="8"/>
@@ -988,6 +1244,8 @@
       <x:c r="C92" s="9"/>
       <x:c r="D92" s="9"/>
       <x:c r="E92" s="9"/>
+      <x:c r="F92" s="25"/>
+      <x:c r="G92" s="25"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="8"/>
@@ -995,6 +1253,8 @@
       <x:c r="C93" s="9"/>
       <x:c r="D93" s="9"/>
       <x:c r="E93" s="9"/>
+      <x:c r="F93" s="29"/>
+      <x:c r="G93" s="29"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="8"/>
@@ -1002,6 +1262,8 @@
       <x:c r="C94" s="9"/>
       <x:c r="D94" s="9"/>
       <x:c r="E94" s="9"/>
+      <x:c r="F94" s="25"/>
+      <x:c r="G94" s="25"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="8"/>
@@ -1009,6 +1271,8 @@
       <x:c r="C95" s="9"/>
       <x:c r="D95" s="9"/>
       <x:c r="E95" s="9"/>
+      <x:c r="F95" s="29"/>
+      <x:c r="G95" s="29"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="8"/>
@@ -1016,6 +1280,8 @@
       <x:c r="C96" s="9"/>
       <x:c r="D96" s="9"/>
       <x:c r="E96" s="9"/>
+      <x:c r="F96" s="25"/>
+      <x:c r="G96" s="25"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="8"/>
@@ -1023,6 +1289,8 @@
       <x:c r="C97" s="9"/>
       <x:c r="D97" s="9"/>
       <x:c r="E97" s="9"/>
+      <x:c r="F97" s="29"/>
+      <x:c r="G97" s="29"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="8"/>
@@ -1030,6 +1298,8 @@
       <x:c r="C98" s="9"/>
       <x:c r="D98" s="9"/>
       <x:c r="E98" s="9"/>
+      <x:c r="F98" s="25"/>
+      <x:c r="G98" s="25"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="8"/>
@@ -1037,6 +1307,8 @@
       <x:c r="C99" s="9"/>
       <x:c r="D99" s="9"/>
       <x:c r="E99" s="9"/>
+      <x:c r="F99" s="29"/>
+      <x:c r="G99" s="29"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="8"/>
@@ -1044,6 +1316,8 @@
       <x:c r="C100" s="9"/>
       <x:c r="D100" s="9"/>
       <x:c r="E100" s="9"/>
+      <x:c r="F100" s="25"/>
+      <x:c r="G100" s="25"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="8"/>
@@ -1051,6 +1325,8 @@
       <x:c r="C101" s="9"/>
       <x:c r="D101" s="9"/>
       <x:c r="E101" s="9"/>
+      <x:c r="F101" s="29"/>
+      <x:c r="G101" s="29"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="8"/>
@@ -1058,6 +1334,8 @@
       <x:c r="C102" s="9"/>
       <x:c r="D102" s="9"/>
       <x:c r="E102" s="9"/>
+      <x:c r="F102" s="25"/>
+      <x:c r="G102" s="25"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="8"/>
@@ -1065,6 +1343,8 @@
       <x:c r="C103" s="9"/>
       <x:c r="D103" s="9"/>
       <x:c r="E103" s="9"/>
+      <x:c r="F103" s="29"/>
+      <x:c r="G103" s="29"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="8"/>
@@ -1072,6 +1352,8 @@
       <x:c r="C104" s="9"/>
       <x:c r="D104" s="9"/>
       <x:c r="E104" s="9"/>
+      <x:c r="F104" s="25"/>
+      <x:c r="G104" s="25"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="8"/>
@@ -1079,6 +1361,8 @@
       <x:c r="C105" s="9"/>
       <x:c r="D105" s="9"/>
       <x:c r="E105" s="9"/>
+      <x:c r="F105" s="29"/>
+      <x:c r="G105" s="29"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="8"/>
@@ -1086,6 +1370,8 @@
       <x:c r="C106" s="9"/>
       <x:c r="D106" s="9"/>
       <x:c r="E106" s="9"/>
+      <x:c r="F106" s="25"/>
+      <x:c r="G106" s="25"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="8"/>
@@ -1093,6 +1379,8 @@
       <x:c r="C107" s="9"/>
       <x:c r="D107" s="9"/>
       <x:c r="E107" s="9"/>
+      <x:c r="F107" s="29"/>
+      <x:c r="G107" s="29"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="8"/>
@@ -1100,6 +1388,8 @@
       <x:c r="C108" s="9"/>
       <x:c r="D108" s="9"/>
       <x:c r="E108" s="9"/>
+      <x:c r="F108" s="25"/>
+      <x:c r="G108" s="25"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="8"/>
@@ -1107,6 +1397,8 @@
       <x:c r="C109" s="9"/>
       <x:c r="D109" s="9"/>
       <x:c r="E109" s="9"/>
+      <x:c r="F109" s="29"/>
+      <x:c r="G109" s="29"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="8"/>
@@ -1114,6 +1406,8 @@
       <x:c r="C110" s="9"/>
       <x:c r="D110" s="9"/>
       <x:c r="E110" s="9"/>
+      <x:c r="F110" s="25"/>
+      <x:c r="G110" s="25"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="8"/>
@@ -1121,6 +1415,8 @@
       <x:c r="C111" s="9"/>
       <x:c r="D111" s="9"/>
       <x:c r="E111" s="9"/>
+      <x:c r="F111" s="29"/>
+      <x:c r="G111" s="29"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="8"/>
@@ -1128,6 +1424,8 @@
       <x:c r="C112" s="9"/>
       <x:c r="D112" s="9"/>
       <x:c r="E112" s="9"/>
+      <x:c r="F112" s="25"/>
+      <x:c r="G112" s="25"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="8"/>
@@ -1135,6 +1433,8 @@
       <x:c r="C113" s="9"/>
       <x:c r="D113" s="9"/>
       <x:c r="E113" s="9"/>
+      <x:c r="F113" s="29"/>
+      <x:c r="G113" s="29"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="8"/>
@@ -1142,6 +1442,8 @@
       <x:c r="C114" s="9"/>
       <x:c r="D114" s="9"/>
       <x:c r="E114" s="9"/>
+      <x:c r="F114" s="25"/>
+      <x:c r="G114" s="25"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="8"/>
@@ -1149,6 +1451,8 @@
       <x:c r="C115" s="9"/>
       <x:c r="D115" s="9"/>
       <x:c r="E115" s="9"/>
+      <x:c r="F115" s="29"/>
+      <x:c r="G115" s="29"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="8"/>
@@ -1156,6 +1460,8 @@
       <x:c r="C116" s="9"/>
       <x:c r="D116" s="9"/>
       <x:c r="E116" s="9"/>
+      <x:c r="F116" s="25"/>
+      <x:c r="G116" s="25"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="8"/>
@@ -1163,6 +1469,8 @@
       <x:c r="C117" s="9"/>
       <x:c r="D117" s="9"/>
       <x:c r="E117" s="9"/>
+      <x:c r="F117" s="29"/>
+      <x:c r="G117" s="29"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="8"/>
@@ -1170,6 +1478,8 @@
       <x:c r="C118" s="9"/>
       <x:c r="D118" s="9"/>
       <x:c r="E118" s="9"/>
+      <x:c r="F118" s="25"/>
+      <x:c r="G118" s="25"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="8"/>
@@ -1177,6 +1487,8 @@
       <x:c r="C119" s="9"/>
       <x:c r="D119" s="9"/>
       <x:c r="E119" s="9"/>
+      <x:c r="F119" s="29"/>
+      <x:c r="G119" s="29"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="8"/>
@@ -1184,6 +1496,8 @@
       <x:c r="C120" s="9"/>
       <x:c r="D120" s="9"/>
       <x:c r="E120" s="9"/>
+      <x:c r="F120" s="25"/>
+      <x:c r="G120" s="25"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="8"/>
@@ -1191,6 +1505,8 @@
       <x:c r="C121" s="9"/>
       <x:c r="D121" s="9"/>
       <x:c r="E121" s="9"/>
+      <x:c r="F121" s="29"/>
+      <x:c r="G121" s="29"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="8"/>
@@ -1198,6 +1514,8 @@
       <x:c r="C122" s="9"/>
       <x:c r="D122" s="9"/>
       <x:c r="E122" s="9"/>
+      <x:c r="F122" s="25"/>
+      <x:c r="G122" s="25"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="8"/>
@@ -1205,6 +1523,8 @@
       <x:c r="C123" s="9"/>
       <x:c r="D123" s="9"/>
       <x:c r="E123" s="9"/>
+      <x:c r="F123" s="29"/>
+      <x:c r="G123" s="29"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="8"/>
@@ -1212,6 +1532,8 @@
       <x:c r="C124" s="9"/>
       <x:c r="D124" s="9"/>
       <x:c r="E124" s="9"/>
+      <x:c r="F124" s="25"/>
+      <x:c r="G124" s="25"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="8"/>
@@ -1219,6 +1541,8 @@
       <x:c r="C125" s="9"/>
       <x:c r="D125" s="9"/>
       <x:c r="E125" s="9"/>
+      <x:c r="F125" s="29"/>
+      <x:c r="G125" s="29"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="8"/>
@@ -1226,6 +1550,8 @@
       <x:c r="C126" s="9"/>
       <x:c r="D126" s="9"/>
       <x:c r="E126" s="9"/>
+      <x:c r="F126" s="25"/>
+      <x:c r="G126" s="25"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="8"/>
@@ -1233,6 +1559,8 @@
       <x:c r="C127" s="9"/>
       <x:c r="D127" s="9"/>
       <x:c r="E127" s="9"/>
+      <x:c r="F127" s="29"/>
+      <x:c r="G127" s="29"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="8"/>
@@ -1240,6 +1568,8 @@
       <x:c r="C128" s="9"/>
       <x:c r="D128" s="9"/>
       <x:c r="E128" s="9"/>
+      <x:c r="F128" s="25"/>
+      <x:c r="G128" s="25"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="8"/>
@@ -1247,6 +1577,8 @@
       <x:c r="C129" s="9"/>
       <x:c r="D129" s="9"/>
       <x:c r="E129" s="9"/>
+      <x:c r="F129" s="29"/>
+      <x:c r="G129" s="29"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="8"/>
@@ -1254,6 +1586,8 @@
       <x:c r="C130" s="9"/>
       <x:c r="D130" s="9"/>
       <x:c r="E130" s="9"/>
+      <x:c r="F130" s="25"/>
+      <x:c r="G130" s="25"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="8"/>
@@ -1261,6 +1595,8 @@
       <x:c r="C131" s="9"/>
       <x:c r="D131" s="9"/>
       <x:c r="E131" s="9"/>
+      <x:c r="F131" s="29"/>
+      <x:c r="G131" s="29"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="8"/>
@@ -1268,6 +1604,8 @@
       <x:c r="C132" s="9"/>
       <x:c r="D132" s="9"/>
       <x:c r="E132" s="9"/>
+      <x:c r="F132" s="25"/>
+      <x:c r="G132" s="25"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="8"/>
@@ -1275,6 +1613,8 @@
       <x:c r="C133" s="9"/>
       <x:c r="D133" s="9"/>
       <x:c r="E133" s="9"/>
+      <x:c r="F133" s="29"/>
+      <x:c r="G133" s="29"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="8"/>
@@ -1282,6 +1622,8 @@
       <x:c r="C134" s="9"/>
       <x:c r="D134" s="9"/>
       <x:c r="E134" s="9"/>
+      <x:c r="F134" s="25"/>
+      <x:c r="G134" s="25"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="8"/>
@@ -1289,6 +1631,8 @@
       <x:c r="C135" s="9"/>
       <x:c r="D135" s="9"/>
       <x:c r="E135" s="9"/>
+      <x:c r="F135" s="29"/>
+      <x:c r="G135" s="29"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="8"/>
@@ -1296,6 +1640,8 @@
       <x:c r="C136" s="9"/>
       <x:c r="D136" s="9"/>
       <x:c r="E136" s="9"/>
+      <x:c r="F136" s="25"/>
+      <x:c r="G136" s="25"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="8"/>
@@ -1303,6 +1649,8 @@
       <x:c r="C137" s="9"/>
       <x:c r="D137" s="9"/>
       <x:c r="E137" s="9"/>
+      <x:c r="F137" s="29"/>
+      <x:c r="G137" s="29"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="8"/>
@@ -1310,6 +1658,8 @@
       <x:c r="C138" s="9"/>
       <x:c r="D138" s="9"/>
       <x:c r="E138" s="9"/>
+      <x:c r="F138" s="25"/>
+      <x:c r="G138" s="25"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="8"/>
@@ -1317,6 +1667,8 @@
       <x:c r="C139" s="9"/>
       <x:c r="D139" s="9"/>
       <x:c r="E139" s="9"/>
+      <x:c r="F139" s="29"/>
+      <x:c r="G139" s="29"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="8"/>
@@ -1324,6 +1676,8 @@
       <x:c r="C140" s="9"/>
       <x:c r="D140" s="9"/>
       <x:c r="E140" s="9"/>
+      <x:c r="F140" s="25"/>
+      <x:c r="G140" s="25"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="8"/>
@@ -1331,6 +1685,8 @@
       <x:c r="C141" s="9"/>
       <x:c r="D141" s="9"/>
       <x:c r="E141" s="9"/>
+      <x:c r="F141" s="29"/>
+      <x:c r="G141" s="29"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="8"/>
@@ -1338,6 +1694,8 @@
       <x:c r="C142" s="9"/>
       <x:c r="D142" s="9"/>
       <x:c r="E142" s="9"/>
+      <x:c r="F142" s="25"/>
+      <x:c r="G142" s="25"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="8"/>
@@ -1345,6 +1703,8 @@
       <x:c r="C143" s="9"/>
       <x:c r="D143" s="9"/>
       <x:c r="E143" s="9"/>
+      <x:c r="F143" s="29"/>
+      <x:c r="G143" s="29"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="8"/>
@@ -1352,6 +1712,8 @@
       <x:c r="C144" s="9"/>
       <x:c r="D144" s="9"/>
       <x:c r="E144" s="9"/>
+      <x:c r="F144" s="25"/>
+      <x:c r="G144" s="25"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="8"/>
@@ -1359,6 +1721,8 @@
       <x:c r="C145" s="9"/>
       <x:c r="D145" s="9"/>
       <x:c r="E145" s="9"/>
+      <x:c r="F145" s="29"/>
+      <x:c r="G145" s="29"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="8"/>
@@ -1366,6 +1730,8 @@
       <x:c r="C146" s="9"/>
       <x:c r="D146" s="9"/>
       <x:c r="E146" s="9"/>
+      <x:c r="F146" s="25"/>
+      <x:c r="G146" s="25"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="8"/>
@@ -1373,6 +1739,8 @@
       <x:c r="C147" s="9"/>
       <x:c r="D147" s="9"/>
       <x:c r="E147" s="9"/>
+      <x:c r="F147" s="29"/>
+      <x:c r="G147" s="29"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="8"/>
@@ -1380,6 +1748,8 @@
       <x:c r="C148" s="9"/>
       <x:c r="D148" s="9"/>
       <x:c r="E148" s="9"/>
+      <x:c r="F148" s="25"/>
+      <x:c r="G148" s="25"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="8"/>
@@ -1387,6 +1757,8 @@
       <x:c r="C149" s="9"/>
       <x:c r="D149" s="9"/>
       <x:c r="E149" s="9"/>
+      <x:c r="F149" s="29"/>
+      <x:c r="G149" s="29"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="8"/>
@@ -1394,6 +1766,8 @@
       <x:c r="C150" s="9"/>
       <x:c r="D150" s="9"/>
       <x:c r="E150" s="9"/>
+      <x:c r="F150" s="25"/>
+      <x:c r="G150" s="25"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="8"/>
@@ -1401,6 +1775,8 @@
       <x:c r="C151" s="9"/>
       <x:c r="D151" s="9"/>
       <x:c r="E151" s="9"/>
+      <x:c r="F151" s="29"/>
+      <x:c r="G151" s="29"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="8"/>
@@ -1408,6 +1784,8 @@
       <x:c r="C152" s="9"/>
       <x:c r="D152" s="9"/>
       <x:c r="E152" s="9"/>
+      <x:c r="F152" s="25"/>
+      <x:c r="G152" s="25"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="8"/>
@@ -1415,6 +1793,8 @@
       <x:c r="C153" s="9"/>
       <x:c r="D153" s="9"/>
       <x:c r="E153" s="9"/>
+      <x:c r="F153" s="29"/>
+      <x:c r="G153" s="29"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="8"/>
@@ -1422,6 +1802,8 @@
       <x:c r="C154" s="9"/>
       <x:c r="D154" s="9"/>
       <x:c r="E154" s="9"/>
+      <x:c r="F154" s="25"/>
+      <x:c r="G154" s="25"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="8"/>
@@ -1429,6 +1811,8 @@
       <x:c r="C155" s="9"/>
       <x:c r="D155" s="9"/>
       <x:c r="E155" s="9"/>
+      <x:c r="F155" s="29"/>
+      <x:c r="G155" s="29"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="8"/>
@@ -1436,6 +1820,8 @@
       <x:c r="C156" s="9"/>
       <x:c r="D156" s="9"/>
       <x:c r="E156" s="9"/>
+      <x:c r="F156" s="25"/>
+      <x:c r="G156" s="25"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="8"/>
@@ -1443,6 +1829,8 @@
       <x:c r="C157" s="9"/>
       <x:c r="D157" s="9"/>
       <x:c r="E157" s="9"/>
+      <x:c r="F157" s="29"/>
+      <x:c r="G157" s="29"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="8"/>
@@ -1450,6 +1838,8 @@
       <x:c r="C158" s="9"/>
       <x:c r="D158" s="9"/>
       <x:c r="E158" s="9"/>
+      <x:c r="F158" s="25"/>
+      <x:c r="G158" s="25"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="8"/>
@@ -1457,6 +1847,8 @@
       <x:c r="C159" s="9"/>
       <x:c r="D159" s="9"/>
       <x:c r="E159" s="9"/>
+      <x:c r="F159" s="29"/>
+      <x:c r="G159" s="29"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="8"/>
@@ -1464,6 +1856,8 @@
       <x:c r="C160" s="9"/>
       <x:c r="D160" s="9"/>
       <x:c r="E160" s="9"/>
+      <x:c r="F160" s="25"/>
+      <x:c r="G160" s="25"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="8"/>
@@ -1471,6 +1865,8 @@
       <x:c r="C161" s="9"/>
       <x:c r="D161" s="9"/>
       <x:c r="E161" s="9"/>
+      <x:c r="F161" s="29"/>
+      <x:c r="G161" s="29"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="8"/>
@@ -1478,6 +1874,8 @@
       <x:c r="C162" s="9"/>
       <x:c r="D162" s="9"/>
       <x:c r="E162" s="9"/>
+      <x:c r="F162" s="25"/>
+      <x:c r="G162" s="25"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="8"/>
@@ -1485,6 +1883,8 @@
       <x:c r="C163" s="9"/>
       <x:c r="D163" s="9"/>
       <x:c r="E163" s="9"/>
+      <x:c r="F163" s="29"/>
+      <x:c r="G163" s="29"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="8"/>
@@ -1492,6 +1892,8 @@
       <x:c r="C164" s="9"/>
       <x:c r="D164" s="9"/>
       <x:c r="E164" s="9"/>
+      <x:c r="F164" s="25"/>
+      <x:c r="G164" s="25"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="8"/>
@@ -1499,6 +1901,8 @@
       <x:c r="C165" s="9"/>
       <x:c r="D165" s="9"/>
       <x:c r="E165" s="9"/>
+      <x:c r="F165" s="29"/>
+      <x:c r="G165" s="29"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="8"/>
@@ -1506,6 +1910,8 @@
       <x:c r="C166" s="9"/>
       <x:c r="D166" s="9"/>
       <x:c r="E166" s="9"/>
+      <x:c r="F166" s="25"/>
+      <x:c r="G166" s="25"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="8"/>
@@ -1513,6 +1919,8 @@
       <x:c r="C167" s="9"/>
       <x:c r="D167" s="9"/>
       <x:c r="E167" s="9"/>
+      <x:c r="F167" s="29"/>
+      <x:c r="G167" s="29"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="8"/>
@@ -1520,6 +1928,8 @@
       <x:c r="C168" s="9"/>
       <x:c r="D168" s="9"/>
       <x:c r="E168" s="9"/>
+      <x:c r="F168" s="25"/>
+      <x:c r="G168" s="25"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="8"/>
@@ -1527,6 +1937,8 @@
       <x:c r="C169" s="9"/>
       <x:c r="D169" s="9"/>
       <x:c r="E169" s="9"/>
+      <x:c r="F169" s="29"/>
+      <x:c r="G169" s="29"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="8"/>
@@ -1534,6 +1946,8 @@
       <x:c r="C170" s="9"/>
       <x:c r="D170" s="9"/>
       <x:c r="E170" s="9"/>
+      <x:c r="F170" s="25"/>
+      <x:c r="G170" s="25"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="8"/>
@@ -1541,6 +1955,8 @@
       <x:c r="C171" s="9"/>
       <x:c r="D171" s="9"/>
       <x:c r="E171" s="9"/>
+      <x:c r="F171" s="29"/>
+      <x:c r="G171" s="29"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="8"/>
@@ -1548,6 +1964,8 @@
       <x:c r="C172" s="9"/>
       <x:c r="D172" s="9"/>
       <x:c r="E172" s="9"/>
+      <x:c r="F172" s="25"/>
+      <x:c r="G172" s="25"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="8"/>
@@ -1555,6 +1973,8 @@
       <x:c r="C173" s="9"/>
       <x:c r="D173" s="9"/>
       <x:c r="E173" s="9"/>
+      <x:c r="F173" s="29"/>
+      <x:c r="G173" s="29"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="8"/>
@@ -1562,6 +1982,8 @@
       <x:c r="C174" s="9"/>
       <x:c r="D174" s="9"/>
       <x:c r="E174" s="9"/>
+      <x:c r="F174" s="25"/>
+      <x:c r="G174" s="25"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="8"/>
@@ -1569,6 +1991,8 @@
       <x:c r="C175" s="9"/>
       <x:c r="D175" s="9"/>
       <x:c r="E175" s="9"/>
+      <x:c r="F175" s="29"/>
+      <x:c r="G175" s="29"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="8"/>
@@ -1576,6 +2000,8 @@
       <x:c r="C176" s="9"/>
       <x:c r="D176" s="9"/>
       <x:c r="E176" s="9"/>
+      <x:c r="F176" s="25"/>
+      <x:c r="G176" s="25"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="8"/>
@@ -1583,6 +2009,8 @@
       <x:c r="C177" s="9"/>
       <x:c r="D177" s="9"/>
       <x:c r="E177" s="9"/>
+      <x:c r="F177" s="29"/>
+      <x:c r="G177" s="29"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="8"/>
@@ -1590,6 +2018,8 @@
       <x:c r="C178" s="9"/>
       <x:c r="D178" s="9"/>
       <x:c r="E178" s="9"/>
+      <x:c r="F178" s="25"/>
+      <x:c r="G178" s="25"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="8"/>
@@ -1597,6 +2027,8 @@
       <x:c r="C179" s="9"/>
       <x:c r="D179" s="9"/>
       <x:c r="E179" s="9"/>
+      <x:c r="F179" s="29"/>
+      <x:c r="G179" s="29"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="8"/>
@@ -1604,6 +2036,8 @@
       <x:c r="C180" s="9"/>
       <x:c r="D180" s="9"/>
       <x:c r="E180" s="9"/>
+      <x:c r="F180" s="25"/>
+      <x:c r="G180" s="25"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="8"/>
@@ -1611,6 +2045,8 @@
       <x:c r="C181" s="9"/>
       <x:c r="D181" s="9"/>
       <x:c r="E181" s="9"/>
+      <x:c r="F181" s="29"/>
+      <x:c r="G181" s="29"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="8"/>
@@ -1618,6 +2054,8 @@
       <x:c r="C182" s="9"/>
       <x:c r="D182" s="9"/>
       <x:c r="E182" s="9"/>
+      <x:c r="F182" s="25"/>
+      <x:c r="G182" s="25"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="8"/>
@@ -1625,6 +2063,8 @@
       <x:c r="C183" s="9"/>
       <x:c r="D183" s="9"/>
       <x:c r="E183" s="9"/>
+      <x:c r="F183" s="29"/>
+      <x:c r="G183" s="29"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="8"/>
@@ -1632,6 +2072,8 @@
       <x:c r="C184" s="9"/>
       <x:c r="D184" s="9"/>
       <x:c r="E184" s="9"/>
+      <x:c r="F184" s="25"/>
+      <x:c r="G184" s="25"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="8"/>
@@ -1639,6 +2081,8 @@
       <x:c r="C185" s="9"/>
       <x:c r="D185" s="9"/>
       <x:c r="E185" s="9"/>
+      <x:c r="F185" s="29"/>
+      <x:c r="G185" s="29"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="8"/>
@@ -1646,6 +2090,8 @@
       <x:c r="C186" s="9"/>
       <x:c r="D186" s="9"/>
       <x:c r="E186" s="9"/>
+      <x:c r="F186" s="25"/>
+      <x:c r="G186" s="25"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="8"/>
@@ -1653,6 +2099,8 @@
       <x:c r="C187" s="9"/>
       <x:c r="D187" s="9"/>
       <x:c r="E187" s="9"/>
+      <x:c r="F187" s="29"/>
+      <x:c r="G187" s="29"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="8"/>
@@ -1660,6 +2108,8 @@
       <x:c r="C188" s="9"/>
       <x:c r="D188" s="9"/>
       <x:c r="E188" s="9"/>
+      <x:c r="F188" s="25"/>
+      <x:c r="G188" s="25"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="8"/>
@@ -1667,6 +2117,8 @@
       <x:c r="C189" s="9"/>
       <x:c r="D189" s="9"/>
       <x:c r="E189" s="9"/>
+      <x:c r="F189" s="29"/>
+      <x:c r="G189" s="29"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="8"/>
@@ -1674,6 +2126,8 @@
       <x:c r="C190" s="9"/>
       <x:c r="D190" s="9"/>
       <x:c r="E190" s="9"/>
+      <x:c r="F190" s="25"/>
+      <x:c r="G190" s="25"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="8"/>
@@ -1681,6 +2135,8 @@
       <x:c r="C191" s="9"/>
       <x:c r="D191" s="9"/>
       <x:c r="E191" s="9"/>
+      <x:c r="F191" s="29"/>
+      <x:c r="G191" s="29"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="8"/>
@@ -1688,6 +2144,8 @@
       <x:c r="C192" s="9"/>
       <x:c r="D192" s="9"/>
       <x:c r="E192" s="9"/>
+      <x:c r="F192" s="25"/>
+      <x:c r="G192" s="25"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="8"/>
@@ -1695,6 +2153,8 @@
       <x:c r="C193" s="9"/>
       <x:c r="D193" s="9"/>
       <x:c r="E193" s="9"/>
+      <x:c r="F193" s="29"/>
+      <x:c r="G193" s="29"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="8"/>
@@ -1702,6 +2162,8 @@
       <x:c r="C194" s="9"/>
       <x:c r="D194" s="9"/>
       <x:c r="E194" s="9"/>
+      <x:c r="F194" s="25"/>
+      <x:c r="G194" s="25"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="8"/>
@@ -1709,6 +2171,8 @@
       <x:c r="C195" s="9"/>
       <x:c r="D195" s="9"/>
       <x:c r="E195" s="9"/>
+      <x:c r="F195" s="29"/>
+      <x:c r="G195" s="29"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="8"/>
@@ -1716,6 +2180,8 @@
       <x:c r="C196" s="9"/>
       <x:c r="D196" s="9"/>
       <x:c r="E196" s="9"/>
+      <x:c r="F196" s="25"/>
+      <x:c r="G196" s="25"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="8"/>
@@ -1723,6 +2189,8 @@
       <x:c r="C197" s="9"/>
       <x:c r="D197" s="9"/>
       <x:c r="E197" s="9"/>
+      <x:c r="F197" s="29"/>
+      <x:c r="G197" s="29"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="8"/>
@@ -1730,6 +2198,8 @@
       <x:c r="C198" s="9"/>
       <x:c r="D198" s="9"/>
       <x:c r="E198" s="9"/>
+      <x:c r="F198" s="25"/>
+      <x:c r="G198" s="25"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="8"/>
@@ -1737,6 +2207,8 @@
       <x:c r="C199" s="9"/>
       <x:c r="D199" s="9"/>
       <x:c r="E199" s="9"/>
+      <x:c r="F199" s="29"/>
+      <x:c r="G199" s="29"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="8"/>
@@ -1744,6 +2216,8 @@
       <x:c r="C200" s="9"/>
       <x:c r="D200" s="9"/>
       <x:c r="E200" s="9"/>
+      <x:c r="F200" s="25"/>
+      <x:c r="G200" s="25"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="8"/>
@@ -1751,6 +2225,8 @@
       <x:c r="C201" s="9"/>
       <x:c r="D201" s="9"/>
       <x:c r="E201" s="9"/>
+      <x:c r="F201" s="29"/>
+      <x:c r="G201" s="29"/>
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="8"/>
@@ -1758,6 +2234,8 @@
       <x:c r="C202" s="9"/>
       <x:c r="D202" s="9"/>
       <x:c r="E202" s="9"/>
+      <x:c r="F202" s="25"/>
+      <x:c r="G202" s="25"/>
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="8"/>
@@ -1765,6 +2243,8 @@
       <x:c r="C203" s="9"/>
       <x:c r="D203" s="9"/>
       <x:c r="E203" s="9"/>
+      <x:c r="F203" s="29"/>
+      <x:c r="G203" s="29"/>
     </x:row>
     <x:row r="204">
       <x:c r="A204" s="8"/>
@@ -1772,6 +2252,8 @@
       <x:c r="C204" s="9"/>
       <x:c r="D204" s="9"/>
       <x:c r="E204" s="9"/>
+      <x:c r="F204" s="25"/>
+      <x:c r="G204" s="25"/>
     </x:row>
     <x:row r="205">
       <x:c r="A205" s="8"/>
@@ -1779,6 +2261,8 @@
       <x:c r="C205" s="9"/>
       <x:c r="D205" s="9"/>
       <x:c r="E205" s="9"/>
+      <x:c r="F205" s="29"/>
+      <x:c r="G205" s="29"/>
     </x:row>
     <x:row r="206">
       <x:c r="A206" s="8"/>
@@ -1786,6 +2270,8 @@
       <x:c r="C206" s="9"/>
       <x:c r="D206" s="9"/>
       <x:c r="E206" s="9"/>
+      <x:c r="F206" s="25"/>
+      <x:c r="G206" s="25"/>
     </x:row>
     <x:row r="207">
       <x:c r="A207" s="8"/>
@@ -1793,6 +2279,8 @@
       <x:c r="C207" s="9"/>
       <x:c r="D207" s="9"/>
       <x:c r="E207" s="9"/>
+      <x:c r="F207" s="29"/>
+      <x:c r="G207" s="29"/>
     </x:row>
     <x:row r="208">
       <x:c r="A208" s="8"/>
@@ -1800,6 +2288,8 @@
       <x:c r="C208" s="9"/>
       <x:c r="D208" s="9"/>
       <x:c r="E208" s="9"/>
+      <x:c r="F208" s="25"/>
+      <x:c r="G208" s="25"/>
     </x:row>
     <x:row r="209">
       <x:c r="A209" s="8"/>
@@ -1807,6 +2297,8 @@
       <x:c r="C209" s="9"/>
       <x:c r="D209" s="9"/>
       <x:c r="E209" s="9"/>
+      <x:c r="F209" s="29"/>
+      <x:c r="G209" s="29"/>
     </x:row>
     <x:row r="210">
       <x:c r="A210" s="8"/>
@@ -1814,6 +2306,8 @@
       <x:c r="C210" s="9"/>
       <x:c r="D210" s="9"/>
       <x:c r="E210" s="9"/>
+      <x:c r="F210" s="25"/>
+      <x:c r="G210" s="25"/>
     </x:row>
     <x:row r="211">
       <x:c r="A211" s="8"/>
@@ -1821,6 +2315,8 @@
       <x:c r="C211" s="9"/>
       <x:c r="D211" s="9"/>
       <x:c r="E211" s="9"/>
+      <x:c r="F211" s="29"/>
+      <x:c r="G211" s="29"/>
     </x:row>
     <x:row r="212">
       <x:c r="A212" s="8"/>
@@ -1828,6 +2324,8 @@
       <x:c r="C212" s="9"/>
       <x:c r="D212" s="9"/>
       <x:c r="E212" s="9"/>
+      <x:c r="F212" s="25"/>
+      <x:c r="G212" s="25"/>
     </x:row>
     <x:row r="213">
       <x:c r="A213" s="8"/>
@@ -1835,6 +2333,8 @@
       <x:c r="C213" s="9"/>
       <x:c r="D213" s="9"/>
       <x:c r="E213" s="9"/>
+      <x:c r="F213" s="29"/>
+      <x:c r="G213" s="29"/>
     </x:row>
     <x:row r="214">
       <x:c r="A214" s="8"/>
@@ -1842,6 +2342,8 @@
       <x:c r="C214" s="9"/>
       <x:c r="D214" s="9"/>
       <x:c r="E214" s="9"/>
+      <x:c r="F214" s="25"/>
+      <x:c r="G214" s="25"/>
     </x:row>
     <x:row r="215">
       <x:c r="A215" s="8"/>
@@ -1849,6 +2351,8 @@
       <x:c r="C215" s="9"/>
       <x:c r="D215" s="9"/>
       <x:c r="E215" s="9"/>
+      <x:c r="F215" s="29"/>
+      <x:c r="G215" s="29"/>
     </x:row>
     <x:row r="216">
       <x:c r="A216" s="8"/>
@@ -1856,6 +2360,8 @@
       <x:c r="C216" s="9"/>
       <x:c r="D216" s="9"/>
       <x:c r="E216" s="9"/>
+      <x:c r="F216" s="25"/>
+      <x:c r="G216" s="25"/>
     </x:row>
     <x:row r="217">
       <x:c r="A217" s="8"/>
@@ -1863,6 +2369,8 @@
       <x:c r="C217" s="9"/>
       <x:c r="D217" s="9"/>
       <x:c r="E217" s="9"/>
+      <x:c r="F217" s="29"/>
+      <x:c r="G217" s="29"/>
     </x:row>
     <x:row r="218">
       <x:c r="A218" s="8"/>
@@ -1870,6 +2378,8 @@
       <x:c r="C218" s="9"/>
       <x:c r="D218" s="9"/>
       <x:c r="E218" s="9"/>
+      <x:c r="F218" s="25"/>
+      <x:c r="G218" s="25"/>
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="8"/>
@@ -1877,6 +2387,8 @@
       <x:c r="C219" s="9"/>
       <x:c r="D219" s="9"/>
       <x:c r="E219" s="9"/>
+      <x:c r="F219" s="29"/>
+      <x:c r="G219" s="29"/>
     </x:row>
     <x:row r="220">
       <x:c r="A220" s="8"/>
@@ -1884,6 +2396,8 @@
       <x:c r="C220" s="9"/>
       <x:c r="D220" s="9"/>
       <x:c r="E220" s="9"/>
+      <x:c r="F220" s="25"/>
+      <x:c r="G220" s="25"/>
     </x:row>
     <x:row r="221">
       <x:c r="A221" s="8"/>
@@ -1891,6 +2405,8 @@
       <x:c r="C221" s="9"/>
       <x:c r="D221" s="9"/>
       <x:c r="E221" s="9"/>
+      <x:c r="F221" s="29"/>
+      <x:c r="G221" s="29"/>
     </x:row>
     <x:row r="222">
       <x:c r="A222" s="8"/>
@@ -1898,6 +2414,8 @@
       <x:c r="C222" s="9"/>
       <x:c r="D222" s="9"/>
       <x:c r="E222" s="9"/>
+      <x:c r="F222" s="25"/>
+      <x:c r="G222" s="25"/>
     </x:row>
     <x:row r="223">
       <x:c r="A223" s="8"/>
@@ -1905,6 +2423,8 @@
       <x:c r="C223" s="9"/>
       <x:c r="D223" s="9"/>
       <x:c r="E223" s="9"/>
+      <x:c r="F223" s="29"/>
+      <x:c r="G223" s="29"/>
     </x:row>
     <x:row r="224">
       <x:c r="A224" s="8"/>
@@ -1912,6 +2432,8 @@
       <x:c r="C224" s="9"/>
       <x:c r="D224" s="9"/>
       <x:c r="E224" s="9"/>
+      <x:c r="F224" s="25"/>
+      <x:c r="G224" s="25"/>
     </x:row>
     <x:row r="225">
       <x:c r="A225" s="8"/>
@@ -1919,6 +2441,8 @@
       <x:c r="C225" s="9"/>
       <x:c r="D225" s="9"/>
       <x:c r="E225" s="9"/>
+      <x:c r="F225" s="29"/>
+      <x:c r="G225" s="29"/>
     </x:row>
     <x:row r="226">
       <x:c r="A226" s="8"/>
@@ -1926,6 +2450,8 @@
       <x:c r="C226" s="9"/>
       <x:c r="D226" s="9"/>
       <x:c r="E226" s="9"/>
+      <x:c r="F226" s="25"/>
+      <x:c r="G226" s="25"/>
     </x:row>
     <x:row r="227">
       <x:c r="A227" s="8"/>
@@ -1933,6 +2459,8 @@
       <x:c r="C227" s="9"/>
       <x:c r="D227" s="9"/>
       <x:c r="E227" s="9"/>
+      <x:c r="F227" s="29"/>
+      <x:c r="G227" s="29"/>
     </x:row>
     <x:row r="228">
       <x:c r="A228" s="8"/>
@@ -1940,6 +2468,8 @@
       <x:c r="C228" s="9"/>
       <x:c r="D228" s="9"/>
       <x:c r="E228" s="9"/>
+      <x:c r="F228" s="25"/>
+      <x:c r="G228" s="25"/>
     </x:row>
     <x:row r="229">
       <x:c r="A229" s="8"/>
@@ -1947,6 +2477,8 @@
       <x:c r="C229" s="9"/>
       <x:c r="D229" s="9"/>
       <x:c r="E229" s="9"/>
+      <x:c r="F229" s="29"/>
+      <x:c r="G229" s="29"/>
     </x:row>
     <x:row r="230">
       <x:c r="A230" s="8"/>
@@ -1954,6 +2486,8 @@
       <x:c r="C230" s="9"/>
       <x:c r="D230" s="9"/>
       <x:c r="E230" s="9"/>
+      <x:c r="F230" s="25"/>
+      <x:c r="G230" s="25"/>
     </x:row>
     <x:row r="231">
       <x:c r="A231" s="8"/>
@@ -1961,6 +2495,8 @@
       <x:c r="C231" s="9"/>
       <x:c r="D231" s="9"/>
       <x:c r="E231" s="9"/>
+      <x:c r="F231" s="29"/>
+      <x:c r="G231" s="29"/>
     </x:row>
     <x:row r="232">
       <x:c r="A232" s="8"/>
@@ -1968,6 +2504,8 @@
       <x:c r="C232" s="9"/>
       <x:c r="D232" s="9"/>
       <x:c r="E232" s="9"/>
+      <x:c r="F232" s="25"/>
+      <x:c r="G232" s="25"/>
     </x:row>
     <x:row r="233">
       <x:c r="A233" s="8"/>
@@ -1975,6 +2513,8 @@
       <x:c r="C233" s="9"/>
       <x:c r="D233" s="9"/>
       <x:c r="E233" s="9"/>
+      <x:c r="F233" s="29"/>
+      <x:c r="G233" s="29"/>
     </x:row>
     <x:row r="234">
       <x:c r="A234" s="8"/>
@@ -1982,6 +2522,8 @@
       <x:c r="C234" s="9"/>
       <x:c r="D234" s="9"/>
       <x:c r="E234" s="9"/>
+      <x:c r="F234" s="25"/>
+      <x:c r="G234" s="25"/>
     </x:row>
     <x:row r="235">
       <x:c r="A235" s="8"/>
@@ -1989,6 +2531,8 @@
       <x:c r="C235" s="9"/>
       <x:c r="D235" s="9"/>
       <x:c r="E235" s="9"/>
+      <x:c r="F235" s="29"/>
+      <x:c r="G235" s="29"/>
     </x:row>
     <x:row r="236">
       <x:c r="A236" s="8"/>
@@ -1996,6 +2540,8 @@
       <x:c r="C236" s="9"/>
       <x:c r="D236" s="9"/>
       <x:c r="E236" s="9"/>
+      <x:c r="F236" s="25"/>
+      <x:c r="G236" s="25"/>
     </x:row>
     <x:row r="237">
       <x:c r="A237" s="8"/>
@@ -2003,6 +2549,8 @@
       <x:c r="C237" s="9"/>
       <x:c r="D237" s="9"/>
       <x:c r="E237" s="9"/>
+      <x:c r="F237" s="29"/>
+      <x:c r="G237" s="29"/>
     </x:row>
     <x:row r="238">
       <x:c r="A238" s="8"/>
@@ -2010,6 +2558,8 @@
       <x:c r="C238" s="9"/>
       <x:c r="D238" s="9"/>
       <x:c r="E238" s="9"/>
+      <x:c r="F238" s="25"/>
+      <x:c r="G238" s="25"/>
     </x:row>
     <x:row r="239">
       <x:c r="A239" s="8"/>
@@ -2017,6 +2567,8 @@
       <x:c r="C239" s="9"/>
       <x:c r="D239" s="9"/>
       <x:c r="E239" s="9"/>
+      <x:c r="F239" s="29"/>
+      <x:c r="G239" s="29"/>
     </x:row>
     <x:row r="240">
       <x:c r="A240" s="8"/>
@@ -2024,6 +2576,8 @@
       <x:c r="C240" s="9"/>
       <x:c r="D240" s="9"/>
       <x:c r="E240" s="9"/>
+      <x:c r="F240" s="25"/>
+      <x:c r="G240" s="25"/>
     </x:row>
     <x:row r="241">
       <x:c r="A241" s="8"/>
@@ -2031,6 +2585,8 @@
       <x:c r="C241" s="9"/>
       <x:c r="D241" s="9"/>
       <x:c r="E241" s="9"/>
+      <x:c r="F241" s="29"/>
+      <x:c r="G241" s="29"/>
     </x:row>
     <x:row r="242">
       <x:c r="A242" s="8"/>
@@ -2038,6 +2594,8 @@
       <x:c r="C242" s="9"/>
       <x:c r="D242" s="9"/>
       <x:c r="E242" s="9"/>
+      <x:c r="F242" s="25"/>
+      <x:c r="G242" s="25"/>
     </x:row>
     <x:row r="243">
       <x:c r="A243" s="8"/>
@@ -2045,6 +2603,8 @@
       <x:c r="C243" s="9"/>
       <x:c r="D243" s="9"/>
       <x:c r="E243" s="9"/>
+      <x:c r="F243" s="29"/>
+      <x:c r="G243" s="29"/>
     </x:row>
     <x:row r="244">
       <x:c r="A244" s="8"/>
@@ -2052,6 +2612,8 @@
       <x:c r="C244" s="9"/>
       <x:c r="D244" s="9"/>
       <x:c r="E244" s="9"/>
+      <x:c r="F244" s="25"/>
+      <x:c r="G244" s="25"/>
     </x:row>
     <x:row r="245">
       <x:c r="A245" s="8"/>
@@ -2059,6 +2621,8 @@
       <x:c r="C245" s="9"/>
       <x:c r="D245" s="9"/>
       <x:c r="E245" s="9"/>
+      <x:c r="F245" s="29"/>
+      <x:c r="G245" s="29"/>
     </x:row>
     <x:row r="246">
       <x:c r="A246" s="8"/>
@@ -2066,6 +2630,8 @@
       <x:c r="C246" s="9"/>
       <x:c r="D246" s="9"/>
       <x:c r="E246" s="9"/>
+      <x:c r="F246" s="25"/>
+      <x:c r="G246" s="25"/>
     </x:row>
     <x:row r="247">
       <x:c r="A247" s="8"/>
@@ -2073,6 +2639,8 @@
       <x:c r="C247" s="9"/>
       <x:c r="D247" s="9"/>
       <x:c r="E247" s="9"/>
+      <x:c r="F247" s="29"/>
+      <x:c r="G247" s="29"/>
     </x:row>
     <x:row r="248">
       <x:c r="A248" s="8"/>
@@ -2080,6 +2648,8 @@
       <x:c r="C248" s="9"/>
       <x:c r="D248" s="9"/>
       <x:c r="E248" s="9"/>
+      <x:c r="F248" s="25"/>
+      <x:c r="G248" s="25"/>
     </x:row>
     <x:row r="249">
       <x:c r="A249" s="8"/>
@@ -2087,6 +2657,8 @@
       <x:c r="C249" s="9"/>
       <x:c r="D249" s="9"/>
       <x:c r="E249" s="9"/>
+      <x:c r="F249" s="29"/>
+      <x:c r="G249" s="29"/>
     </x:row>
     <x:row r="250">
       <x:c r="A250" s="8"/>
@@ -2094,6 +2666,8 @@
       <x:c r="C250" s="9"/>
       <x:c r="D250" s="9"/>
       <x:c r="E250" s="9"/>
+      <x:c r="F250" s="25"/>
+      <x:c r="G250" s="25"/>
     </x:row>
     <x:row r="251">
       <x:c r="A251" s="8"/>
@@ -2101,6 +2675,8 @@
       <x:c r="C251" s="9"/>
       <x:c r="D251" s="9"/>
       <x:c r="E251" s="9"/>
+      <x:c r="F251" s="29"/>
+      <x:c r="G251" s="29"/>
     </x:row>
     <x:row r="252">
       <x:c r="A252" s="8"/>
@@ -2108,6 +2684,8 @@
       <x:c r="C252" s="9"/>
       <x:c r="D252" s="9"/>
       <x:c r="E252" s="9"/>
+      <x:c r="F252" s="25"/>
+      <x:c r="G252" s="25"/>
     </x:row>
     <x:row r="253">
       <x:c r="A253" s="8"/>
@@ -2115,6 +2693,8 @@
       <x:c r="C253" s="9"/>
       <x:c r="D253" s="9"/>
       <x:c r="E253" s="9"/>
+      <x:c r="F253" s="29"/>
+      <x:c r="G253" s="29"/>
     </x:row>
     <x:row r="254">
       <x:c r="A254" s="8"/>
@@ -2122,6 +2702,8 @@
       <x:c r="C254" s="9"/>
       <x:c r="D254" s="9"/>
       <x:c r="E254" s="9"/>
+      <x:c r="F254" s="25"/>
+      <x:c r="G254" s="25"/>
     </x:row>
     <x:row r="255">
       <x:c r="A255" s="8"/>
@@ -2129,6 +2711,8 @@
       <x:c r="C255" s="9"/>
       <x:c r="D255" s="9"/>
       <x:c r="E255" s="9"/>
+      <x:c r="F255" s="29"/>
+      <x:c r="G255" s="29"/>
     </x:row>
     <x:row r="256">
       <x:c r="A256" s="8"/>
@@ -2136,6 +2720,8 @@
       <x:c r="C256" s="9"/>
       <x:c r="D256" s="9"/>
       <x:c r="E256" s="9"/>
+      <x:c r="F256" s="25"/>
+      <x:c r="G256" s="25"/>
     </x:row>
     <x:row r="257">
       <x:c r="A257" s="8"/>
@@ -2143,6 +2729,8 @@
       <x:c r="C257" s="9"/>
       <x:c r="D257" s="9"/>
       <x:c r="E257" s="9"/>
+      <x:c r="F257" s="29"/>
+      <x:c r="G257" s="29"/>
     </x:row>
     <x:row r="258">
       <x:c r="A258" s="8"/>
@@ -2150,6 +2738,8 @@
       <x:c r="C258" s="9"/>
       <x:c r="D258" s="9"/>
       <x:c r="E258" s="9"/>
+      <x:c r="F258" s="25"/>
+      <x:c r="G258" s="25"/>
     </x:row>
     <x:row r="259">
       <x:c r="A259" s="8"/>
@@ -2157,6 +2747,8 @@
       <x:c r="C259" s="9"/>
       <x:c r="D259" s="9"/>
       <x:c r="E259" s="9"/>
+      <x:c r="F259" s="29"/>
+      <x:c r="G259" s="29"/>
     </x:row>
     <x:row r="260">
       <x:c r="A260" s="8"/>
@@ -2164,6 +2756,8 @@
       <x:c r="C260" s="9"/>
       <x:c r="D260" s="9"/>
       <x:c r="E260" s="9"/>
+      <x:c r="F260" s="25"/>
+      <x:c r="G260" s="25"/>
     </x:row>
     <x:row r="261">
       <x:c r="A261" s="8"/>
@@ -2171,6 +2765,8 @@
       <x:c r="C261" s="9"/>
       <x:c r="D261" s="9"/>
       <x:c r="E261" s="9"/>
+      <x:c r="F261" s="29"/>
+      <x:c r="G261" s="29"/>
     </x:row>
     <x:row r="262">
       <x:c r="A262" s="8"/>
@@ -2178,6 +2774,8 @@
       <x:c r="C262" s="9"/>
       <x:c r="D262" s="9"/>
       <x:c r="E262" s="9"/>
+      <x:c r="F262" s="25"/>
+      <x:c r="G262" s="25"/>
     </x:row>
     <x:row r="263">
       <x:c r="A263" s="8"/>
@@ -2185,6 +2783,8 @@
       <x:c r="C263" s="9"/>
       <x:c r="D263" s="9"/>
       <x:c r="E263" s="9"/>
+      <x:c r="F263" s="29"/>
+      <x:c r="G263" s="29"/>
     </x:row>
     <x:row r="264">
       <x:c r="A264" s="8"/>
@@ -2192,6 +2792,8 @@
       <x:c r="C264" s="9"/>
       <x:c r="D264" s="9"/>
       <x:c r="E264" s="9"/>
+      <x:c r="F264" s="25"/>
+      <x:c r="G264" s="25"/>
     </x:row>
     <x:row r="265">
       <x:c r="A265" s="8"/>
@@ -2199,6 +2801,8 @@
       <x:c r="C265" s="9"/>
       <x:c r="D265" s="9"/>
       <x:c r="E265" s="9"/>
+      <x:c r="F265" s="29"/>
+      <x:c r="G265" s="29"/>
     </x:row>
     <x:row r="266">
       <x:c r="A266" s="8"/>
@@ -2206,6 +2810,8 @@
       <x:c r="C266" s="9"/>
       <x:c r="D266" s="9"/>
       <x:c r="E266" s="9"/>
+      <x:c r="F266" s="25"/>
+      <x:c r="G266" s="25"/>
     </x:row>
     <x:row r="267">
       <x:c r="A267" s="8"/>
@@ -2213,6 +2819,8 @@
       <x:c r="C267" s="9"/>
       <x:c r="D267" s="9"/>
       <x:c r="E267" s="9"/>
+      <x:c r="F267" s="29"/>
+      <x:c r="G267" s="29"/>
     </x:row>
     <x:row r="268">
       <x:c r="A268" s="8"/>
@@ -2220,6 +2828,8 @@
       <x:c r="C268" s="9"/>
       <x:c r="D268" s="9"/>
       <x:c r="E268" s="9"/>
+      <x:c r="F268" s="25"/>
+      <x:c r="G268" s="25"/>
     </x:row>
     <x:row r="269">
       <x:c r="A269" s="8"/>
@@ -2227,6 +2837,8 @@
       <x:c r="C269" s="9"/>
       <x:c r="D269" s="9"/>
       <x:c r="E269" s="9"/>
+      <x:c r="F269" s="29"/>
+      <x:c r="G269" s="29"/>
     </x:row>
     <x:row r="270">
       <x:c r="A270" s="8"/>
@@ -2234,6 +2846,8 @@
       <x:c r="C270" s="9"/>
       <x:c r="D270" s="9"/>
       <x:c r="E270" s="9"/>
+      <x:c r="F270" s="25"/>
+      <x:c r="G270" s="25"/>
     </x:row>
     <x:row r="271">
       <x:c r="A271" s="8"/>
@@ -2241,6 +2855,8 @@
       <x:c r="C271" s="9"/>
       <x:c r="D271" s="9"/>
       <x:c r="E271" s="9"/>
+      <x:c r="F271" s="29"/>
+      <x:c r="G271" s="29"/>
     </x:row>
     <x:row r="272">
       <x:c r="A272" s="8"/>
@@ -2248,6 +2864,8 @@
       <x:c r="C272" s="9"/>
       <x:c r="D272" s="9"/>
       <x:c r="E272" s="9"/>
+      <x:c r="F272" s="25"/>
+      <x:c r="G272" s="25"/>
     </x:row>
     <x:row r="273">
       <x:c r="A273" s="8"/>
@@ -2255,6 +2873,8 @@
       <x:c r="C273" s="9"/>
       <x:c r="D273" s="9"/>
       <x:c r="E273" s="9"/>
+      <x:c r="F273" s="29"/>
+      <x:c r="G273" s="29"/>
     </x:row>
     <x:row r="274">
       <x:c r="A274" s="8"/>
@@ -2262,6 +2882,8 @@
       <x:c r="C274" s="9"/>
       <x:c r="D274" s="9"/>
       <x:c r="E274" s="9"/>
+      <x:c r="F274" s="25"/>
+      <x:c r="G274" s="25"/>
     </x:row>
     <x:row r="275">
       <x:c r="A275" s="8"/>
@@ -2269,6 +2891,8 @@
       <x:c r="C275" s="9"/>
       <x:c r="D275" s="9"/>
       <x:c r="E275" s="9"/>
+      <x:c r="F275" s="29"/>
+      <x:c r="G275" s="29"/>
     </x:row>
     <x:row r="276">
       <x:c r="A276" s="8"/>
@@ -2276,6 +2900,8 @@
       <x:c r="C276" s="9"/>
       <x:c r="D276" s="9"/>
       <x:c r="E276" s="9"/>
+      <x:c r="F276" s="25"/>
+      <x:c r="G276" s="25"/>
     </x:row>
     <x:row r="277">
       <x:c r="A277" s="8"/>
@@ -2283,6 +2909,8 @@
       <x:c r="C277" s="9"/>
       <x:c r="D277" s="9"/>
       <x:c r="E277" s="9"/>
+      <x:c r="F277" s="29"/>
+      <x:c r="G277" s="29"/>
     </x:row>
     <x:row r="278">
       <x:c r="A278" s="8"/>
@@ -2290,6 +2918,8 @@
       <x:c r="C278" s="9"/>
       <x:c r="D278" s="9"/>
       <x:c r="E278" s="9"/>
+      <x:c r="F278" s="25"/>
+      <x:c r="G278" s="25"/>
     </x:row>
     <x:row r="279">
       <x:c r="A279" s="8"/>
@@ -2297,6 +2927,8 @@
       <x:c r="C279" s="9"/>
       <x:c r="D279" s="9"/>
       <x:c r="E279" s="9"/>
+      <x:c r="F279" s="29"/>
+      <x:c r="G279" s="29"/>
     </x:row>
     <x:row r="280">
       <x:c r="A280" s="8"/>
@@ -2304,6 +2936,8 @@
       <x:c r="C280" s="9"/>
       <x:c r="D280" s="9"/>
       <x:c r="E280" s="9"/>
+      <x:c r="F280" s="25"/>
+      <x:c r="G280" s="25"/>
     </x:row>
     <x:row r="281">
       <x:c r="A281" s="8"/>
@@ -2311,6 +2945,8 @@
       <x:c r="C281" s="9"/>
       <x:c r="D281" s="9"/>
       <x:c r="E281" s="9"/>
+      <x:c r="F281" s="29"/>
+      <x:c r="G281" s="29"/>
     </x:row>
     <x:row r="282">
       <x:c r="A282" s="8"/>
@@ -2318,6 +2954,8 @@
       <x:c r="C282" s="9"/>
       <x:c r="D282" s="9"/>
       <x:c r="E282" s="9"/>
+      <x:c r="F282" s="25"/>
+      <x:c r="G282" s="25"/>
     </x:row>
     <x:row r="283">
       <x:c r="A283" s="8"/>
@@ -2325,6 +2963,8 @@
       <x:c r="C283" s="9"/>
       <x:c r="D283" s="9"/>
       <x:c r="E283" s="9"/>
+      <x:c r="F283" s="29"/>
+      <x:c r="G283" s="29"/>
     </x:row>
     <x:row r="284">
       <x:c r="A284" s="8"/>
@@ -2332,6 +2972,8 @@
       <x:c r="C284" s="9"/>
       <x:c r="D284" s="9"/>
       <x:c r="E284" s="9"/>
+      <x:c r="F284" s="25"/>
+      <x:c r="G284" s="25"/>
     </x:row>
     <x:row r="285">
       <x:c r="A285" s="8"/>
@@ -2339,6 +2981,8 @@
       <x:c r="C285" s="9"/>
       <x:c r="D285" s="9"/>
       <x:c r="E285" s="9"/>
+      <x:c r="F285" s="29"/>
+      <x:c r="G285" s="29"/>
     </x:row>
     <x:row r="286">
       <x:c r="A286" s="8"/>
@@ -2346,6 +2990,8 @@
       <x:c r="C286" s="9"/>
       <x:c r="D286" s="9"/>
       <x:c r="E286" s="9"/>
+      <x:c r="F286" s="25"/>
+      <x:c r="G286" s="25"/>
     </x:row>
     <x:row r="287">
       <x:c r="A287" s="8"/>
@@ -2353,6 +2999,8 @@
       <x:c r="C287" s="9"/>
       <x:c r="D287" s="9"/>
       <x:c r="E287" s="9"/>
+      <x:c r="F287" s="29"/>
+      <x:c r="G287" s="29"/>
     </x:row>
     <x:row r="288">
       <x:c r="A288" s="8"/>
@@ -2360,6 +3008,8 @@
       <x:c r="C288" s="9"/>
       <x:c r="D288" s="9"/>
       <x:c r="E288" s="9"/>
+      <x:c r="F288" s="25"/>
+      <x:c r="G288" s="25"/>
     </x:row>
     <x:row r="289">
       <x:c r="A289" s="8"/>
@@ -2367,6 +3017,8 @@
       <x:c r="C289" s="9"/>
       <x:c r="D289" s="9"/>
       <x:c r="E289" s="9"/>
+      <x:c r="F289" s="29"/>
+      <x:c r="G289" s="29"/>
     </x:row>
     <x:row r="290">
       <x:c r="A290" s="8"/>
@@ -2374,6 +3026,8 @@
       <x:c r="C290" s="9"/>
       <x:c r="D290" s="9"/>
       <x:c r="E290" s="9"/>
+      <x:c r="F290" s="25"/>
+      <x:c r="G290" s="25"/>
     </x:row>
     <x:row r="291">
       <x:c r="A291" s="8"/>
@@ -2381,6 +3035,8 @@
       <x:c r="C291" s="9"/>
       <x:c r="D291" s="9"/>
       <x:c r="E291" s="9"/>
+      <x:c r="F291" s="29"/>
+      <x:c r="G291" s="29"/>
     </x:row>
     <x:row r="292">
       <x:c r="A292" s="8"/>
@@ -2388,6 +3044,8 @@
       <x:c r="C292" s="9"/>
       <x:c r="D292" s="9"/>
       <x:c r="E292" s="9"/>
+      <x:c r="F292" s="25"/>
+      <x:c r="G292" s="25"/>
     </x:row>
     <x:row r="293">
       <x:c r="A293" s="8"/>
@@ -2395,6 +3053,8 @@
       <x:c r="C293" s="9"/>
       <x:c r="D293" s="9"/>
       <x:c r="E293" s="9"/>
+      <x:c r="F293" s="29"/>
+      <x:c r="G293" s="29"/>
     </x:row>
     <x:row r="294">
       <x:c r="A294" s="8"/>
@@ -2402,6 +3062,8 @@
       <x:c r="C294" s="9"/>
       <x:c r="D294" s="9"/>
       <x:c r="E294" s="9"/>
+      <x:c r="F294" s="25"/>
+      <x:c r="G294" s="25"/>
     </x:row>
     <x:row r="295">
       <x:c r="A295" s="8"/>
@@ -2409,6 +3071,8 @@
       <x:c r="C295" s="9"/>
       <x:c r="D295" s="9"/>
       <x:c r="E295" s="9"/>
+      <x:c r="F295" s="29"/>
+      <x:c r="G295" s="29"/>
     </x:row>
     <x:row r="296">
       <x:c r="A296" s="8"/>
@@ -2416,6 +3080,8 @@
       <x:c r="C296" s="9"/>
       <x:c r="D296" s="9"/>
       <x:c r="E296" s="9"/>
+      <x:c r="F296" s="25"/>
+      <x:c r="G296" s="25"/>
     </x:row>
     <x:row r="297">
       <x:c r="A297" s="8"/>
@@ -2423,6 +3089,8 @@
       <x:c r="C297" s="9"/>
       <x:c r="D297" s="9"/>
       <x:c r="E297" s="9"/>
+      <x:c r="F297" s="29"/>
+      <x:c r="G297" s="29"/>
     </x:row>
     <x:row r="298">
       <x:c r="A298" s="8"/>
@@ -2430,6 +3098,8 @@
       <x:c r="C298" s="9"/>
       <x:c r="D298" s="9"/>
       <x:c r="E298" s="9"/>
+      <x:c r="F298" s="25"/>
+      <x:c r="G298" s="25"/>
     </x:row>
     <x:row r="299">
       <x:c r="A299" s="8"/>
@@ -2437,6 +3107,8 @@
       <x:c r="C299" s="9"/>
       <x:c r="D299" s="9"/>
       <x:c r="E299" s="9"/>
+      <x:c r="F299" s="29"/>
+      <x:c r="G299" s="29"/>
     </x:row>
     <x:row r="300">
       <x:c r="A300" s="8"/>
@@ -2444,6 +3116,8 @@
       <x:c r="C300" s="9"/>
       <x:c r="D300" s="9"/>
       <x:c r="E300" s="9"/>
+      <x:c r="F300" s="25"/>
+      <x:c r="G300" s="25"/>
     </x:row>
     <x:row r="301">
       <x:c r="A301" s="8"/>
@@ -2451,6 +3125,8 @@
       <x:c r="C301" s="9"/>
       <x:c r="D301" s="9"/>
       <x:c r="E301" s="9"/>
+      <x:c r="F301" s="29"/>
+      <x:c r="G301" s="29"/>
     </x:row>
     <x:row r="302">
       <x:c r="A302" s="8"/>
@@ -2458,6 +3134,8 @@
       <x:c r="C302" s="9"/>
       <x:c r="D302" s="9"/>
       <x:c r="E302" s="9"/>
+      <x:c r="F302" s="25"/>
+      <x:c r="G302" s="25"/>
     </x:row>
     <x:row r="303">
       <x:c r="A303" s="8"/>
@@ -2465,6 +3143,8 @@
       <x:c r="C303" s="9"/>
       <x:c r="D303" s="9"/>
       <x:c r="E303" s="9"/>
+      <x:c r="F303" s="29"/>
+      <x:c r="G303" s="29"/>
     </x:row>
     <x:row r="304">
       <x:c r="A304" s="8"/>
@@ -2472,6 +3152,8 @@
       <x:c r="C304" s="9"/>
       <x:c r="D304" s="9"/>
       <x:c r="E304" s="9"/>
+      <x:c r="F304" s="25"/>
+      <x:c r="G304" s="25"/>
     </x:row>
     <x:row r="305">
       <x:c r="A305" s="8"/>
@@ -2479,6 +3161,8 @@
       <x:c r="C305" s="9"/>
       <x:c r="D305" s="9"/>
       <x:c r="E305" s="9"/>
+      <x:c r="F305" s="29"/>
+      <x:c r="G305" s="29"/>
     </x:row>
     <x:row r="306">
       <x:c r="A306" s="8"/>
@@ -2486,6 +3170,8 @@
       <x:c r="C306" s="9"/>
       <x:c r="D306" s="9"/>
       <x:c r="E306" s="9"/>
+      <x:c r="F306" s="25"/>
+      <x:c r="G306" s="25"/>
     </x:row>
     <x:row r="307">
       <x:c r="A307" s="8"/>
@@ -2493,6 +3179,8 @@
       <x:c r="C307" s="9"/>
       <x:c r="D307" s="9"/>
       <x:c r="E307" s="9"/>
+      <x:c r="F307" s="29"/>
+      <x:c r="G307" s="29"/>
     </x:row>
     <x:row r="308">
       <x:c r="A308" s="8"/>
@@ -2500,6 +3188,8 @@
       <x:c r="C308" s="9"/>
       <x:c r="D308" s="9"/>
       <x:c r="E308" s="9"/>
+      <x:c r="F308" s="25"/>
+      <x:c r="G308" s="25"/>
     </x:row>
     <x:row r="309">
       <x:c r="A309" s="8"/>
@@ -2507,6 +3197,8 @@
       <x:c r="C309" s="9"/>
       <x:c r="D309" s="9"/>
       <x:c r="E309" s="9"/>
+      <x:c r="F309" s="29"/>
+      <x:c r="G309" s="29"/>
     </x:row>
     <x:row r="310">
       <x:c r="A310" s="8"/>
@@ -2514,6 +3206,8 @@
       <x:c r="C310" s="9"/>
       <x:c r="D310" s="9"/>
       <x:c r="E310" s="9"/>
+      <x:c r="F310" s="25"/>
+      <x:c r="G310" s="25"/>
     </x:row>
     <x:row r="311">
       <x:c r="A311" s="8"/>
@@ -2521,6 +3215,8 @@
       <x:c r="C311" s="9"/>
       <x:c r="D311" s="9"/>
       <x:c r="E311" s="9"/>
+      <x:c r="F311" s="29"/>
+      <x:c r="G311" s="29"/>
     </x:row>
     <x:row r="312">
       <x:c r="A312" s="8"/>
@@ -2528,6 +3224,8 @@
       <x:c r="C312" s="9"/>
       <x:c r="D312" s="9"/>
       <x:c r="E312" s="9"/>
+      <x:c r="F312" s="25"/>
+      <x:c r="G312" s="25"/>
     </x:row>
     <x:row r="313">
       <x:c r="A313" s="8"/>
@@ -2535,6 +3233,8 @@
       <x:c r="C313" s="9"/>
       <x:c r="D313" s="9"/>
       <x:c r="E313" s="9"/>
+      <x:c r="F313" s="29"/>
+      <x:c r="G313" s="29"/>
     </x:row>
     <x:row r="314">
       <x:c r="A314" s="8"/>
@@ -2542,6 +3242,8 @@
       <x:c r="C314" s="9"/>
       <x:c r="D314" s="9"/>
       <x:c r="E314" s="9"/>
+      <x:c r="F314" s="25"/>
+      <x:c r="G314" s="25"/>
     </x:row>
     <x:row r="315">
       <x:c r="A315" s="8"/>
@@ -2549,6 +3251,8 @@
       <x:c r="C315" s="9"/>
       <x:c r="D315" s="9"/>
       <x:c r="E315" s="9"/>
+      <x:c r="F315" s="29"/>
+      <x:c r="G315" s="29"/>
     </x:row>
     <x:row r="316">
       <x:c r="A316" s="8"/>
@@ -2556,6 +3260,8 @@
       <x:c r="C316" s="9"/>
       <x:c r="D316" s="9"/>
       <x:c r="E316" s="9"/>
+      <x:c r="F316" s="25"/>
+      <x:c r="G316" s="25"/>
     </x:row>
     <x:row r="317">
       <x:c r="A317" s="8"/>
@@ -2563,6 +3269,8 @@
       <x:c r="C317" s="9"/>
       <x:c r="D317" s="9"/>
       <x:c r="E317" s="9"/>
+      <x:c r="F317" s="29"/>
+      <x:c r="G317" s="29"/>
     </x:row>
     <x:row r="318">
       <x:c r="A318" s="8"/>
@@ -2570,6 +3278,8 @@
       <x:c r="C318" s="9"/>
       <x:c r="D318" s="9"/>
       <x:c r="E318" s="9"/>
+      <x:c r="F318" s="25"/>
+      <x:c r="G318" s="25"/>
     </x:row>
     <x:row r="319">
       <x:c r="A319" s="8"/>
@@ -2577,6 +3287,8 @@
       <x:c r="C319" s="9"/>
       <x:c r="D319" s="9"/>
       <x:c r="E319" s="9"/>
+      <x:c r="F319" s="29"/>
+      <x:c r="G319" s="29"/>
     </x:row>
     <x:row r="320">
       <x:c r="A320" s="8"/>
@@ -2584,6 +3296,8 @@
       <x:c r="C320" s="9"/>
       <x:c r="D320" s="9"/>
       <x:c r="E320" s="9"/>
+      <x:c r="F320" s="25"/>
+      <x:c r="G320" s="25"/>
     </x:row>
     <x:row r="321">
       <x:c r="A321" s="8"/>
@@ -2591,6 +3305,8 @@
       <x:c r="C321" s="9"/>
       <x:c r="D321" s="9"/>
       <x:c r="E321" s="9"/>
+      <x:c r="F321" s="29"/>
+      <x:c r="G321" s="29"/>
     </x:row>
     <x:row r="322">
       <x:c r="A322" s="8"/>
@@ -2598,6 +3314,8 @@
       <x:c r="C322" s="9"/>
       <x:c r="D322" s="9"/>
       <x:c r="E322" s="9"/>
+      <x:c r="F322" s="25"/>
+      <x:c r="G322" s="25"/>
     </x:row>
     <x:row r="323">
       <x:c r="A323" s="8"/>
@@ -2605,6 +3323,8 @@
       <x:c r="C323" s="9"/>
       <x:c r="D323" s="9"/>
       <x:c r="E323" s="9"/>
+      <x:c r="F323" s="29"/>
+      <x:c r="G323" s="29"/>
     </x:row>
     <x:row r="324">
       <x:c r="A324" s="8"/>
@@ -2612,6 +3332,8 @@
       <x:c r="C324" s="9"/>
       <x:c r="D324" s="9"/>
       <x:c r="E324" s="9"/>
+      <x:c r="F324" s="25"/>
+      <x:c r="G324" s="25"/>
     </x:row>
     <x:row r="325">
       <x:c r="A325" s="8"/>
@@ -2619,6 +3341,8 @@
       <x:c r="C325" s="9"/>
       <x:c r="D325" s="9"/>
       <x:c r="E325" s="9"/>
+      <x:c r="F325" s="29"/>
+      <x:c r="G325" s="29"/>
     </x:row>
     <x:row r="326">
       <x:c r="A326" s="8"/>
@@ -2626,6 +3350,8 @@
       <x:c r="C326" s="9"/>
       <x:c r="D326" s="9"/>
       <x:c r="E326" s="9"/>
+      <x:c r="F326" s="25"/>
+      <x:c r="G326" s="25"/>
     </x:row>
     <x:row r="327">
       <x:c r="A327" s="8"/>
@@ -2633,6 +3359,8 @@
       <x:c r="C327" s="9"/>
       <x:c r="D327" s="9"/>
       <x:c r="E327" s="9"/>
+      <x:c r="F327" s="29"/>
+      <x:c r="G327" s="29"/>
     </x:row>
     <x:row r="328">
       <x:c r="A328" s="8"/>
@@ -2640,6 +3368,8 @@
       <x:c r="C328" s="9"/>
       <x:c r="D328" s="9"/>
       <x:c r="E328" s="9"/>
+      <x:c r="F328" s="25"/>
+      <x:c r="G328" s="25"/>
     </x:row>
     <x:row r="329">
       <x:c r="A329" s="8"/>
@@ -2647,6 +3377,8 @@
       <x:c r="C329" s="9"/>
       <x:c r="D329" s="9"/>
       <x:c r="E329" s="9"/>
+      <x:c r="F329" s="29"/>
+      <x:c r="G329" s="29"/>
     </x:row>
     <x:row r="330">
       <x:c r="A330" s="8"/>
@@ -2654,6 +3386,8 @@
       <x:c r="C330" s="9"/>
       <x:c r="D330" s="9"/>
       <x:c r="E330" s="9"/>
+      <x:c r="F330" s="25"/>
+      <x:c r="G330" s="25"/>
     </x:row>
     <x:row r="331">
       <x:c r="A331" s="8"/>
@@ -2661,6 +3395,8 @@
       <x:c r="C331" s="9"/>
       <x:c r="D331" s="9"/>
       <x:c r="E331" s="9"/>
+      <x:c r="F331" s="29"/>
+      <x:c r="G331" s="29"/>
     </x:row>
     <x:row r="332">
       <x:c r="A332" s="8"/>
@@ -2668,6 +3404,8 @@
       <x:c r="C332" s="9"/>
       <x:c r="D332" s="9"/>
       <x:c r="E332" s="9"/>
+      <x:c r="F332" s="25"/>
+      <x:c r="G332" s="25"/>
     </x:row>
     <x:row r="333">
       <x:c r="A333" s="8"/>
@@ -2675,6 +3413,8 @@
       <x:c r="C333" s="9"/>
       <x:c r="D333" s="9"/>
       <x:c r="E333" s="9"/>
+      <x:c r="F333" s="29"/>
+      <x:c r="G333" s="29"/>
     </x:row>
     <x:row r="334">
       <x:c r="A334" s="8"/>
@@ -2682,6 +3422,8 @@
       <x:c r="C334" s="9"/>
       <x:c r="D334" s="9"/>
       <x:c r="E334" s="9"/>
+      <x:c r="F334" s="25"/>
+      <x:c r="G334" s="25"/>
     </x:row>
     <x:row r="335">
       <x:c r="A335" s="8"/>
@@ -2689,6 +3431,8 @@
       <x:c r="C335" s="9"/>
       <x:c r="D335" s="9"/>
       <x:c r="E335" s="9"/>
+      <x:c r="F335" s="29"/>
+      <x:c r="G335" s="29"/>
     </x:row>
     <x:row r="336">
       <x:c r="A336" s="8"/>
@@ -2696,6 +3440,8 @@
       <x:c r="C336" s="9"/>
       <x:c r="D336" s="9"/>
       <x:c r="E336" s="9"/>
+      <x:c r="F336" s="25"/>
+      <x:c r="G336" s="25"/>
     </x:row>
     <x:row r="337">
       <x:c r="A337" s="8"/>
@@ -2703,6 +3449,8 @@
       <x:c r="C337" s="9"/>
       <x:c r="D337" s="9"/>
       <x:c r="E337" s="9"/>
+      <x:c r="F337" s="29"/>
+      <x:c r="G337" s="29"/>
     </x:row>
     <x:row r="338">
       <x:c r="A338" s="8"/>
@@ -2710,6 +3458,8 @@
       <x:c r="C338" s="9"/>
       <x:c r="D338" s="9"/>
       <x:c r="E338" s="9"/>
+      <x:c r="F338" s="25"/>
+      <x:c r="G338" s="25"/>
     </x:row>
     <x:row r="339">
       <x:c r="A339" s="8"/>
@@ -2717,6 +3467,8 @@
       <x:c r="C339" s="9"/>
       <x:c r="D339" s="9"/>
       <x:c r="E339" s="9"/>
+      <x:c r="F339" s="29"/>
+      <x:c r="G339" s="29"/>
     </x:row>
     <x:row r="340">
       <x:c r="A340" s="8"/>
@@ -2724,6 +3476,8 @@
       <x:c r="C340" s="9"/>
       <x:c r="D340" s="9"/>
       <x:c r="E340" s="9"/>
+      <x:c r="F340" s="25"/>
+      <x:c r="G340" s="25"/>
     </x:row>
     <x:row r="341">
       <x:c r="A341" s="8"/>
@@ -2731,6 +3485,8 @@
       <x:c r="C341" s="9"/>
       <x:c r="D341" s="9"/>
       <x:c r="E341" s="9"/>
+      <x:c r="F341" s="29"/>
+      <x:c r="G341" s="29"/>
     </x:row>
     <x:row r="342">
       <x:c r="A342" s="8"/>
@@ -2738,6 +3494,8 @@
       <x:c r="C342" s="9"/>
       <x:c r="D342" s="9"/>
       <x:c r="E342" s="9"/>
+      <x:c r="F342" s="25"/>
+      <x:c r="G342" s="25"/>
     </x:row>
     <x:row r="343">
       <x:c r="A343" s="8"/>
@@ -2745,6 +3503,8 @@
       <x:c r="C343" s="9"/>
       <x:c r="D343" s="9"/>
       <x:c r="E343" s="9"/>
+      <x:c r="F343" s="29"/>
+      <x:c r="G343" s="29"/>
     </x:row>
     <x:row r="344">
       <x:c r="A344" s="8"/>
@@ -2752,6 +3512,8 @@
       <x:c r="C344" s="9"/>
       <x:c r="D344" s="9"/>
       <x:c r="E344" s="9"/>
+      <x:c r="F344" s="25"/>
+      <x:c r="G344" s="25"/>
     </x:row>
     <x:row r="345">
       <x:c r="A345" s="8"/>
@@ -2759,6 +3521,8 @@
       <x:c r="C345" s="9"/>
       <x:c r="D345" s="9"/>
       <x:c r="E345" s="9"/>
+      <x:c r="F345" s="29"/>
+      <x:c r="G345" s="29"/>
     </x:row>
     <x:row r="346">
       <x:c r="A346" s="8"/>
@@ -2766,6 +3530,8 @@
       <x:c r="C346" s="9"/>
       <x:c r="D346" s="9"/>
       <x:c r="E346" s="9"/>
+      <x:c r="F346" s="25"/>
+      <x:c r="G346" s="25"/>
     </x:row>
     <x:row r="347">
       <x:c r="A347" s="8"/>
@@ -2773,6 +3539,8 @@
       <x:c r="C347" s="9"/>
       <x:c r="D347" s="9"/>
       <x:c r="E347" s="9"/>
+      <x:c r="F347" s="29"/>
+      <x:c r="G347" s="29"/>
     </x:row>
     <x:row r="348">
       <x:c r="A348" s="8"/>
@@ -2780,6 +3548,8 @@
       <x:c r="C348" s="9"/>
       <x:c r="D348" s="9"/>
       <x:c r="E348" s="9"/>
+      <x:c r="F348" s="25"/>
+      <x:c r="G348" s="25"/>
     </x:row>
     <x:row r="349">
       <x:c r="A349" s="8"/>
@@ -2787,6 +3557,8 @@
       <x:c r="C349" s="9"/>
       <x:c r="D349" s="9"/>
       <x:c r="E349" s="9"/>
+      <x:c r="F349" s="29"/>
+      <x:c r="G349" s="29"/>
     </x:row>
     <x:row r="350">
       <x:c r="A350" s="8"/>
@@ -2794,6 +3566,8 @@
       <x:c r="C350" s="9"/>
       <x:c r="D350" s="9"/>
       <x:c r="E350" s="9"/>
+      <x:c r="F350" s="25"/>
+      <x:c r="G350" s="25"/>
     </x:row>
     <x:row r="351">
       <x:c r="A351" s="8"/>
@@ -2801,6 +3575,8 @@
       <x:c r="C351" s="9"/>
       <x:c r="D351" s="9"/>
       <x:c r="E351" s="9"/>
+      <x:c r="F351" s="29"/>
+      <x:c r="G351" s="29"/>
     </x:row>
     <x:row r="352">
       <x:c r="A352" s="8"/>
@@ -2808,6 +3584,8 @@
       <x:c r="C352" s="9"/>
       <x:c r="D352" s="9"/>
       <x:c r="E352" s="9"/>
+      <x:c r="F352" s="25"/>
+      <x:c r="G352" s="25"/>
     </x:row>
     <x:row r="353">
       <x:c r="A353" s="8"/>
@@ -2815,6 +3593,8 @@
       <x:c r="C353" s="9"/>
       <x:c r="D353" s="9"/>
       <x:c r="E353" s="9"/>
+      <x:c r="F353" s="29"/>
+      <x:c r="G353" s="29"/>
     </x:row>
     <x:row r="354">
       <x:c r="A354" s="8"/>
@@ -2822,6 +3602,8 @@
       <x:c r="C354" s="9"/>
       <x:c r="D354" s="9"/>
       <x:c r="E354" s="9"/>
+      <x:c r="F354" s="25"/>
+      <x:c r="G354" s="25"/>
     </x:row>
     <x:row r="355">
       <x:c r="A355" s="8"/>
@@ -2829,6 +3611,8 @@
       <x:c r="C355" s="9"/>
       <x:c r="D355" s="9"/>
       <x:c r="E355" s="9"/>
+      <x:c r="F355" s="29"/>
+      <x:c r="G355" s="29"/>
     </x:row>
     <x:row r="356">
       <x:c r="A356" s="8"/>
@@ -2836,6 +3620,8 @@
       <x:c r="C356" s="9"/>
       <x:c r="D356" s="9"/>
       <x:c r="E356" s="9"/>
+      <x:c r="F356" s="25"/>
+      <x:c r="G356" s="25"/>
     </x:row>
     <x:row r="357">
       <x:c r="A357" s="8"/>
@@ -2843,6 +3629,8 @@
       <x:c r="C357" s="9"/>
       <x:c r="D357" s="9"/>
       <x:c r="E357" s="9"/>
+      <x:c r="F357" s="29"/>
+      <x:c r="G357" s="29"/>
     </x:row>
     <x:row r="358">
       <x:c r="A358" s="8"/>
@@ -2850,6 +3638,8 @@
       <x:c r="C358" s="9"/>
       <x:c r="D358" s="9"/>
       <x:c r="E358" s="9"/>
+      <x:c r="F358" s="25"/>
+      <x:c r="G358" s="25"/>
     </x:row>
     <x:row r="359">
       <x:c r="A359" s="8"/>
@@ -2857,6 +3647,8 @@
       <x:c r="C359" s="9"/>
       <x:c r="D359" s="9"/>
       <x:c r="E359" s="9"/>
+      <x:c r="F359" s="29"/>
+      <x:c r="G359" s="29"/>
     </x:row>
     <x:row r="360">
       <x:c r="A360" s="8"/>
@@ -2864,6 +3656,8 @@
       <x:c r="C360" s="9"/>
       <x:c r="D360" s="9"/>
       <x:c r="E360" s="9"/>
+      <x:c r="F360" s="25"/>
+      <x:c r="G360" s="25"/>
     </x:row>
     <x:row r="361">
       <x:c r="A361" s="8"/>
@@ -2871,6 +3665,8 @@
       <x:c r="C361" s="9"/>
       <x:c r="D361" s="9"/>
       <x:c r="E361" s="9"/>
+      <x:c r="F361" s="29"/>
+      <x:c r="G361" s="29"/>
     </x:row>
     <x:row r="362">
       <x:c r="A362" s="8"/>
@@ -2878,6 +3674,8 @@
       <x:c r="C362" s="9"/>
       <x:c r="D362" s="9"/>
       <x:c r="E362" s="9"/>
+      <x:c r="F362" s="25"/>
+      <x:c r="G362" s="25"/>
     </x:row>
     <x:row r="363">
       <x:c r="A363" s="8"/>
@@ -2885,6 +3683,8 @@
       <x:c r="C363" s="9"/>
       <x:c r="D363" s="9"/>
       <x:c r="E363" s="9"/>
+      <x:c r="F363" s="29"/>
+      <x:c r="G363" s="29"/>
     </x:row>
     <x:row r="364">
       <x:c r="A364" s="8"/>
@@ -2892,6 +3692,8 @@
       <x:c r="C364" s="9"/>
       <x:c r="D364" s="9"/>
       <x:c r="E364" s="9"/>
+      <x:c r="F364" s="25"/>
+      <x:c r="G364" s="25"/>
     </x:row>
     <x:row r="365">
       <x:c r="A365" s="8"/>
@@ -2899,6 +3701,8 @@
       <x:c r="C365" s="9"/>
       <x:c r="D365" s="9"/>
       <x:c r="E365" s="9"/>
+      <x:c r="F365" s="29"/>
+      <x:c r="G365" s="29"/>
     </x:row>
     <x:row r="366">
       <x:c r="A366" s="8"/>
@@ -2906,6 +3710,8 @@
       <x:c r="C366" s="9"/>
       <x:c r="D366" s="9"/>
       <x:c r="E366" s="9"/>
+      <x:c r="F366" s="25"/>
+      <x:c r="G366" s="25"/>
     </x:row>
     <x:row r="367">
       <x:c r="A367" s="8"/>
@@ -2913,6 +3719,8 @@
       <x:c r="C367" s="9"/>
       <x:c r="D367" s="9"/>
       <x:c r="E367" s="9"/>
+      <x:c r="F367" s="29"/>
+      <x:c r="G367" s="29"/>
     </x:row>
     <x:row r="368">
       <x:c r="A368" s="8"/>
@@ -2920,6 +3728,8 @@
       <x:c r="C368" s="9"/>
       <x:c r="D368" s="9"/>
       <x:c r="E368" s="9"/>
+      <x:c r="F368" s="25"/>
+      <x:c r="G368" s="25"/>
     </x:row>
     <x:row r="369">
       <x:c r="A369" s="8"/>
@@ -2927,6 +3737,8 @@
       <x:c r="C369" s="9"/>
       <x:c r="D369" s="9"/>
       <x:c r="E369" s="9"/>
+      <x:c r="F369" s="29"/>
+      <x:c r="G369" s="29"/>
     </x:row>
     <x:row r="370">
       <x:c r="A370" s="8"/>
@@ -2934,6 +3746,8 @@
       <x:c r="C370" s="9"/>
       <x:c r="D370" s="9"/>
       <x:c r="E370" s="9"/>
+      <x:c r="F370" s="25"/>
+      <x:c r="G370" s="25"/>
     </x:row>
     <x:row r="371">
       <x:c r="A371" s="8"/>
@@ -2941,6 +3755,8 @@
       <x:c r="C371" s="9"/>
       <x:c r="D371" s="9"/>
       <x:c r="E371" s="9"/>
+      <x:c r="F371" s="29"/>
+      <x:c r="G371" s="29"/>
     </x:row>
     <x:row r="372">
       <x:c r="A372" s="8"/>
@@ -2948,6 +3764,8 @@
       <x:c r="C372" s="9"/>
       <x:c r="D372" s="9"/>
       <x:c r="E372" s="9"/>
+      <x:c r="F372" s="25"/>
+      <x:c r="G372" s="25"/>
     </x:row>
     <x:row r="373">
       <x:c r="A373" s="8"/>
@@ -2955,6 +3773,8 @@
       <x:c r="C373" s="9"/>
       <x:c r="D373" s="9"/>
       <x:c r="E373" s="9"/>
+      <x:c r="F373" s="29"/>
+      <x:c r="G373" s="29"/>
     </x:row>
     <x:row r="374">
       <x:c r="A374" s="8"/>
@@ -2962,6 +3782,8 @@
       <x:c r="C374" s="9"/>
       <x:c r="D374" s="9"/>
       <x:c r="E374" s="9"/>
+      <x:c r="F374" s="25"/>
+      <x:c r="G374" s="25"/>
     </x:row>
     <x:row r="375">
       <x:c r="A375" s="8"/>
@@ -2969,6 +3791,8 @@
       <x:c r="C375" s="9"/>
       <x:c r="D375" s="9"/>
       <x:c r="E375" s="9"/>
+      <x:c r="F375" s="29"/>
+      <x:c r="G375" s="29"/>
     </x:row>
     <x:row r="376">
       <x:c r="A376" s="8"/>
@@ -2976,6 +3800,8 @@
       <x:c r="C376" s="9"/>
       <x:c r="D376" s="9"/>
       <x:c r="E376" s="9"/>
+      <x:c r="F376" s="25"/>
+      <x:c r="G376" s="25"/>
     </x:row>
     <x:row r="377">
       <x:c r="A377" s="8"/>
@@ -2983,6 +3809,8 @@
       <x:c r="C377" s="9"/>
       <x:c r="D377" s="9"/>
       <x:c r="E377" s="9"/>
+      <x:c r="F377" s="29"/>
+      <x:c r="G377" s="29"/>
     </x:row>
     <x:row r="378">
       <x:c r="A378" s="8"/>
@@ -2990,6 +3818,8 @@
       <x:c r="C378" s="9"/>
       <x:c r="D378" s="9"/>
       <x:c r="E378" s="9"/>
+      <x:c r="F378" s="25"/>
+      <x:c r="G378" s="25"/>
     </x:row>
     <x:row r="379">
       <x:c r="A379" s="8"/>
@@ -2997,6 +3827,8 @@
       <x:c r="C379" s="9"/>
       <x:c r="D379" s="9"/>
       <x:c r="E379" s="9"/>
+      <x:c r="F379" s="29"/>
+      <x:c r="G379" s="29"/>
     </x:row>
     <x:row r="380">
       <x:c r="A380" s="8"/>
@@ -3004,6 +3836,8 @@
       <x:c r="C380" s="9"/>
       <x:c r="D380" s="9"/>
       <x:c r="E380" s="9"/>
+      <x:c r="F380" s="25"/>
+      <x:c r="G380" s="25"/>
     </x:row>
     <x:row r="381">
       <x:c r="A381" s="8"/>
@@ -3011,6 +3845,8 @@
       <x:c r="C381" s="9"/>
       <x:c r="D381" s="9"/>
       <x:c r="E381" s="9"/>
+      <x:c r="F381" s="29"/>
+      <x:c r="G381" s="29"/>
     </x:row>
     <x:row r="382">
       <x:c r="A382" s="8"/>
@@ -3018,6 +3854,8 @@
       <x:c r="C382" s="9"/>
       <x:c r="D382" s="9"/>
       <x:c r="E382" s="9"/>
+      <x:c r="F382" s="25"/>
+      <x:c r="G382" s="25"/>
     </x:row>
     <x:row r="383">
       <x:c r="A383" s="8"/>
@@ -3025,6 +3863,8 @@
       <x:c r="C383" s="9"/>
       <x:c r="D383" s="9"/>
       <x:c r="E383" s="9"/>
+      <x:c r="F383" s="29"/>
+      <x:c r="G383" s="29"/>
     </x:row>
     <x:row r="384">
       <x:c r="A384" s="8"/>
@@ -3032,6 +3872,8 @@
       <x:c r="C384" s="9"/>
       <x:c r="D384" s="9"/>
       <x:c r="E384" s="9"/>
+      <x:c r="F384" s="25"/>
+      <x:c r="G384" s="25"/>
     </x:row>
     <x:row r="385">
       <x:c r="A385" s="8"/>
@@ -3039,6 +3881,8 @@
       <x:c r="C385" s="9"/>
       <x:c r="D385" s="9"/>
       <x:c r="E385" s="9"/>
+      <x:c r="F385" s="29"/>
+      <x:c r="G385" s="29"/>
     </x:row>
     <x:row r="386">
       <x:c r="A386" s="8"/>
@@ -3046,6 +3890,8 @@
       <x:c r="C386" s="9"/>
       <x:c r="D386" s="9"/>
       <x:c r="E386" s="9"/>
+      <x:c r="F386" s="25"/>
+      <x:c r="G386" s="25"/>
     </x:row>
     <x:row r="387">
       <x:c r="A387" s="8"/>
@@ -3053,6 +3899,8 @@
       <x:c r="C387" s="9"/>
       <x:c r="D387" s="9"/>
       <x:c r="E387" s="9"/>
+      <x:c r="F387" s="29"/>
+      <x:c r="G387" s="29"/>
     </x:row>
     <x:row r="388">
       <x:c r="A388" s="8"/>
@@ -3060,6 +3908,8 @@
       <x:c r="C388" s="9"/>
       <x:c r="D388" s="9"/>
       <x:c r="E388" s="9"/>
+      <x:c r="F388" s="25"/>
+      <x:c r="G388" s="25"/>
     </x:row>
     <x:row r="389">
       <x:c r="A389" s="8"/>
@@ -3067,6 +3917,8 @@
       <x:c r="C389" s="9"/>
       <x:c r="D389" s="9"/>
       <x:c r="E389" s="9"/>
+      <x:c r="F389" s="29"/>
+      <x:c r="G389" s="29"/>
     </x:row>
     <x:row r="390">
       <x:c r="A390" s="8"/>
@@ -3074,6 +3926,8 @@
       <x:c r="C390" s="9"/>
       <x:c r="D390" s="9"/>
       <x:c r="E390" s="9"/>
+      <x:c r="F390" s="25"/>
+      <x:c r="G390" s="25"/>
     </x:row>
     <x:row r="391">
       <x:c r="A391" s="8"/>
@@ -3081,6 +3935,8 @@
       <x:c r="C391" s="9"/>
       <x:c r="D391" s="9"/>
       <x:c r="E391" s="9"/>
+      <x:c r="F391" s="29"/>
+      <x:c r="G391" s="29"/>
     </x:row>
     <x:row r="392">
       <x:c r="A392" s="8"/>
@@ -3088,6 +3944,8 @@
       <x:c r="C392" s="9"/>
       <x:c r="D392" s="9"/>
       <x:c r="E392" s="9"/>
+      <x:c r="F392" s="25"/>
+      <x:c r="G392" s="25"/>
     </x:row>
     <x:row r="393">
       <x:c r="A393" s="8"/>
@@ -3095,6 +3953,8 @@
       <x:c r="C393" s="9"/>
       <x:c r="D393" s="9"/>
       <x:c r="E393" s="9"/>
+      <x:c r="F393" s="29"/>
+      <x:c r="G393" s="29"/>
     </x:row>
     <x:row r="394">
       <x:c r="A394" s="8"/>
@@ -3102,6 +3962,8 @@
       <x:c r="C394" s="9"/>
       <x:c r="D394" s="9"/>
       <x:c r="E394" s="9"/>
+      <x:c r="F394" s="25"/>
+      <x:c r="G394" s="25"/>
     </x:row>
     <x:row r="395">
       <x:c r="A395" s="8"/>
@@ -3109,6 +3971,8 @@
       <x:c r="C395" s="9"/>
       <x:c r="D395" s="9"/>
       <x:c r="E395" s="9"/>
+      <x:c r="F395" s="29"/>
+      <x:c r="G395" s="29"/>
     </x:row>
     <x:row r="396">
       <x:c r="A396" s="8"/>
@@ -3116,6 +3980,8 @@
       <x:c r="C396" s="9"/>
       <x:c r="D396" s="9"/>
       <x:c r="E396" s="9"/>
+      <x:c r="F396" s="25"/>
+      <x:c r="G396" s="25"/>
     </x:row>
     <x:row r="397">
       <x:c r="A397" s="8"/>
@@ -3123,6 +3989,8 @@
       <x:c r="C397" s="9"/>
       <x:c r="D397" s="9"/>
       <x:c r="E397" s="9"/>
+      <x:c r="F397" s="29"/>
+      <x:c r="G397" s="29"/>
     </x:row>
     <x:row r="398">
       <x:c r="A398" s="8"/>
@@ -3130,6 +3998,8 @@
       <x:c r="C398" s="9"/>
       <x:c r="D398" s="9"/>
       <x:c r="E398" s="9"/>
+      <x:c r="F398" s="25"/>
+      <x:c r="G398" s="25"/>
     </x:row>
     <x:row r="399">
       <x:c r="A399" s="8"/>
@@ -3137,6 +4007,8 @@
       <x:c r="C399" s="9"/>
       <x:c r="D399" s="9"/>
       <x:c r="E399" s="9"/>
+      <x:c r="F399" s="29"/>
+      <x:c r="G399" s="29"/>
     </x:row>
     <x:row r="400">
       <x:c r="A400" s="8"/>
@@ -3144,6 +4016,8 @@
       <x:c r="C400" s="9"/>
       <x:c r="D400" s="9"/>
       <x:c r="E400" s="9"/>
+      <x:c r="F400" s="25"/>
+      <x:c r="G400" s="25"/>
     </x:row>
     <x:row r="401">
       <x:c r="A401" s="8"/>
@@ -3151,6 +4025,8 @@
       <x:c r="C401" s="9"/>
       <x:c r="D401" s="9"/>
       <x:c r="E401" s="9"/>
+      <x:c r="F401" s="29"/>
+      <x:c r="G401" s="29"/>
     </x:row>
     <x:row r="402">
       <x:c r="A402" s="8"/>
@@ -3158,6 +4034,8 @@
       <x:c r="C402" s="9"/>
       <x:c r="D402" s="9"/>
       <x:c r="E402" s="9"/>
+      <x:c r="F402" s="25"/>
+      <x:c r="G402" s="25"/>
     </x:row>
     <x:row r="403">
       <x:c r="A403" s="8"/>
@@ -3165,6 +4043,8 @@
       <x:c r="C403" s="9"/>
       <x:c r="D403" s="9"/>
       <x:c r="E403" s="9"/>
+      <x:c r="F403" s="29"/>
+      <x:c r="G403" s="29"/>
     </x:row>
     <x:row r="404">
       <x:c r="A404" s="8"/>
@@ -3172,6 +4052,8 @@
       <x:c r="C404" s="9"/>
       <x:c r="D404" s="9"/>
       <x:c r="E404" s="9"/>
+      <x:c r="F404" s="25"/>
+      <x:c r="G404" s="25"/>
     </x:row>
     <x:row r="405">
       <x:c r="A405" s="8"/>
@@ -3179,6 +4061,8 @@
       <x:c r="C405" s="9"/>
       <x:c r="D405" s="9"/>
       <x:c r="E405" s="9"/>
+      <x:c r="F405" s="29"/>
+      <x:c r="G405" s="29"/>
     </x:row>
     <x:row r="406">
       <x:c r="A406" s="8"/>
@@ -3186,6 +4070,8 @@
       <x:c r="C406" s="9"/>
       <x:c r="D406" s="9"/>
       <x:c r="E406" s="9"/>
+      <x:c r="F406" s="25"/>
+      <x:c r="G406" s="25"/>
     </x:row>
     <x:row r="407">
       <x:c r="A407" s="8"/>
@@ -3193,6 +4079,8 @@
       <x:c r="C407" s="9"/>
       <x:c r="D407" s="9"/>
       <x:c r="E407" s="9"/>
+      <x:c r="F407" s="29"/>
+      <x:c r="G407" s="29"/>
     </x:row>
     <x:row r="408">
       <x:c r="A408" s="8"/>
@@ -3200,6 +4088,8 @@
       <x:c r="C408" s="9"/>
       <x:c r="D408" s="9"/>
       <x:c r="E408" s="9"/>
+      <x:c r="F408" s="25"/>
+      <x:c r="G408" s="25"/>
     </x:row>
     <x:row r="409">
       <x:c r="A409" s="8"/>
@@ -3207,6 +4097,8 @@
       <x:c r="C409" s="9"/>
       <x:c r="D409" s="9"/>
       <x:c r="E409" s="9"/>
+      <x:c r="F409" s="29"/>
+      <x:c r="G409" s="29"/>
     </x:row>
     <x:row r="410">
       <x:c r="A410" s="8"/>
@@ -3214,6 +4106,8 @@
       <x:c r="C410" s="9"/>
       <x:c r="D410" s="9"/>
       <x:c r="E410" s="9"/>
+      <x:c r="F410" s="25"/>
+      <x:c r="G410" s="25"/>
     </x:row>
     <x:row r="411">
       <x:c r="A411" s="8"/>
@@ -3221,6 +4115,8 @@
       <x:c r="C411" s="9"/>
       <x:c r="D411" s="9"/>
       <x:c r="E411" s="9"/>
+      <x:c r="F411" s="29"/>
+      <x:c r="G411" s="29"/>
     </x:row>
     <x:row r="412">
       <x:c r="A412" s="8"/>
@@ -3228,6 +4124,8 @@
       <x:c r="C412" s="9"/>
       <x:c r="D412" s="9"/>
       <x:c r="E412" s="9"/>
+      <x:c r="F412" s="25"/>
+      <x:c r="G412" s="25"/>
     </x:row>
     <x:row r="413">
       <x:c r="A413" s="8"/>
@@ -3235,6 +4133,8 @@
       <x:c r="C413" s="9"/>
       <x:c r="D413" s="9"/>
       <x:c r="E413" s="9"/>
+      <x:c r="F413" s="29"/>
+      <x:c r="G413" s="29"/>
     </x:row>
     <x:row r="414">
       <x:c r="A414" s="8"/>
@@ -3242,6 +4142,8 @@
       <x:c r="C414" s="9"/>
       <x:c r="D414" s="9"/>
       <x:c r="E414" s="9"/>
+      <x:c r="F414" s="25"/>
+      <x:c r="G414" s="25"/>
     </x:row>
     <x:row r="415">
       <x:c r="A415" s="8"/>
@@ -3249,6 +4151,8 @@
       <x:c r="C415" s="9"/>
       <x:c r="D415" s="9"/>
       <x:c r="E415" s="9"/>
+      <x:c r="F415" s="29"/>
+      <x:c r="G415" s="29"/>
     </x:row>
     <x:row r="416">
       <x:c r="A416" s="8"/>
@@ -3256,6 +4160,8 @@
       <x:c r="C416" s="9"/>
       <x:c r="D416" s="9"/>
       <x:c r="E416" s="9"/>
+      <x:c r="F416" s="25"/>
+      <x:c r="G416" s="25"/>
     </x:row>
     <x:row r="417">
       <x:c r="A417" s="8"/>
@@ -3263,6 +4169,8 @@
       <x:c r="C417" s="9"/>
       <x:c r="D417" s="9"/>
       <x:c r="E417" s="9"/>
+      <x:c r="F417" s="29"/>
+      <x:c r="G417" s="29"/>
     </x:row>
     <x:row r="418">
       <x:c r="A418" s="8"/>
@@ -3270,6 +4178,8 @@
       <x:c r="C418" s="9"/>
       <x:c r="D418" s="9"/>
       <x:c r="E418" s="9"/>
+      <x:c r="F418" s="25"/>
+      <x:c r="G418" s="25"/>
     </x:row>
     <x:row r="419">
       <x:c r="A419" s="8"/>
@@ -3277,6 +4187,8 @@
       <x:c r="C419" s="9"/>
       <x:c r="D419" s="9"/>
       <x:c r="E419" s="9"/>
+      <x:c r="F419" s="29"/>
+      <x:c r="G419" s="29"/>
     </x:row>
     <x:row r="420">
       <x:c r="A420" s="8"/>
@@ -3284,6 +4196,8 @@
       <x:c r="C420" s="9"/>
       <x:c r="D420" s="9"/>
       <x:c r="E420" s="9"/>
+      <x:c r="F420" s="25"/>
+      <x:c r="G420" s="25"/>
     </x:row>
     <x:row r="421">
       <x:c r="A421" s="8"/>
@@ -3291,6 +4205,8 @@
       <x:c r="C421" s="9"/>
       <x:c r="D421" s="9"/>
       <x:c r="E421" s="9"/>
+      <x:c r="F421" s="29"/>
+      <x:c r="G421" s="29"/>
     </x:row>
     <x:row r="422">
       <x:c r="A422" s="8"/>
@@ -3298,6 +4214,8 @@
       <x:c r="C422" s="9"/>
       <x:c r="D422" s="9"/>
       <x:c r="E422" s="9"/>
+      <x:c r="F422" s="25"/>
+      <x:c r="G422" s="25"/>
     </x:row>
     <x:row r="423">
       <x:c r="A423" s="8"/>
@@ -3305,6 +4223,8 @@
       <x:c r="C423" s="9"/>
       <x:c r="D423" s="9"/>
       <x:c r="E423" s="9"/>
+      <x:c r="F423" s="29"/>
+      <x:c r="G423" s="29"/>
     </x:row>
     <x:row r="424">
       <x:c r="A424" s="8"/>
@@ -3312,6 +4232,8 @@
       <x:c r="C424" s="9"/>
       <x:c r="D424" s="9"/>
       <x:c r="E424" s="9"/>
+      <x:c r="F424" s="25"/>
+      <x:c r="G424" s="25"/>
     </x:row>
     <x:row r="425">
       <x:c r="A425" s="8"/>
@@ -3319,6 +4241,8 @@
       <x:c r="C425" s="9"/>
       <x:c r="D425" s="9"/>
       <x:c r="E425" s="9"/>
+      <x:c r="F425" s="29"/>
+      <x:c r="G425" s="29"/>
     </x:row>
     <x:row r="426">
       <x:c r="A426" s="8"/>
@@ -3326,6 +4250,8 @@
       <x:c r="C426" s="9"/>
       <x:c r="D426" s="9"/>
       <x:c r="E426" s="9"/>
+      <x:c r="F426" s="25"/>
+      <x:c r="G426" s="25"/>
     </x:row>
     <x:row r="427">
       <x:c r="A427" s="8"/>
@@ -3333,6 +4259,8 @@
       <x:c r="C427" s="9"/>
       <x:c r="D427" s="9"/>
       <x:c r="E427" s="9"/>
+      <x:c r="F427" s="29"/>
+      <x:c r="G427" s="29"/>
     </x:row>
     <x:row r="428">
       <x:c r="A428" s="8"/>
@@ -3340,6 +4268,8 @@
       <x:c r="C428" s="9"/>
       <x:c r="D428" s="9"/>
       <x:c r="E428" s="9"/>
+      <x:c r="F428" s="25"/>
+      <x:c r="G428" s="25"/>
     </x:row>
     <x:row r="429">
       <x:c r="A429" s="8"/>
@@ -3347,6 +4277,8 @@
       <x:c r="C429" s="9"/>
       <x:c r="D429" s="9"/>
       <x:c r="E429" s="9"/>
+      <x:c r="F429" s="29"/>
+      <x:c r="G429" s="29"/>
     </x:row>
     <x:row r="430">
       <x:c r="A430" s="8"/>
@@ -3354,6 +4286,8 @@
       <x:c r="C430" s="9"/>
       <x:c r="D430" s="9"/>
       <x:c r="E430" s="9"/>
+      <x:c r="F430" s="25"/>
+      <x:c r="G430" s="25"/>
     </x:row>
     <x:row r="431">
       <x:c r="A431" s="8"/>
@@ -3361,6 +4295,8 @@
       <x:c r="C431" s="9"/>
       <x:c r="D431" s="9"/>
       <x:c r="E431" s="9"/>
+      <x:c r="F431" s="29"/>
+      <x:c r="G431" s="29"/>
     </x:row>
     <x:row r="432">
       <x:c r="A432" s="8"/>
@@ -3368,6 +4304,8 @@
       <x:c r="C432" s="9"/>
       <x:c r="D432" s="9"/>
       <x:c r="E432" s="9"/>
+      <x:c r="F432" s="25"/>
+      <x:c r="G432" s="25"/>
     </x:row>
     <x:row r="433">
       <x:c r="A433" s="8"/>
@@ -3375,6 +4313,8 @@
       <x:c r="C433" s="9"/>
       <x:c r="D433" s="9"/>
       <x:c r="E433" s="9"/>
+      <x:c r="F433" s="29"/>
+      <x:c r="G433" s="29"/>
     </x:row>
     <x:row r="434">
       <x:c r="A434" s="8"/>
@@ -3382,6 +4322,8 @@
       <x:c r="C434" s="9"/>
       <x:c r="D434" s="9"/>
       <x:c r="E434" s="9"/>
+      <x:c r="F434" s="25"/>
+      <x:c r="G434" s="25"/>
     </x:row>
     <x:row r="435">
       <x:c r="A435" s="8"/>
@@ -3389,6 +4331,8 @@
       <x:c r="C435" s="9"/>
       <x:c r="D435" s="9"/>
       <x:c r="E435" s="9"/>
+      <x:c r="F435" s="29"/>
+      <x:c r="G435" s="29"/>
     </x:row>
     <x:row r="436">
       <x:c r="A436" s="8"/>
@@ -3396,6 +4340,8 @@
       <x:c r="C436" s="9"/>
       <x:c r="D436" s="9"/>
       <x:c r="E436" s="9"/>
+      <x:c r="F436" s="25"/>
+      <x:c r="G436" s="25"/>
     </x:row>
     <x:row r="437">
       <x:c r="A437" s="8"/>
@@ -3403,6 +4349,8 @@
       <x:c r="C437" s="9"/>
       <x:c r="D437" s="9"/>
       <x:c r="E437" s="9"/>
+      <x:c r="F437" s="29"/>
+      <x:c r="G437" s="29"/>
     </x:row>
     <x:row r="438">
       <x:c r="A438" s="8"/>
@@ -3410,6 +4358,8 @@
       <x:c r="C438" s="9"/>
       <x:c r="D438" s="9"/>
       <x:c r="E438" s="9"/>
+      <x:c r="F438" s="25"/>
+      <x:c r="G438" s="25"/>
     </x:row>
     <x:row r="439">
       <x:c r="A439" s="8"/>
@@ -3417,6 +4367,8 @@
       <x:c r="C439" s="9"/>
       <x:c r="D439" s="9"/>
       <x:c r="E439" s="9"/>
+      <x:c r="F439" s="29"/>
+      <x:c r="G439" s="29"/>
     </x:row>
     <x:row r="440">
       <x:c r="A440" s="8"/>
@@ -3424,6 +4376,8 @@
       <x:c r="C440" s="9"/>
       <x:c r="D440" s="9"/>
       <x:c r="E440" s="9"/>
+      <x:c r="F440" s="25"/>
+      <x:c r="G440" s="25"/>
     </x:row>
     <x:row r="441">
       <x:c r="A441" s="8"/>
@@ -3431,6 +4385,8 @@
       <x:c r="C441" s="9"/>
       <x:c r="D441" s="9"/>
       <x:c r="E441" s="9"/>
+      <x:c r="F441" s="29"/>
+      <x:c r="G441" s="29"/>
     </x:row>
     <x:row r="442">
       <x:c r="A442" s="8"/>
@@ -3438,6 +4394,8 @@
       <x:c r="C442" s="9"/>
       <x:c r="D442" s="9"/>
       <x:c r="E442" s="9"/>
+      <x:c r="F442" s="25"/>
+      <x:c r="G442" s="25"/>
     </x:row>
     <x:row r="443">
       <x:c r="A443" s="8"/>
@@ -3445,6 +4403,8 @@
       <x:c r="C443" s="9"/>
       <x:c r="D443" s="9"/>
       <x:c r="E443" s="9"/>
+      <x:c r="F443" s="29"/>
+      <x:c r="G443" s="29"/>
     </x:row>
     <x:row r="444">
       <x:c r="A444" s="8"/>
@@ -3452,6 +4412,8 @@
       <x:c r="C444" s="9"/>
       <x:c r="D444" s="9"/>
       <x:c r="E444" s="9"/>
+      <x:c r="F444" s="25"/>
+      <x:c r="G444" s="25"/>
     </x:row>
     <x:row r="445">
       <x:c r="A445" s="8"/>
@@ -3459,6 +4421,8 @@
       <x:c r="C445" s="9"/>
       <x:c r="D445" s="9"/>
       <x:c r="E445" s="9"/>
+      <x:c r="F445" s="29"/>
+      <x:c r="G445" s="29"/>
     </x:row>
     <x:row r="446">
       <x:c r="A446" s="8"/>
@@ -3466,6 +4430,8 @@
       <x:c r="C446" s="9"/>
       <x:c r="D446" s="9"/>
       <x:c r="E446" s="9"/>
+      <x:c r="F446" s="25"/>
+      <x:c r="G446" s="25"/>
     </x:row>
     <x:row r="447">
       <x:c r="A447" s="8"/>
@@ -3473,6 +4439,8 @@
       <x:c r="C447" s="9"/>
       <x:c r="D447" s="9"/>
       <x:c r="E447" s="9"/>
+      <x:c r="F447" s="29"/>
+      <x:c r="G447" s="29"/>
     </x:row>
     <x:row r="448">
       <x:c r="A448" s="8"/>
@@ -3480,6 +4448,8 @@
       <x:c r="C448" s="9"/>
       <x:c r="D448" s="9"/>
       <x:c r="E448" s="9"/>
+      <x:c r="F448" s="25"/>
+      <x:c r="G448" s="25"/>
     </x:row>
     <x:row r="449">
       <x:c r="A449" s="8"/>
@@ -3487,6 +4457,8 @@
       <x:c r="C449" s="9"/>
       <x:c r="D449" s="9"/>
       <x:c r="E449" s="9"/>
+      <x:c r="F449" s="29"/>
+      <x:c r="G449" s="29"/>
     </x:row>
     <x:row r="450">
       <x:c r="A450" s="8"/>
@@ -3494,6 +4466,8 @@
       <x:c r="C450" s="9"/>
       <x:c r="D450" s="9"/>
       <x:c r="E450" s="9"/>
+      <x:c r="F450" s="25"/>
+      <x:c r="G450" s="25"/>
     </x:row>
     <x:row r="451">
       <x:c r="A451" s="8"/>
@@ -3501,6 +4475,8 @@
       <x:c r="C451" s="9"/>
       <x:c r="D451" s="9"/>
       <x:c r="E451" s="9"/>
+      <x:c r="F451" s="29"/>
+      <x:c r="G451" s="29"/>
     </x:row>
     <x:row r="452">
       <x:c r="A452" s="8"/>
@@ -3508,6 +4484,8 @@
       <x:c r="C452" s="9"/>
       <x:c r="D452" s="9"/>
       <x:c r="E452" s="9"/>
+      <x:c r="F452" s="25"/>
+      <x:c r="G452" s="25"/>
     </x:row>
     <x:row r="453">
       <x:c r="A453" s="8"/>
@@ -3515,6 +4493,8 @@
       <x:c r="C453" s="9"/>
       <x:c r="D453" s="9"/>
       <x:c r="E453" s="9"/>
+      <x:c r="F453" s="29"/>
+      <x:c r="G453" s="29"/>
     </x:row>
     <x:row r="454">
       <x:c r="A454" s="8"/>
@@ -3522,6 +4502,8 @@
       <x:c r="C454" s="9"/>
       <x:c r="D454" s="9"/>
       <x:c r="E454" s="9"/>
+      <x:c r="F454" s="25"/>
+      <x:c r="G454" s="25"/>
     </x:row>
     <x:row r="455">
       <x:c r="A455" s="8"/>
@@ -3529,6 +4511,8 @@
       <x:c r="C455" s="9"/>
       <x:c r="D455" s="9"/>
       <x:c r="E455" s="9"/>
+      <x:c r="F455" s="29"/>
+      <x:c r="G455" s="29"/>
     </x:row>
     <x:row r="456">
       <x:c r="A456" s="8"/>
@@ -3536,6 +4520,8 @@
       <x:c r="C456" s="9"/>
       <x:c r="D456" s="9"/>
       <x:c r="E456" s="9"/>
+      <x:c r="F456" s="25"/>
+      <x:c r="G456" s="25"/>
     </x:row>
     <x:row r="457">
       <x:c r="A457" s="8"/>
@@ -3543,6 +4529,8 @@
       <x:c r="C457" s="9"/>
       <x:c r="D457" s="9"/>
       <x:c r="E457" s="9"/>
+      <x:c r="F457" s="29"/>
+      <x:c r="G457" s="29"/>
     </x:row>
     <x:row r="458">
       <x:c r="A458" s="8"/>
@@ -3550,6 +4538,8 @@
       <x:c r="C458" s="9"/>
       <x:c r="D458" s="9"/>
       <x:c r="E458" s="9"/>
+      <x:c r="F458" s="25"/>
+      <x:c r="G458" s="25"/>
     </x:row>
     <x:row r="459">
       <x:c r="A459" s="8"/>
@@ -3557,6 +4547,8 @@
       <x:c r="C459" s="9"/>
       <x:c r="D459" s="9"/>
       <x:c r="E459" s="9"/>
+      <x:c r="F459" s="29"/>
+      <x:c r="G459" s="29"/>
     </x:row>
     <x:row r="460">
       <x:c r="A460" s="8"/>
@@ -3564,6 +4556,8 @@
       <x:c r="C460" s="9"/>
       <x:c r="D460" s="9"/>
       <x:c r="E460" s="9"/>
+      <x:c r="F460" s="25"/>
+      <x:c r="G460" s="25"/>
     </x:row>
     <x:row r="461">
       <x:c r="A461" s="8"/>
@@ -3571,6 +4565,8 @@
       <x:c r="C461" s="9"/>
       <x:c r="D461" s="9"/>
       <x:c r="E461" s="9"/>
+      <x:c r="F461" s="29"/>
+      <x:c r="G461" s="29"/>
     </x:row>
     <x:row r="462">
       <x:c r="A462" s="8"/>
@@ -3578,6 +4574,8 @@
       <x:c r="C462" s="9"/>
       <x:c r="D462" s="9"/>
       <x:c r="E462" s="9"/>
+      <x:c r="F462" s="25"/>
+      <x:c r="G462" s="25"/>
     </x:row>
     <x:row r="463">
       <x:c r="A463" s="8"/>
@@ -3585,6 +4583,8 @@
       <x:c r="C463" s="9"/>
       <x:c r="D463" s="9"/>
       <x:c r="E463" s="9"/>
+      <x:c r="F463" s="29"/>
+      <x:c r="G463" s="29"/>
     </x:row>
     <x:row r="464">
       <x:c r="A464" s="8"/>
@@ -3592,6 +4592,8 @@
       <x:c r="C464" s="9"/>
       <x:c r="D464" s="9"/>
       <x:c r="E464" s="9"/>
+      <x:c r="F464" s="25"/>
+      <x:c r="G464" s="25"/>
     </x:row>
     <x:row r="465">
       <x:c r="A465" s="8"/>
@@ -3599,6 +4601,8 @@
       <x:c r="C465" s="9"/>
       <x:c r="D465" s="9"/>
       <x:c r="E465" s="9"/>
+      <x:c r="F465" s="29"/>
+      <x:c r="G465" s="29"/>
     </x:row>
     <x:row r="466">
       <x:c r="A466" s="8"/>
@@ -3606,6 +4610,8 @@
       <x:c r="C466" s="9"/>
       <x:c r="D466" s="9"/>
       <x:c r="E466" s="9"/>
+      <x:c r="F466" s="25"/>
+      <x:c r="G466" s="25"/>
     </x:row>
     <x:row r="467">
       <x:c r="A467" s="8"/>
@@ -3613,6 +4619,8 @@
       <x:c r="C467" s="9"/>
       <x:c r="D467" s="9"/>
       <x:c r="E467" s="9"/>
+      <x:c r="F467" s="29"/>
+      <x:c r="G467" s="29"/>
     </x:row>
     <x:row r="468">
       <x:c r="A468" s="8"/>
@@ -3620,6 +4628,8 @@
       <x:c r="C468" s="9"/>
       <x:c r="D468" s="9"/>
       <x:c r="E468" s="9"/>
+      <x:c r="F468" s="25"/>
+      <x:c r="G468" s="25"/>
     </x:row>
     <x:row r="469">
       <x:c r="A469" s="8"/>
@@ -3627,6 +4637,8 @@
       <x:c r="C469" s="9"/>
       <x:c r="D469" s="9"/>
       <x:c r="E469" s="9"/>
+      <x:c r="F469" s="29"/>
+      <x:c r="G469" s="29"/>
     </x:row>
     <x:row r="470">
       <x:c r="A470" s="8"/>
@@ -3634,6 +4646,8 @@
       <x:c r="C470" s="9"/>
       <x:c r="D470" s="9"/>
       <x:c r="E470" s="9"/>
+      <x:c r="F470" s="25"/>
+      <x:c r="G470" s="25"/>
     </x:row>
     <x:row r="471">
       <x:c r="A471" s="8"/>
@@ -3641,6 +4655,8 @@
       <x:c r="C471" s="9"/>
       <x:c r="D471" s="9"/>
       <x:c r="E471" s="9"/>
+      <x:c r="F471" s="29"/>
+      <x:c r="G471" s="29"/>
     </x:row>
     <x:row r="472">
       <x:c r="A472" s="8"/>
@@ -3648,6 +4664,8 @@
       <x:c r="C472" s="9"/>
       <x:c r="D472" s="9"/>
       <x:c r="E472" s="9"/>
+      <x:c r="F472" s="25"/>
+      <x:c r="G472" s="25"/>
     </x:row>
     <x:row r="473">
       <x:c r="A473" s="8"/>
@@ -3655,6 +4673,8 @@
       <x:c r="C473" s="9"/>
       <x:c r="D473" s="9"/>
       <x:c r="E473" s="9"/>
+      <x:c r="F473" s="29"/>
+      <x:c r="G473" s="29"/>
     </x:row>
     <x:row r="474">
       <x:c r="A474" s="8"/>
@@ -3662,6 +4682,8 @@
       <x:c r="C474" s="9"/>
       <x:c r="D474" s="9"/>
       <x:c r="E474" s="9"/>
+      <x:c r="F474" s="25"/>
+      <x:c r="G474" s="25"/>
     </x:row>
     <x:row r="475">
       <x:c r="A475" s="8"/>
@@ -3669,6 +4691,8 @@
       <x:c r="C475" s="9"/>
       <x:c r="D475" s="9"/>
       <x:c r="E475" s="9"/>
+      <x:c r="F475" s="29"/>
+      <x:c r="G475" s="29"/>
     </x:row>
     <x:row r="476">
       <x:c r="A476" s="8"/>
@@ -3676,6 +4700,8 @@
       <x:c r="C476" s="9"/>
       <x:c r="D476" s="9"/>
       <x:c r="E476" s="9"/>
+      <x:c r="F476" s="25"/>
+      <x:c r="G476" s="25"/>
     </x:row>
     <x:row r="477">
       <x:c r="A477" s="8"/>
@@ -3683,6 +4709,8 @@
       <x:c r="C477" s="9"/>
       <x:c r="D477" s="9"/>
       <x:c r="E477" s="9"/>
+      <x:c r="F477" s="29"/>
+      <x:c r="G477" s="29"/>
     </x:row>
     <x:row r="478">
       <x:c r="A478" s="8"/>
@@ -3690,6 +4718,8 @@
       <x:c r="C478" s="9"/>
       <x:c r="D478" s="9"/>
       <x:c r="E478" s="9"/>
+      <x:c r="F478" s="25"/>
+      <x:c r="G478" s="25"/>
     </x:row>
     <x:row r="479">
       <x:c r="A479" s="8"/>
@@ -3697,6 +4727,8 @@
       <x:c r="C479" s="9"/>
       <x:c r="D479" s="9"/>
       <x:c r="E479" s="9"/>
+      <x:c r="F479" s="29"/>
+      <x:c r="G479" s="29"/>
     </x:row>
     <x:row r="480">
       <x:c r="A480" s="8"/>
@@ -3704,6 +4736,8 @@
       <x:c r="C480" s="9"/>
       <x:c r="D480" s="9"/>
       <x:c r="E480" s="9"/>
+      <x:c r="F480" s="25"/>
+      <x:c r="G480" s="25"/>
     </x:row>
     <x:row r="481">
       <x:c r="A481" s="8"/>
@@ -3711,6 +4745,8 @@
       <x:c r="C481" s="9"/>
       <x:c r="D481" s="9"/>
       <x:c r="E481" s="9"/>
+      <x:c r="F481" s="29"/>
+      <x:c r="G481" s="29"/>
     </x:row>
     <x:row r="482">
       <x:c r="A482" s="8"/>
@@ -3718,6 +4754,8 @@
       <x:c r="C482" s="9"/>
       <x:c r="D482" s="9"/>
       <x:c r="E482" s="9"/>
+      <x:c r="F482" s="25"/>
+      <x:c r="G482" s="25"/>
     </x:row>
     <x:row r="483">
       <x:c r="A483" s="8"/>
@@ -3725,6 +4763,8 @@
       <x:c r="C483" s="9"/>
       <x:c r="D483" s="9"/>
       <x:c r="E483" s="9"/>
+      <x:c r="F483" s="29"/>
+      <x:c r="G483" s="29"/>
     </x:row>
     <x:row r="484">
       <x:c r="A484" s="8"/>
@@ -3732,6 +4772,8 @@
       <x:c r="C484" s="9"/>
       <x:c r="D484" s="9"/>
       <x:c r="E484" s="9"/>
+      <x:c r="F484" s="25"/>
+      <x:c r="G484" s="25"/>
     </x:row>
     <x:row r="485">
       <x:c r="A485" s="8"/>
@@ -3739,6 +4781,8 @@
       <x:c r="C485" s="9"/>
       <x:c r="D485" s="9"/>
       <x:c r="E485" s="9"/>
+      <x:c r="F485" s="29"/>
+      <x:c r="G485" s="29"/>
     </x:row>
     <x:row r="486">
       <x:c r="A486" s="8"/>
@@ -3746,6 +4790,8 @@
       <x:c r="C486" s="9"/>
       <x:c r="D486" s="9"/>
       <x:c r="E486" s="9"/>
+      <x:c r="F486" s="25"/>
+      <x:c r="G486" s="25"/>
     </x:row>
     <x:row r="487">
       <x:c r="A487" s="8"/>
@@ -3753,6 +4799,8 @@
       <x:c r="C487" s="9"/>
       <x:c r="D487" s="9"/>
       <x:c r="E487" s="9"/>
+      <x:c r="F487" s="29"/>
+      <x:c r="G487" s="29"/>
     </x:row>
     <x:row r="488">
       <x:c r="A488" s="8"/>
@@ -3760,6 +4808,8 @@
       <x:c r="C488" s="9"/>
       <x:c r="D488" s="9"/>
       <x:c r="E488" s="9"/>
+      <x:c r="F488" s="25"/>
+      <x:c r="G488" s="25"/>
     </x:row>
     <x:row r="489">
       <x:c r="A489" s="8"/>
@@ -3767,6 +4817,8 @@
       <x:c r="C489" s="9"/>
       <x:c r="D489" s="9"/>
       <x:c r="E489" s="9"/>
+      <x:c r="F489" s="29"/>
+      <x:c r="G489" s="29"/>
     </x:row>
     <x:row r="490">
       <x:c r="A490" s="8"/>
@@ -3774,6 +4826,8 @@
       <x:c r="C490" s="9"/>
       <x:c r="D490" s="9"/>
       <x:c r="E490" s="9"/>
+      <x:c r="F490" s="25"/>
+      <x:c r="G490" s="25"/>
     </x:row>
     <x:row r="491">
       <x:c r="A491" s="8"/>
@@ -3781,6 +4835,8 @@
       <x:c r="C491" s="9"/>
       <x:c r="D491" s="9"/>
       <x:c r="E491" s="9"/>
+      <x:c r="F491" s="29"/>
+      <x:c r="G491" s="29"/>
     </x:row>
     <x:row r="492">
       <x:c r="A492" s="8"/>
@@ -3788,6 +4844,8 @@
       <x:c r="C492" s="9"/>
       <x:c r="D492" s="9"/>
       <x:c r="E492" s="9"/>
+      <x:c r="F492" s="25"/>
+      <x:c r="G492" s="25"/>
     </x:row>
     <x:row r="493">
       <x:c r="A493" s="8"/>
@@ -3795,6 +4853,8 @@
       <x:c r="C493" s="9"/>
       <x:c r="D493" s="9"/>
       <x:c r="E493" s="9"/>
+      <x:c r="F493" s="29"/>
+      <x:c r="G493" s="29"/>
     </x:row>
     <x:row r="494">
       <x:c r="A494" s="8"/>
@@ -3802,6 +4862,8 @@
       <x:c r="C494" s="9"/>
       <x:c r="D494" s="9"/>
       <x:c r="E494" s="9"/>
+      <x:c r="F494" s="25"/>
+      <x:c r="G494" s="25"/>
     </x:row>
     <x:row r="495">
       <x:c r="A495" s="8"/>
@@ -3809,6 +4871,8 @@
       <x:c r="C495" s="9"/>
       <x:c r="D495" s="9"/>
       <x:c r="E495" s="9"/>
+      <x:c r="F495" s="29"/>
+      <x:c r="G495" s="29"/>
     </x:row>
     <x:row r="496">
       <x:c r="A496" s="8"/>
@@ -3816,6 +4880,8 @@
       <x:c r="C496" s="9"/>
       <x:c r="D496" s="9"/>
       <x:c r="E496" s="9"/>
+      <x:c r="F496" s="25"/>
+      <x:c r="G496" s="25"/>
     </x:row>
     <x:row r="497">
       <x:c r="A497" s="8"/>
@@ -3823,6 +4889,8 @@
       <x:c r="C497" s="9"/>
       <x:c r="D497" s="9"/>
       <x:c r="E497" s="9"/>
+      <x:c r="F497" s="29"/>
+      <x:c r="G497" s="29"/>
     </x:row>
     <x:row r="498">
       <x:c r="A498" s="8"/>
@@ -3830,6 +4898,8 @@
       <x:c r="C498" s="9"/>
       <x:c r="D498" s="9"/>
       <x:c r="E498" s="9"/>
+      <x:c r="F498" s="25"/>
+      <x:c r="G498" s="25"/>
     </x:row>
     <x:row r="499">
       <x:c r="A499" s="8"/>
@@ -3837,6 +4907,8 @@
       <x:c r="C499" s="9"/>
       <x:c r="D499" s="9"/>
       <x:c r="E499" s="9"/>
+      <x:c r="F499" s="29"/>
+      <x:c r="G499" s="29"/>
     </x:row>
     <x:row r="500">
       <x:c r="A500" s="8"/>
@@ -3844,11 +4916,21 @@
       <x:c r="C500" s="9"/>
       <x:c r="D500" s="9"/>
       <x:c r="E500" s="9"/>
+      <x:c r="F500" s="25"/>
+      <x:c r="G500" s="25"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="D2:D500">
+      <x:formula1>"AUTO,FCO,FNO,OGU"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E2:E500">
+      <x:formula1>"Pronaf B,Pronaf B para mulheres,Pronaf B agroecológico/orgânico,Pronaf B quintais produtivos"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re564b99b99b84191"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdf2a2a93db34ddc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3861,79 +4943,95 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="85" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="86" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A1" s="14" t="str">
+      <x:c r="A1" s="31" t="str">
         <x:v>MODELO DE CONSULTA EM LISTA</x:v>
       </x:c>
-      <x:c r="B1" s="14" t="str">
+      <x:c r="B1" s="31" t="str">
         <x:v>Preencha somente a aba Consultas</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="15" t="str">
+      <x:c r="A2" s="35" t="str">
         <x:v>CPF_CNPJ</x:v>
       </x:c>
-      <x:c r="B2" s="16" t="str">
+      <x:c r="B2" s="37" t="str">
         <x:v>Obrigatório. Pode ser digitado com ou sem pontos, barra e traço.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="15" t="str">
+      <x:c r="A3" s="35" t="str">
         <x:v>CAR</x:v>
       </x:c>
-      <x:c r="B3" s="16" t="str">
+      <x:c r="B3" s="37" t="str">
         <x:v>Opcional. Se ficar vazio, todos os CARs distintos encontrados para o CPF/CNPJ serão analisados.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="15" t="str">
+      <x:c r="A4" s="35" t="str">
         <x:v>PROPRIETARIO_POSSUIDOR</x:v>
       </x:c>
-      <x:c r="B4" s="16" t="str">
+      <x:c r="B4" s="37" t="str">
         <x:v>Opcional. Use quando o proprietário/possuidor for diferente do CPF/CNPJ consultado.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="15" t="str">
+      <x:c r="A5" s="35" t="str">
+        <x:v>FONTE_RECURSOS</x:v>
+      </x:c>
+      <x:c r="B5" s="37" t="str">
+        <x:v>Obrigatório. Escolha AUTO para sugestão pela UF do CAR ou informe FCO, FNO ou OGU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="35" t="str">
+        <x:v>LINHA_CREDITO</x:v>
+      </x:c>
+      <x:c r="B6" s="37" t="str">
+        <x:v>Obrigatório. Selecione uma das linhas Pronaf B disponíveis na lista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="35" t="str">
         <x:v>REFERENCIA_INTERNA</x:v>
       </x:c>
-      <x:c r="B5" s="16" t="str">
+      <x:c r="B7" s="37" t="str">
         <x:v>Opcional. Número da proposta, contrato ou outro código usado pela instituição.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="15" t="str">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="35" t="str">
         <x:v>OBSERVACAO</x:v>
       </x:c>
-      <x:c r="B6" s="16" t="str">
+      <x:c r="B8" s="37" t="str">
         <x:v>Opcional. Texto que deverá acompanhar o item no relatório consolidado.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="15" t="str">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="35" t="str">
         <x:v>Exemplo CPF</x:v>
       </x:c>
-      <x:c r="B7" s="16" t="str">
+      <x:c r="B9" s="37" t="str">
         <x:v>123.456.789-00</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="15" t="str">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="35" t="str">
         <x:v>Exemplo CAR</x:v>
       </x:c>
-      <x:c r="B8" s="16" t="str">
+      <x:c r="B10" s="37" t="str">
         <x:v>RO-1101500-XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="15" t="str">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="35" t="str">
         <x:v>Saída</x:v>
       </x:c>
-      <x:c r="B9" s="16" t="str">
-        <x:v>Um PDF consolidado, agrupado por CPF/CNPJ, e um JSON de auditoria.</x:v>
+      <x:c r="B11" s="37" t="str">
+        <x:v>Um PDF consolidado de pré-análise, agrupado por CPF/CNPJ, e um JSON de auditoria.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(analysis): add explainable microcredit workflows
</commit_message>
<xml_diff>
--- a/assets/modelo_consulta_lote.xlsx
+++ b/assets/modelo_consulta_lote.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultas" sheetId="1" r:id="R384b169ef2f740f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" r:id="R75c0191f12d04e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultas" sheetId="1" r:id="R33e1b5d7b903427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" r:id="Rb3cf97369ee24a52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -69,14 +69,39 @@
         <x:fgColor rgb="FFEDF5F1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF165C41"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFB7DEE8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF5F1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF3DB7E9"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -109,6 +134,49 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -331,8 +399,10 @@
     <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="49" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -346,9 +416,15 @@
         <x:v>PROPRIETARIO_POSSUIDOR</x:v>
       </x:c>
       <x:c r="D1" s="7" t="str">
+        <x:v>FONTE_RECURSOS</x:v>
+      </x:c>
+      <x:c r="E1" s="7" t="str">
+        <x:v>LINHA_CREDITO</x:v>
+      </x:c>
+      <x:c r="F1" s="21" t="str">
         <x:v>REFERENCIA_INTERNA</x:v>
       </x:c>
-      <x:c r="E1" s="7" t="str">
+      <x:c r="G1" s="21" t="str">
         <x:v>OBSERVACAO</x:v>
       </x:c>
     </x:row>
@@ -358,6 +434,8 @@
       <x:c r="C2" s="9" t="str"/>
       <x:c r="D2" s="9" t="str"/>
       <x:c r="E2" s="9" t="str"/>
+      <x:c r="F2" s="25"/>
+      <x:c r="G2" s="25"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8"/>
@@ -365,6 +443,8 @@
       <x:c r="C3" s="9"/>
       <x:c r="D3" s="9"/>
       <x:c r="E3" s="9"/>
+      <x:c r="F3" s="29"/>
+      <x:c r="G3" s="29"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="8"/>
@@ -372,6 +452,8 @@
       <x:c r="C4" s="9"/>
       <x:c r="D4" s="9"/>
       <x:c r="E4" s="9"/>
+      <x:c r="F4" s="25"/>
+      <x:c r="G4" s="25"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8"/>
@@ -379,6 +461,8 @@
       <x:c r="C5" s="9"/>
       <x:c r="D5" s="9"/>
       <x:c r="E5" s="9"/>
+      <x:c r="F5" s="29"/>
+      <x:c r="G5" s="29"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8"/>
@@ -386,6 +470,8 @@
       <x:c r="C6" s="9"/>
       <x:c r="D6" s="9"/>
       <x:c r="E6" s="9"/>
+      <x:c r="F6" s="25"/>
+      <x:c r="G6" s="25"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="8"/>
@@ -393,6 +479,8 @@
       <x:c r="C7" s="9"/>
       <x:c r="D7" s="9"/>
       <x:c r="E7" s="9"/>
+      <x:c r="F7" s="29"/>
+      <x:c r="G7" s="29"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="8"/>
@@ -400,6 +488,8 @@
       <x:c r="C8" s="9"/>
       <x:c r="D8" s="9"/>
       <x:c r="E8" s="9"/>
+      <x:c r="F8" s="25"/>
+      <x:c r="G8" s="25"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="8"/>
@@ -407,6 +497,8 @@
       <x:c r="C9" s="9"/>
       <x:c r="D9" s="9"/>
       <x:c r="E9" s="9"/>
+      <x:c r="F9" s="29"/>
+      <x:c r="G9" s="29"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8"/>
@@ -414,6 +506,8 @@
       <x:c r="C10" s="9"/>
       <x:c r="D10" s="9"/>
       <x:c r="E10" s="9"/>
+      <x:c r="F10" s="25"/>
+      <x:c r="G10" s="25"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8"/>
@@ -421,6 +515,8 @@
       <x:c r="C11" s="9"/>
       <x:c r="D11" s="9"/>
       <x:c r="E11" s="9"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8"/>
@@ -428,6 +524,8 @@
       <x:c r="C12" s="9"/>
       <x:c r="D12" s="9"/>
       <x:c r="E12" s="9"/>
+      <x:c r="F12" s="25"/>
+      <x:c r="G12" s="25"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8"/>
@@ -435,6 +533,8 @@
       <x:c r="C13" s="9"/>
       <x:c r="D13" s="9"/>
       <x:c r="E13" s="9"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8"/>
@@ -442,6 +542,8 @@
       <x:c r="C14" s="9"/>
       <x:c r="D14" s="9"/>
       <x:c r="E14" s="9"/>
+      <x:c r="F14" s="25"/>
+      <x:c r="G14" s="25"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8"/>
@@ -449,6 +551,8 @@
       <x:c r="C15" s="9"/>
       <x:c r="D15" s="9"/>
       <x:c r="E15" s="9"/>
+      <x:c r="F15" s="29"/>
+      <x:c r="G15" s="29"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8"/>
@@ -456,6 +560,8 @@
       <x:c r="C16" s="9"/>
       <x:c r="D16" s="9"/>
       <x:c r="E16" s="9"/>
+      <x:c r="F16" s="25"/>
+      <x:c r="G16" s="25"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8"/>
@@ -463,6 +569,8 @@
       <x:c r="C17" s="9"/>
       <x:c r="D17" s="9"/>
       <x:c r="E17" s="9"/>
+      <x:c r="F17" s="29"/>
+      <x:c r="G17" s="29"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8"/>
@@ -470,6 +578,8 @@
       <x:c r="C18" s="9"/>
       <x:c r="D18" s="9"/>
       <x:c r="E18" s="9"/>
+      <x:c r="F18" s="25"/>
+      <x:c r="G18" s="25"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8"/>
@@ -477,6 +587,8 @@
       <x:c r="C19" s="9"/>
       <x:c r="D19" s="9"/>
       <x:c r="E19" s="9"/>
+      <x:c r="F19" s="29"/>
+      <x:c r="G19" s="29"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8"/>
@@ -484,6 +596,8 @@
       <x:c r="C20" s="9"/>
       <x:c r="D20" s="9"/>
       <x:c r="E20" s="9"/>
+      <x:c r="F20" s="25"/>
+      <x:c r="G20" s="25"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="8"/>
@@ -491,6 +605,8 @@
       <x:c r="C21" s="9"/>
       <x:c r="D21" s="9"/>
       <x:c r="E21" s="9"/>
+      <x:c r="F21" s="29"/>
+      <x:c r="G21" s="29"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="8"/>
@@ -498,6 +614,8 @@
       <x:c r="C22" s="9"/>
       <x:c r="D22" s="9"/>
       <x:c r="E22" s="9"/>
+      <x:c r="F22" s="25"/>
+      <x:c r="G22" s="25"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="8"/>
@@ -505,6 +623,8 @@
       <x:c r="C23" s="9"/>
       <x:c r="D23" s="9"/>
       <x:c r="E23" s="9"/>
+      <x:c r="F23" s="29"/>
+      <x:c r="G23" s="29"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="8"/>
@@ -512,6 +632,8 @@
       <x:c r="C24" s="9"/>
       <x:c r="D24" s="9"/>
       <x:c r="E24" s="9"/>
+      <x:c r="F24" s="25"/>
+      <x:c r="G24" s="25"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="8"/>
@@ -519,6 +641,8 @@
       <x:c r="C25" s="9"/>
       <x:c r="D25" s="9"/>
       <x:c r="E25" s="9"/>
+      <x:c r="F25" s="29"/>
+      <x:c r="G25" s="29"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="8"/>
@@ -526,6 +650,8 @@
       <x:c r="C26" s="9"/>
       <x:c r="D26" s="9"/>
       <x:c r="E26" s="9"/>
+      <x:c r="F26" s="25"/>
+      <x:c r="G26" s="25"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="8"/>
@@ -533,6 +659,8 @@
       <x:c r="C27" s="9"/>
       <x:c r="D27" s="9"/>
       <x:c r="E27" s="9"/>
+      <x:c r="F27" s="29"/>
+      <x:c r="G27" s="29"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="8"/>
@@ -540,6 +668,8 @@
       <x:c r="C28" s="9"/>
       <x:c r="D28" s="9"/>
       <x:c r="E28" s="9"/>
+      <x:c r="F28" s="25"/>
+      <x:c r="G28" s="25"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="8"/>
@@ -547,6 +677,8 @@
       <x:c r="C29" s="9"/>
       <x:c r="D29" s="9"/>
       <x:c r="E29" s="9"/>
+      <x:c r="F29" s="29"/>
+      <x:c r="G29" s="29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="8"/>
@@ -554,6 +686,8 @@
       <x:c r="C30" s="9"/>
       <x:c r="D30" s="9"/>
       <x:c r="E30" s="9"/>
+      <x:c r="F30" s="25"/>
+      <x:c r="G30" s="25"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="8"/>
@@ -561,6 +695,8 @@
       <x:c r="C31" s="9"/>
       <x:c r="D31" s="9"/>
       <x:c r="E31" s="9"/>
+      <x:c r="F31" s="29"/>
+      <x:c r="G31" s="29"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="8"/>
@@ -568,6 +704,8 @@
       <x:c r="C32" s="9"/>
       <x:c r="D32" s="9"/>
       <x:c r="E32" s="9"/>
+      <x:c r="F32" s="25"/>
+      <x:c r="G32" s="25"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="8"/>
@@ -575,6 +713,8 @@
       <x:c r="C33" s="9"/>
       <x:c r="D33" s="9"/>
       <x:c r="E33" s="9"/>
+      <x:c r="F33" s="29"/>
+      <x:c r="G33" s="29"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="8"/>
@@ -582,6 +722,8 @@
       <x:c r="C34" s="9"/>
       <x:c r="D34" s="9"/>
       <x:c r="E34" s="9"/>
+      <x:c r="F34" s="25"/>
+      <x:c r="G34" s="25"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="8"/>
@@ -589,6 +731,8 @@
       <x:c r="C35" s="9"/>
       <x:c r="D35" s="9"/>
       <x:c r="E35" s="9"/>
+      <x:c r="F35" s="29"/>
+      <x:c r="G35" s="29"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="8"/>
@@ -596,6 +740,8 @@
       <x:c r="C36" s="9"/>
       <x:c r="D36" s="9"/>
       <x:c r="E36" s="9"/>
+      <x:c r="F36" s="25"/>
+      <x:c r="G36" s="25"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="8"/>
@@ -603,6 +749,8 @@
       <x:c r="C37" s="9"/>
       <x:c r="D37" s="9"/>
       <x:c r="E37" s="9"/>
+      <x:c r="F37" s="29"/>
+      <x:c r="G37" s="29"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="8"/>
@@ -610,6 +758,8 @@
       <x:c r="C38" s="9"/>
       <x:c r="D38" s="9"/>
       <x:c r="E38" s="9"/>
+      <x:c r="F38" s="25"/>
+      <x:c r="G38" s="25"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="8"/>
@@ -617,6 +767,8 @@
       <x:c r="C39" s="9"/>
       <x:c r="D39" s="9"/>
       <x:c r="E39" s="9"/>
+      <x:c r="F39" s="29"/>
+      <x:c r="G39" s="29"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="8"/>
@@ -624,6 +776,8 @@
       <x:c r="C40" s="9"/>
       <x:c r="D40" s="9"/>
       <x:c r="E40" s="9"/>
+      <x:c r="F40" s="25"/>
+      <x:c r="G40" s="25"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="8"/>
@@ -631,6 +785,8 @@
       <x:c r="C41" s="9"/>
       <x:c r="D41" s="9"/>
       <x:c r="E41" s="9"/>
+      <x:c r="F41" s="29"/>
+      <x:c r="G41" s="29"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="8"/>
@@ -638,6 +794,8 @@
       <x:c r="C42" s="9"/>
       <x:c r="D42" s="9"/>
       <x:c r="E42" s="9"/>
+      <x:c r="F42" s="25"/>
+      <x:c r="G42" s="25"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="8"/>
@@ -645,6 +803,8 @@
       <x:c r="C43" s="9"/>
       <x:c r="D43" s="9"/>
       <x:c r="E43" s="9"/>
+      <x:c r="F43" s="29"/>
+      <x:c r="G43" s="29"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="8"/>
@@ -652,6 +812,8 @@
       <x:c r="C44" s="9"/>
       <x:c r="D44" s="9"/>
       <x:c r="E44" s="9"/>
+      <x:c r="F44" s="25"/>
+      <x:c r="G44" s="25"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="8"/>
@@ -659,6 +821,8 @@
       <x:c r="C45" s="9"/>
       <x:c r="D45" s="9"/>
       <x:c r="E45" s="9"/>
+      <x:c r="F45" s="29"/>
+      <x:c r="G45" s="29"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="8"/>
@@ -666,6 +830,8 @@
       <x:c r="C46" s="9"/>
       <x:c r="D46" s="9"/>
       <x:c r="E46" s="9"/>
+      <x:c r="F46" s="25"/>
+      <x:c r="G46" s="25"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="8"/>
@@ -673,6 +839,8 @@
       <x:c r="C47" s="9"/>
       <x:c r="D47" s="9"/>
       <x:c r="E47" s="9"/>
+      <x:c r="F47" s="29"/>
+      <x:c r="G47" s="29"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="8"/>
@@ -680,6 +848,8 @@
       <x:c r="C48" s="9"/>
       <x:c r="D48" s="9"/>
       <x:c r="E48" s="9"/>
+      <x:c r="F48" s="25"/>
+      <x:c r="G48" s="25"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="8"/>
@@ -687,6 +857,8 @@
       <x:c r="C49" s="9"/>
       <x:c r="D49" s="9"/>
       <x:c r="E49" s="9"/>
+      <x:c r="F49" s="29"/>
+      <x:c r="G49" s="29"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="8"/>
@@ -694,6 +866,8 @@
       <x:c r="C50" s="9"/>
       <x:c r="D50" s="9"/>
       <x:c r="E50" s="9"/>
+      <x:c r="F50" s="25"/>
+      <x:c r="G50" s="25"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="8"/>
@@ -701,6 +875,8 @@
       <x:c r="C51" s="9"/>
       <x:c r="D51" s="9"/>
       <x:c r="E51" s="9"/>
+      <x:c r="F51" s="29"/>
+      <x:c r="G51" s="29"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="8"/>
@@ -708,6 +884,8 @@
       <x:c r="C52" s="9"/>
       <x:c r="D52" s="9"/>
       <x:c r="E52" s="9"/>
+      <x:c r="F52" s="25"/>
+      <x:c r="G52" s="25"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="8"/>
@@ -715,6 +893,8 @@
       <x:c r="C53" s="9"/>
       <x:c r="D53" s="9"/>
       <x:c r="E53" s="9"/>
+      <x:c r="F53" s="29"/>
+      <x:c r="G53" s="29"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="8"/>
@@ -722,6 +902,8 @@
       <x:c r="C54" s="9"/>
       <x:c r="D54" s="9"/>
       <x:c r="E54" s="9"/>
+      <x:c r="F54" s="25"/>
+      <x:c r="G54" s="25"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="8"/>
@@ -729,6 +911,8 @@
       <x:c r="C55" s="9"/>
       <x:c r="D55" s="9"/>
       <x:c r="E55" s="9"/>
+      <x:c r="F55" s="29"/>
+      <x:c r="G55" s="29"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="8"/>
@@ -736,6 +920,8 @@
       <x:c r="C56" s="9"/>
       <x:c r="D56" s="9"/>
       <x:c r="E56" s="9"/>
+      <x:c r="F56" s="25"/>
+      <x:c r="G56" s="25"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="8"/>
@@ -743,6 +929,8 @@
       <x:c r="C57" s="9"/>
       <x:c r="D57" s="9"/>
       <x:c r="E57" s="9"/>
+      <x:c r="F57" s="29"/>
+      <x:c r="G57" s="29"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="8"/>
@@ -750,6 +938,8 @@
       <x:c r="C58" s="9"/>
       <x:c r="D58" s="9"/>
       <x:c r="E58" s="9"/>
+      <x:c r="F58" s="25"/>
+      <x:c r="G58" s="25"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="8"/>
@@ -757,6 +947,8 @@
       <x:c r="C59" s="9"/>
       <x:c r="D59" s="9"/>
       <x:c r="E59" s="9"/>
+      <x:c r="F59" s="29"/>
+      <x:c r="G59" s="29"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="8"/>
@@ -764,6 +956,8 @@
       <x:c r="C60" s="9"/>
       <x:c r="D60" s="9"/>
       <x:c r="E60" s="9"/>
+      <x:c r="F60" s="25"/>
+      <x:c r="G60" s="25"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="8"/>
@@ -771,6 +965,8 @@
       <x:c r="C61" s="9"/>
       <x:c r="D61" s="9"/>
       <x:c r="E61" s="9"/>
+      <x:c r="F61" s="29"/>
+      <x:c r="G61" s="29"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="8"/>
@@ -778,6 +974,8 @@
       <x:c r="C62" s="9"/>
       <x:c r="D62" s="9"/>
       <x:c r="E62" s="9"/>
+      <x:c r="F62" s="25"/>
+      <x:c r="G62" s="25"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="8"/>
@@ -785,6 +983,8 @@
       <x:c r="C63" s="9"/>
       <x:c r="D63" s="9"/>
       <x:c r="E63" s="9"/>
+      <x:c r="F63" s="29"/>
+      <x:c r="G63" s="29"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="8"/>
@@ -792,6 +992,8 @@
       <x:c r="C64" s="9"/>
       <x:c r="D64" s="9"/>
       <x:c r="E64" s="9"/>
+      <x:c r="F64" s="25"/>
+      <x:c r="G64" s="25"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="8"/>
@@ -799,6 +1001,8 @@
       <x:c r="C65" s="9"/>
       <x:c r="D65" s="9"/>
       <x:c r="E65" s="9"/>
+      <x:c r="F65" s="29"/>
+      <x:c r="G65" s="29"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="8"/>
@@ -806,6 +1010,8 @@
       <x:c r="C66" s="9"/>
       <x:c r="D66" s="9"/>
       <x:c r="E66" s="9"/>
+      <x:c r="F66" s="25"/>
+      <x:c r="G66" s="25"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="8"/>
@@ -813,6 +1019,8 @@
       <x:c r="C67" s="9"/>
       <x:c r="D67" s="9"/>
       <x:c r="E67" s="9"/>
+      <x:c r="F67" s="29"/>
+      <x:c r="G67" s="29"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="8"/>
@@ -820,6 +1028,8 @@
       <x:c r="C68" s="9"/>
       <x:c r="D68" s="9"/>
       <x:c r="E68" s="9"/>
+      <x:c r="F68" s="25"/>
+      <x:c r="G68" s="25"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="8"/>
@@ -827,6 +1037,8 @@
       <x:c r="C69" s="9"/>
       <x:c r="D69" s="9"/>
       <x:c r="E69" s="9"/>
+      <x:c r="F69" s="29"/>
+      <x:c r="G69" s="29"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="8"/>
@@ -834,6 +1046,8 @@
       <x:c r="C70" s="9"/>
       <x:c r="D70" s="9"/>
       <x:c r="E70" s="9"/>
+      <x:c r="F70" s="25"/>
+      <x:c r="G70" s="25"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="8"/>
@@ -841,6 +1055,8 @@
       <x:c r="C71" s="9"/>
       <x:c r="D71" s="9"/>
       <x:c r="E71" s="9"/>
+      <x:c r="F71" s="29"/>
+      <x:c r="G71" s="29"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="8"/>
@@ -848,6 +1064,8 @@
       <x:c r="C72" s="9"/>
       <x:c r="D72" s="9"/>
       <x:c r="E72" s="9"/>
+      <x:c r="F72" s="25"/>
+      <x:c r="G72" s="25"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="8"/>
@@ -855,6 +1073,8 @@
       <x:c r="C73" s="9"/>
       <x:c r="D73" s="9"/>
       <x:c r="E73" s="9"/>
+      <x:c r="F73" s="29"/>
+      <x:c r="G73" s="29"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="8"/>
@@ -862,6 +1082,8 @@
       <x:c r="C74" s="9"/>
       <x:c r="D74" s="9"/>
       <x:c r="E74" s="9"/>
+      <x:c r="F74" s="25"/>
+      <x:c r="G74" s="25"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="8"/>
@@ -869,6 +1091,8 @@
       <x:c r="C75" s="9"/>
       <x:c r="D75" s="9"/>
       <x:c r="E75" s="9"/>
+      <x:c r="F75" s="29"/>
+      <x:c r="G75" s="29"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="8"/>
@@ -876,6 +1100,8 @@
       <x:c r="C76" s="9"/>
       <x:c r="D76" s="9"/>
       <x:c r="E76" s="9"/>
+      <x:c r="F76" s="25"/>
+      <x:c r="G76" s="25"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="8"/>
@@ -883,6 +1109,8 @@
       <x:c r="C77" s="9"/>
       <x:c r="D77" s="9"/>
       <x:c r="E77" s="9"/>
+      <x:c r="F77" s="29"/>
+      <x:c r="G77" s="29"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="8"/>
@@ -890,6 +1118,8 @@
       <x:c r="C78" s="9"/>
       <x:c r="D78" s="9"/>
       <x:c r="E78" s="9"/>
+      <x:c r="F78" s="25"/>
+      <x:c r="G78" s="25"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="8"/>
@@ -897,6 +1127,8 @@
       <x:c r="C79" s="9"/>
       <x:c r="D79" s="9"/>
       <x:c r="E79" s="9"/>
+      <x:c r="F79" s="29"/>
+      <x:c r="G79" s="29"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="8"/>
@@ -904,6 +1136,8 @@
       <x:c r="C80" s="9"/>
       <x:c r="D80" s="9"/>
       <x:c r="E80" s="9"/>
+      <x:c r="F80" s="25"/>
+      <x:c r="G80" s="25"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="8"/>
@@ -911,6 +1145,8 @@
       <x:c r="C81" s="9"/>
       <x:c r="D81" s="9"/>
       <x:c r="E81" s="9"/>
+      <x:c r="F81" s="29"/>
+      <x:c r="G81" s="29"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="8"/>
@@ -918,6 +1154,8 @@
       <x:c r="C82" s="9"/>
       <x:c r="D82" s="9"/>
       <x:c r="E82" s="9"/>
+      <x:c r="F82" s="25"/>
+      <x:c r="G82" s="25"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="8"/>
@@ -925,6 +1163,8 @@
       <x:c r="C83" s="9"/>
       <x:c r="D83" s="9"/>
       <x:c r="E83" s="9"/>
+      <x:c r="F83" s="29"/>
+      <x:c r="G83" s="29"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="8"/>
@@ -932,6 +1172,8 @@
       <x:c r="C84" s="9"/>
       <x:c r="D84" s="9"/>
       <x:c r="E84" s="9"/>
+      <x:c r="F84" s="25"/>
+      <x:c r="G84" s="25"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="8"/>
@@ -939,6 +1181,8 @@
       <x:c r="C85" s="9"/>
       <x:c r="D85" s="9"/>
       <x:c r="E85" s="9"/>
+      <x:c r="F85" s="29"/>
+      <x:c r="G85" s="29"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="8"/>
@@ -946,6 +1190,8 @@
       <x:c r="C86" s="9"/>
       <x:c r="D86" s="9"/>
       <x:c r="E86" s="9"/>
+      <x:c r="F86" s="25"/>
+      <x:c r="G86" s="25"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="8"/>
@@ -953,6 +1199,8 @@
       <x:c r="C87" s="9"/>
       <x:c r="D87" s="9"/>
       <x:c r="E87" s="9"/>
+      <x:c r="F87" s="29"/>
+      <x:c r="G87" s="29"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="8"/>
@@ -960,6 +1208,8 @@
       <x:c r="C88" s="9"/>
       <x:c r="D88" s="9"/>
       <x:c r="E88" s="9"/>
+      <x:c r="F88" s="25"/>
+      <x:c r="G88" s="25"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="8"/>
@@ -967,6 +1217,8 @@
       <x:c r="C89" s="9"/>
       <x:c r="D89" s="9"/>
       <x:c r="E89" s="9"/>
+      <x:c r="F89" s="29"/>
+      <x:c r="G89" s="29"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="8"/>
@@ -974,6 +1226,8 @@
       <x:c r="C90" s="9"/>
       <x:c r="D90" s="9"/>
       <x:c r="E90" s="9"/>
+      <x:c r="F90" s="25"/>
+      <x:c r="G90" s="25"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="8"/>
@@ -981,6 +1235,8 @@
       <x:c r="C91" s="9"/>
       <x:c r="D91" s="9"/>
       <x:c r="E91" s="9"/>
+      <x:c r="F91" s="29"/>
+      <x:c r="G91" s="29"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="8"/>
@@ -988,6 +1244,8 @@
       <x:c r="C92" s="9"/>
       <x:c r="D92" s="9"/>
       <x:c r="E92" s="9"/>
+      <x:c r="F92" s="25"/>
+      <x:c r="G92" s="25"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="8"/>
@@ -995,6 +1253,8 @@
       <x:c r="C93" s="9"/>
       <x:c r="D93" s="9"/>
       <x:c r="E93" s="9"/>
+      <x:c r="F93" s="29"/>
+      <x:c r="G93" s="29"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="8"/>
@@ -1002,6 +1262,8 @@
       <x:c r="C94" s="9"/>
       <x:c r="D94" s="9"/>
       <x:c r="E94" s="9"/>
+      <x:c r="F94" s="25"/>
+      <x:c r="G94" s="25"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="8"/>
@@ -1009,6 +1271,8 @@
       <x:c r="C95" s="9"/>
       <x:c r="D95" s="9"/>
       <x:c r="E95" s="9"/>
+      <x:c r="F95" s="29"/>
+      <x:c r="G95" s="29"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="8"/>
@@ -1016,6 +1280,8 @@
       <x:c r="C96" s="9"/>
       <x:c r="D96" s="9"/>
       <x:c r="E96" s="9"/>
+      <x:c r="F96" s="25"/>
+      <x:c r="G96" s="25"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="8"/>
@@ -1023,6 +1289,8 @@
       <x:c r="C97" s="9"/>
       <x:c r="D97" s="9"/>
       <x:c r="E97" s="9"/>
+      <x:c r="F97" s="29"/>
+      <x:c r="G97" s="29"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="8"/>
@@ -1030,6 +1298,8 @@
       <x:c r="C98" s="9"/>
       <x:c r="D98" s="9"/>
       <x:c r="E98" s="9"/>
+      <x:c r="F98" s="25"/>
+      <x:c r="G98" s="25"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="8"/>
@@ -1037,6 +1307,8 @@
       <x:c r="C99" s="9"/>
       <x:c r="D99" s="9"/>
       <x:c r="E99" s="9"/>
+      <x:c r="F99" s="29"/>
+      <x:c r="G99" s="29"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="8"/>
@@ -1044,6 +1316,8 @@
       <x:c r="C100" s="9"/>
       <x:c r="D100" s="9"/>
       <x:c r="E100" s="9"/>
+      <x:c r="F100" s="25"/>
+      <x:c r="G100" s="25"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="8"/>
@@ -1051,6 +1325,8 @@
       <x:c r="C101" s="9"/>
       <x:c r="D101" s="9"/>
       <x:c r="E101" s="9"/>
+      <x:c r="F101" s="29"/>
+      <x:c r="G101" s="29"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="8"/>
@@ -1058,6 +1334,8 @@
       <x:c r="C102" s="9"/>
       <x:c r="D102" s="9"/>
       <x:c r="E102" s="9"/>
+      <x:c r="F102" s="25"/>
+      <x:c r="G102" s="25"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="8"/>
@@ -1065,6 +1343,8 @@
       <x:c r="C103" s="9"/>
       <x:c r="D103" s="9"/>
       <x:c r="E103" s="9"/>
+      <x:c r="F103" s="29"/>
+      <x:c r="G103" s="29"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="8"/>
@@ -1072,6 +1352,8 @@
       <x:c r="C104" s="9"/>
       <x:c r="D104" s="9"/>
       <x:c r="E104" s="9"/>
+      <x:c r="F104" s="25"/>
+      <x:c r="G104" s="25"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="8"/>
@@ -1079,6 +1361,8 @@
       <x:c r="C105" s="9"/>
       <x:c r="D105" s="9"/>
       <x:c r="E105" s="9"/>
+      <x:c r="F105" s="29"/>
+      <x:c r="G105" s="29"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="8"/>
@@ -1086,6 +1370,8 @@
       <x:c r="C106" s="9"/>
       <x:c r="D106" s="9"/>
       <x:c r="E106" s="9"/>
+      <x:c r="F106" s="25"/>
+      <x:c r="G106" s="25"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="8"/>
@@ -1093,6 +1379,8 @@
       <x:c r="C107" s="9"/>
       <x:c r="D107" s="9"/>
       <x:c r="E107" s="9"/>
+      <x:c r="F107" s="29"/>
+      <x:c r="G107" s="29"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="8"/>
@@ -1100,6 +1388,8 @@
       <x:c r="C108" s="9"/>
       <x:c r="D108" s="9"/>
       <x:c r="E108" s="9"/>
+      <x:c r="F108" s="25"/>
+      <x:c r="G108" s="25"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="8"/>
@@ -1107,6 +1397,8 @@
       <x:c r="C109" s="9"/>
       <x:c r="D109" s="9"/>
       <x:c r="E109" s="9"/>
+      <x:c r="F109" s="29"/>
+      <x:c r="G109" s="29"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="8"/>
@@ -1114,6 +1406,8 @@
       <x:c r="C110" s="9"/>
       <x:c r="D110" s="9"/>
       <x:c r="E110" s="9"/>
+      <x:c r="F110" s="25"/>
+      <x:c r="G110" s="25"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="8"/>
@@ -1121,6 +1415,8 @@
       <x:c r="C111" s="9"/>
       <x:c r="D111" s="9"/>
       <x:c r="E111" s="9"/>
+      <x:c r="F111" s="29"/>
+      <x:c r="G111" s="29"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="8"/>
@@ -1128,6 +1424,8 @@
       <x:c r="C112" s="9"/>
       <x:c r="D112" s="9"/>
       <x:c r="E112" s="9"/>
+      <x:c r="F112" s="25"/>
+      <x:c r="G112" s="25"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="8"/>
@@ -1135,6 +1433,8 @@
       <x:c r="C113" s="9"/>
       <x:c r="D113" s="9"/>
       <x:c r="E113" s="9"/>
+      <x:c r="F113" s="29"/>
+      <x:c r="G113" s="29"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="8"/>
@@ -1142,6 +1442,8 @@
       <x:c r="C114" s="9"/>
       <x:c r="D114" s="9"/>
       <x:c r="E114" s="9"/>
+      <x:c r="F114" s="25"/>
+      <x:c r="G114" s="25"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="8"/>
@@ -1149,6 +1451,8 @@
       <x:c r="C115" s="9"/>
       <x:c r="D115" s="9"/>
       <x:c r="E115" s="9"/>
+      <x:c r="F115" s="29"/>
+      <x:c r="G115" s="29"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="8"/>
@@ -1156,6 +1460,8 @@
       <x:c r="C116" s="9"/>
       <x:c r="D116" s="9"/>
       <x:c r="E116" s="9"/>
+      <x:c r="F116" s="25"/>
+      <x:c r="G116" s="25"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="8"/>
@@ -1163,6 +1469,8 @@
       <x:c r="C117" s="9"/>
       <x:c r="D117" s="9"/>
       <x:c r="E117" s="9"/>
+      <x:c r="F117" s="29"/>
+      <x:c r="G117" s="29"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="8"/>
@@ -1170,6 +1478,8 @@
       <x:c r="C118" s="9"/>
       <x:c r="D118" s="9"/>
       <x:c r="E118" s="9"/>
+      <x:c r="F118" s="25"/>
+      <x:c r="G118" s="25"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="8"/>
@@ -1177,6 +1487,8 @@
       <x:c r="C119" s="9"/>
       <x:c r="D119" s="9"/>
       <x:c r="E119" s="9"/>
+      <x:c r="F119" s="29"/>
+      <x:c r="G119" s="29"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="8"/>
@@ -1184,6 +1496,8 @@
       <x:c r="C120" s="9"/>
       <x:c r="D120" s="9"/>
       <x:c r="E120" s="9"/>
+      <x:c r="F120" s="25"/>
+      <x:c r="G120" s="25"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="8"/>
@@ -1191,6 +1505,8 @@
       <x:c r="C121" s="9"/>
       <x:c r="D121" s="9"/>
       <x:c r="E121" s="9"/>
+      <x:c r="F121" s="29"/>
+      <x:c r="G121" s="29"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="8"/>
@@ -1198,6 +1514,8 @@
       <x:c r="C122" s="9"/>
       <x:c r="D122" s="9"/>
       <x:c r="E122" s="9"/>
+      <x:c r="F122" s="25"/>
+      <x:c r="G122" s="25"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="8"/>
@@ -1205,6 +1523,8 @@
       <x:c r="C123" s="9"/>
       <x:c r="D123" s="9"/>
       <x:c r="E123" s="9"/>
+      <x:c r="F123" s="29"/>
+      <x:c r="G123" s="29"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="8"/>
@@ -1212,6 +1532,8 @@
       <x:c r="C124" s="9"/>
       <x:c r="D124" s="9"/>
       <x:c r="E124" s="9"/>
+      <x:c r="F124" s="25"/>
+      <x:c r="G124" s="25"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="8"/>
@@ -1219,6 +1541,8 @@
       <x:c r="C125" s="9"/>
       <x:c r="D125" s="9"/>
       <x:c r="E125" s="9"/>
+      <x:c r="F125" s="29"/>
+      <x:c r="G125" s="29"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="8"/>
@@ -1226,6 +1550,8 @@
       <x:c r="C126" s="9"/>
       <x:c r="D126" s="9"/>
       <x:c r="E126" s="9"/>
+      <x:c r="F126" s="25"/>
+      <x:c r="G126" s="25"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="8"/>
@@ -1233,6 +1559,8 @@
       <x:c r="C127" s="9"/>
       <x:c r="D127" s="9"/>
       <x:c r="E127" s="9"/>
+      <x:c r="F127" s="29"/>
+      <x:c r="G127" s="29"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="8"/>
@@ -1240,6 +1568,8 @@
       <x:c r="C128" s="9"/>
       <x:c r="D128" s="9"/>
       <x:c r="E128" s="9"/>
+      <x:c r="F128" s="25"/>
+      <x:c r="G128" s="25"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="8"/>
@@ -1247,6 +1577,8 @@
       <x:c r="C129" s="9"/>
       <x:c r="D129" s="9"/>
       <x:c r="E129" s="9"/>
+      <x:c r="F129" s="29"/>
+      <x:c r="G129" s="29"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="8"/>
@@ -1254,6 +1586,8 @@
       <x:c r="C130" s="9"/>
       <x:c r="D130" s="9"/>
       <x:c r="E130" s="9"/>
+      <x:c r="F130" s="25"/>
+      <x:c r="G130" s="25"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="8"/>
@@ -1261,6 +1595,8 @@
       <x:c r="C131" s="9"/>
       <x:c r="D131" s="9"/>
       <x:c r="E131" s="9"/>
+      <x:c r="F131" s="29"/>
+      <x:c r="G131" s="29"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="8"/>
@@ -1268,6 +1604,8 @@
       <x:c r="C132" s="9"/>
       <x:c r="D132" s="9"/>
       <x:c r="E132" s="9"/>
+      <x:c r="F132" s="25"/>
+      <x:c r="G132" s="25"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="8"/>
@@ -1275,6 +1613,8 @@
       <x:c r="C133" s="9"/>
       <x:c r="D133" s="9"/>
       <x:c r="E133" s="9"/>
+      <x:c r="F133" s="29"/>
+      <x:c r="G133" s="29"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="8"/>
@@ -1282,6 +1622,8 @@
       <x:c r="C134" s="9"/>
       <x:c r="D134" s="9"/>
       <x:c r="E134" s="9"/>
+      <x:c r="F134" s="25"/>
+      <x:c r="G134" s="25"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="8"/>
@@ -1289,6 +1631,8 @@
       <x:c r="C135" s="9"/>
       <x:c r="D135" s="9"/>
       <x:c r="E135" s="9"/>
+      <x:c r="F135" s="29"/>
+      <x:c r="G135" s="29"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="8"/>
@@ -1296,6 +1640,8 @@
       <x:c r="C136" s="9"/>
       <x:c r="D136" s="9"/>
       <x:c r="E136" s="9"/>
+      <x:c r="F136" s="25"/>
+      <x:c r="G136" s="25"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="8"/>
@@ -1303,6 +1649,8 @@
       <x:c r="C137" s="9"/>
       <x:c r="D137" s="9"/>
       <x:c r="E137" s="9"/>
+      <x:c r="F137" s="29"/>
+      <x:c r="G137" s="29"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="8"/>
@@ -1310,6 +1658,8 @@
       <x:c r="C138" s="9"/>
       <x:c r="D138" s="9"/>
       <x:c r="E138" s="9"/>
+      <x:c r="F138" s="25"/>
+      <x:c r="G138" s="25"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="8"/>
@@ -1317,6 +1667,8 @@
       <x:c r="C139" s="9"/>
       <x:c r="D139" s="9"/>
       <x:c r="E139" s="9"/>
+      <x:c r="F139" s="29"/>
+      <x:c r="G139" s="29"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="8"/>
@@ -1324,6 +1676,8 @@
       <x:c r="C140" s="9"/>
       <x:c r="D140" s="9"/>
       <x:c r="E140" s="9"/>
+      <x:c r="F140" s="25"/>
+      <x:c r="G140" s="25"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="8"/>
@@ -1331,6 +1685,8 @@
       <x:c r="C141" s="9"/>
       <x:c r="D141" s="9"/>
       <x:c r="E141" s="9"/>
+      <x:c r="F141" s="29"/>
+      <x:c r="G141" s="29"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="8"/>
@@ -1338,6 +1694,8 @@
       <x:c r="C142" s="9"/>
       <x:c r="D142" s="9"/>
       <x:c r="E142" s="9"/>
+      <x:c r="F142" s="25"/>
+      <x:c r="G142" s="25"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="8"/>
@@ -1345,6 +1703,8 @@
       <x:c r="C143" s="9"/>
       <x:c r="D143" s="9"/>
       <x:c r="E143" s="9"/>
+      <x:c r="F143" s="29"/>
+      <x:c r="G143" s="29"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="8"/>
@@ -1352,6 +1712,8 @@
       <x:c r="C144" s="9"/>
       <x:c r="D144" s="9"/>
       <x:c r="E144" s="9"/>
+      <x:c r="F144" s="25"/>
+      <x:c r="G144" s="25"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="8"/>
@@ -1359,6 +1721,8 @@
       <x:c r="C145" s="9"/>
       <x:c r="D145" s="9"/>
       <x:c r="E145" s="9"/>
+      <x:c r="F145" s="29"/>
+      <x:c r="G145" s="29"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="8"/>
@@ -1366,6 +1730,8 @@
       <x:c r="C146" s="9"/>
       <x:c r="D146" s="9"/>
       <x:c r="E146" s="9"/>
+      <x:c r="F146" s="25"/>
+      <x:c r="G146" s="25"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="8"/>
@@ -1373,6 +1739,8 @@
       <x:c r="C147" s="9"/>
       <x:c r="D147" s="9"/>
       <x:c r="E147" s="9"/>
+      <x:c r="F147" s="29"/>
+      <x:c r="G147" s="29"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="8"/>
@@ -1380,6 +1748,8 @@
       <x:c r="C148" s="9"/>
       <x:c r="D148" s="9"/>
       <x:c r="E148" s="9"/>
+      <x:c r="F148" s="25"/>
+      <x:c r="G148" s="25"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="8"/>
@@ -1387,6 +1757,8 @@
       <x:c r="C149" s="9"/>
       <x:c r="D149" s="9"/>
       <x:c r="E149" s="9"/>
+      <x:c r="F149" s="29"/>
+      <x:c r="G149" s="29"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="8"/>
@@ -1394,6 +1766,8 @@
       <x:c r="C150" s="9"/>
       <x:c r="D150" s="9"/>
       <x:c r="E150" s="9"/>
+      <x:c r="F150" s="25"/>
+      <x:c r="G150" s="25"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="8"/>
@@ -1401,6 +1775,8 @@
       <x:c r="C151" s="9"/>
       <x:c r="D151" s="9"/>
       <x:c r="E151" s="9"/>
+      <x:c r="F151" s="29"/>
+      <x:c r="G151" s="29"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="8"/>
@@ -1408,6 +1784,8 @@
       <x:c r="C152" s="9"/>
       <x:c r="D152" s="9"/>
       <x:c r="E152" s="9"/>
+      <x:c r="F152" s="25"/>
+      <x:c r="G152" s="25"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="8"/>
@@ -1415,6 +1793,8 @@
       <x:c r="C153" s="9"/>
       <x:c r="D153" s="9"/>
       <x:c r="E153" s="9"/>
+      <x:c r="F153" s="29"/>
+      <x:c r="G153" s="29"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="8"/>
@@ -1422,6 +1802,8 @@
       <x:c r="C154" s="9"/>
       <x:c r="D154" s="9"/>
       <x:c r="E154" s="9"/>
+      <x:c r="F154" s="25"/>
+      <x:c r="G154" s="25"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="8"/>
@@ -1429,6 +1811,8 @@
       <x:c r="C155" s="9"/>
       <x:c r="D155" s="9"/>
       <x:c r="E155" s="9"/>
+      <x:c r="F155" s="29"/>
+      <x:c r="G155" s="29"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="8"/>
@@ -1436,6 +1820,8 @@
       <x:c r="C156" s="9"/>
       <x:c r="D156" s="9"/>
       <x:c r="E156" s="9"/>
+      <x:c r="F156" s="25"/>
+      <x:c r="G156" s="25"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="8"/>
@@ -1443,6 +1829,8 @@
       <x:c r="C157" s="9"/>
       <x:c r="D157" s="9"/>
       <x:c r="E157" s="9"/>
+      <x:c r="F157" s="29"/>
+      <x:c r="G157" s="29"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="8"/>
@@ -1450,6 +1838,8 @@
       <x:c r="C158" s="9"/>
       <x:c r="D158" s="9"/>
       <x:c r="E158" s="9"/>
+      <x:c r="F158" s="25"/>
+      <x:c r="G158" s="25"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="8"/>
@@ -1457,6 +1847,8 @@
       <x:c r="C159" s="9"/>
       <x:c r="D159" s="9"/>
       <x:c r="E159" s="9"/>
+      <x:c r="F159" s="29"/>
+      <x:c r="G159" s="29"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="8"/>
@@ -1464,6 +1856,8 @@
       <x:c r="C160" s="9"/>
       <x:c r="D160" s="9"/>
       <x:c r="E160" s="9"/>
+      <x:c r="F160" s="25"/>
+      <x:c r="G160" s="25"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="8"/>
@@ -1471,6 +1865,8 @@
       <x:c r="C161" s="9"/>
       <x:c r="D161" s="9"/>
       <x:c r="E161" s="9"/>
+      <x:c r="F161" s="29"/>
+      <x:c r="G161" s="29"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="8"/>
@@ -1478,6 +1874,8 @@
       <x:c r="C162" s="9"/>
       <x:c r="D162" s="9"/>
       <x:c r="E162" s="9"/>
+      <x:c r="F162" s="25"/>
+      <x:c r="G162" s="25"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="8"/>
@@ -1485,6 +1883,8 @@
       <x:c r="C163" s="9"/>
       <x:c r="D163" s="9"/>
       <x:c r="E163" s="9"/>
+      <x:c r="F163" s="29"/>
+      <x:c r="G163" s="29"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="8"/>
@@ -1492,6 +1892,8 @@
       <x:c r="C164" s="9"/>
       <x:c r="D164" s="9"/>
       <x:c r="E164" s="9"/>
+      <x:c r="F164" s="25"/>
+      <x:c r="G164" s="25"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="8"/>
@@ -1499,6 +1901,8 @@
       <x:c r="C165" s="9"/>
       <x:c r="D165" s="9"/>
       <x:c r="E165" s="9"/>
+      <x:c r="F165" s="29"/>
+      <x:c r="G165" s="29"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="8"/>
@@ -1506,6 +1910,8 @@
       <x:c r="C166" s="9"/>
       <x:c r="D166" s="9"/>
       <x:c r="E166" s="9"/>
+      <x:c r="F166" s="25"/>
+      <x:c r="G166" s="25"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="8"/>
@@ -1513,6 +1919,8 @@
       <x:c r="C167" s="9"/>
       <x:c r="D167" s="9"/>
       <x:c r="E167" s="9"/>
+      <x:c r="F167" s="29"/>
+      <x:c r="G167" s="29"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="8"/>
@@ -1520,6 +1928,8 @@
       <x:c r="C168" s="9"/>
       <x:c r="D168" s="9"/>
       <x:c r="E168" s="9"/>
+      <x:c r="F168" s="25"/>
+      <x:c r="G168" s="25"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="8"/>
@@ -1527,6 +1937,8 @@
       <x:c r="C169" s="9"/>
       <x:c r="D169" s="9"/>
       <x:c r="E169" s="9"/>
+      <x:c r="F169" s="29"/>
+      <x:c r="G169" s="29"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="8"/>
@@ -1534,6 +1946,8 @@
       <x:c r="C170" s="9"/>
       <x:c r="D170" s="9"/>
       <x:c r="E170" s="9"/>
+      <x:c r="F170" s="25"/>
+      <x:c r="G170" s="25"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="8"/>
@@ -1541,6 +1955,8 @@
       <x:c r="C171" s="9"/>
       <x:c r="D171" s="9"/>
       <x:c r="E171" s="9"/>
+      <x:c r="F171" s="29"/>
+      <x:c r="G171" s="29"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="8"/>
@@ -1548,6 +1964,8 @@
       <x:c r="C172" s="9"/>
       <x:c r="D172" s="9"/>
       <x:c r="E172" s="9"/>
+      <x:c r="F172" s="25"/>
+      <x:c r="G172" s="25"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="8"/>
@@ -1555,6 +1973,8 @@
       <x:c r="C173" s="9"/>
       <x:c r="D173" s="9"/>
       <x:c r="E173" s="9"/>
+      <x:c r="F173" s="29"/>
+      <x:c r="G173" s="29"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="8"/>
@@ -1562,6 +1982,8 @@
       <x:c r="C174" s="9"/>
       <x:c r="D174" s="9"/>
       <x:c r="E174" s="9"/>
+      <x:c r="F174" s="25"/>
+      <x:c r="G174" s="25"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="8"/>
@@ -1569,6 +1991,8 @@
       <x:c r="C175" s="9"/>
       <x:c r="D175" s="9"/>
       <x:c r="E175" s="9"/>
+      <x:c r="F175" s="29"/>
+      <x:c r="G175" s="29"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="8"/>
@@ -1576,6 +2000,8 @@
       <x:c r="C176" s="9"/>
       <x:c r="D176" s="9"/>
       <x:c r="E176" s="9"/>
+      <x:c r="F176" s="25"/>
+      <x:c r="G176" s="25"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="8"/>
@@ -1583,6 +2009,8 @@
       <x:c r="C177" s="9"/>
       <x:c r="D177" s="9"/>
       <x:c r="E177" s="9"/>
+      <x:c r="F177" s="29"/>
+      <x:c r="G177" s="29"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="8"/>
@@ -1590,6 +2018,8 @@
       <x:c r="C178" s="9"/>
       <x:c r="D178" s="9"/>
       <x:c r="E178" s="9"/>
+      <x:c r="F178" s="25"/>
+      <x:c r="G178" s="25"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="8"/>
@@ -1597,6 +2027,8 @@
       <x:c r="C179" s="9"/>
       <x:c r="D179" s="9"/>
       <x:c r="E179" s="9"/>
+      <x:c r="F179" s="29"/>
+      <x:c r="G179" s="29"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="8"/>
@@ -1604,6 +2036,8 @@
       <x:c r="C180" s="9"/>
       <x:c r="D180" s="9"/>
       <x:c r="E180" s="9"/>
+      <x:c r="F180" s="25"/>
+      <x:c r="G180" s="25"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="8"/>
@@ -1611,6 +2045,8 @@
       <x:c r="C181" s="9"/>
       <x:c r="D181" s="9"/>
       <x:c r="E181" s="9"/>
+      <x:c r="F181" s="29"/>
+      <x:c r="G181" s="29"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="8"/>
@@ -1618,6 +2054,8 @@
       <x:c r="C182" s="9"/>
       <x:c r="D182" s="9"/>
       <x:c r="E182" s="9"/>
+      <x:c r="F182" s="25"/>
+      <x:c r="G182" s="25"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="8"/>
@@ -1625,6 +2063,8 @@
       <x:c r="C183" s="9"/>
       <x:c r="D183" s="9"/>
       <x:c r="E183" s="9"/>
+      <x:c r="F183" s="29"/>
+      <x:c r="G183" s="29"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="8"/>
@@ -1632,6 +2072,8 @@
       <x:c r="C184" s="9"/>
       <x:c r="D184" s="9"/>
       <x:c r="E184" s="9"/>
+      <x:c r="F184" s="25"/>
+      <x:c r="G184" s="25"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="8"/>
@@ -1639,6 +2081,8 @@
       <x:c r="C185" s="9"/>
       <x:c r="D185" s="9"/>
       <x:c r="E185" s="9"/>
+      <x:c r="F185" s="29"/>
+      <x:c r="G185" s="29"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="8"/>
@@ -1646,6 +2090,8 @@
       <x:c r="C186" s="9"/>
       <x:c r="D186" s="9"/>
       <x:c r="E186" s="9"/>
+      <x:c r="F186" s="25"/>
+      <x:c r="G186" s="25"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="8"/>
@@ -1653,6 +2099,8 @@
       <x:c r="C187" s="9"/>
       <x:c r="D187" s="9"/>
       <x:c r="E187" s="9"/>
+      <x:c r="F187" s="29"/>
+      <x:c r="G187" s="29"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="8"/>
@@ -1660,6 +2108,8 @@
       <x:c r="C188" s="9"/>
       <x:c r="D188" s="9"/>
       <x:c r="E188" s="9"/>
+      <x:c r="F188" s="25"/>
+      <x:c r="G188" s="25"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="8"/>
@@ -1667,6 +2117,8 @@
       <x:c r="C189" s="9"/>
       <x:c r="D189" s="9"/>
       <x:c r="E189" s="9"/>
+      <x:c r="F189" s="29"/>
+      <x:c r="G189" s="29"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="8"/>
@@ -1674,6 +2126,8 @@
       <x:c r="C190" s="9"/>
       <x:c r="D190" s="9"/>
       <x:c r="E190" s="9"/>
+      <x:c r="F190" s="25"/>
+      <x:c r="G190" s="25"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="8"/>
@@ -1681,6 +2135,8 @@
       <x:c r="C191" s="9"/>
       <x:c r="D191" s="9"/>
       <x:c r="E191" s="9"/>
+      <x:c r="F191" s="29"/>
+      <x:c r="G191" s="29"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="8"/>
@@ -1688,6 +2144,8 @@
       <x:c r="C192" s="9"/>
       <x:c r="D192" s="9"/>
       <x:c r="E192" s="9"/>
+      <x:c r="F192" s="25"/>
+      <x:c r="G192" s="25"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="8"/>
@@ -1695,6 +2153,8 @@
       <x:c r="C193" s="9"/>
       <x:c r="D193" s="9"/>
       <x:c r="E193" s="9"/>
+      <x:c r="F193" s="29"/>
+      <x:c r="G193" s="29"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="8"/>
@@ -1702,6 +2162,8 @@
       <x:c r="C194" s="9"/>
       <x:c r="D194" s="9"/>
       <x:c r="E194" s="9"/>
+      <x:c r="F194" s="25"/>
+      <x:c r="G194" s="25"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="8"/>
@@ -1709,6 +2171,8 @@
       <x:c r="C195" s="9"/>
       <x:c r="D195" s="9"/>
       <x:c r="E195" s="9"/>
+      <x:c r="F195" s="29"/>
+      <x:c r="G195" s="29"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="8"/>
@@ -1716,6 +2180,8 @@
       <x:c r="C196" s="9"/>
       <x:c r="D196" s="9"/>
       <x:c r="E196" s="9"/>
+      <x:c r="F196" s="25"/>
+      <x:c r="G196" s="25"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="8"/>
@@ -1723,6 +2189,8 @@
       <x:c r="C197" s="9"/>
       <x:c r="D197" s="9"/>
       <x:c r="E197" s="9"/>
+      <x:c r="F197" s="29"/>
+      <x:c r="G197" s="29"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="8"/>
@@ -1730,6 +2198,8 @@
       <x:c r="C198" s="9"/>
       <x:c r="D198" s="9"/>
       <x:c r="E198" s="9"/>
+      <x:c r="F198" s="25"/>
+      <x:c r="G198" s="25"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="8"/>
@@ -1737,6 +2207,8 @@
       <x:c r="C199" s="9"/>
       <x:c r="D199" s="9"/>
       <x:c r="E199" s="9"/>
+      <x:c r="F199" s="29"/>
+      <x:c r="G199" s="29"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="8"/>
@@ -1744,6 +2216,8 @@
       <x:c r="C200" s="9"/>
       <x:c r="D200" s="9"/>
       <x:c r="E200" s="9"/>
+      <x:c r="F200" s="25"/>
+      <x:c r="G200" s="25"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="8"/>
@@ -1751,6 +2225,8 @@
       <x:c r="C201" s="9"/>
       <x:c r="D201" s="9"/>
       <x:c r="E201" s="9"/>
+      <x:c r="F201" s="29"/>
+      <x:c r="G201" s="29"/>
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="8"/>
@@ -1758,6 +2234,8 @@
       <x:c r="C202" s="9"/>
       <x:c r="D202" s="9"/>
       <x:c r="E202" s="9"/>
+      <x:c r="F202" s="25"/>
+      <x:c r="G202" s="25"/>
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="8"/>
@@ -1765,6 +2243,8 @@
       <x:c r="C203" s="9"/>
       <x:c r="D203" s="9"/>
       <x:c r="E203" s="9"/>
+      <x:c r="F203" s="29"/>
+      <x:c r="G203" s="29"/>
     </x:row>
     <x:row r="204">
       <x:c r="A204" s="8"/>
@@ -1772,6 +2252,8 @@
       <x:c r="C204" s="9"/>
       <x:c r="D204" s="9"/>
       <x:c r="E204" s="9"/>
+      <x:c r="F204" s="25"/>
+      <x:c r="G204" s="25"/>
     </x:row>
     <x:row r="205">
       <x:c r="A205" s="8"/>
@@ -1779,6 +2261,8 @@
       <x:c r="C205" s="9"/>
       <x:c r="D205" s="9"/>
       <x:c r="E205" s="9"/>
+      <x:c r="F205" s="29"/>
+      <x:c r="G205" s="29"/>
     </x:row>
     <x:row r="206">
       <x:c r="A206" s="8"/>
@@ -1786,6 +2270,8 @@
       <x:c r="C206" s="9"/>
       <x:c r="D206" s="9"/>
       <x:c r="E206" s="9"/>
+      <x:c r="F206" s="25"/>
+      <x:c r="G206" s="25"/>
     </x:row>
     <x:row r="207">
       <x:c r="A207" s="8"/>
@@ -1793,6 +2279,8 @@
       <x:c r="C207" s="9"/>
       <x:c r="D207" s="9"/>
       <x:c r="E207" s="9"/>
+      <x:c r="F207" s="29"/>
+      <x:c r="G207" s="29"/>
     </x:row>
     <x:row r="208">
       <x:c r="A208" s="8"/>
@@ -1800,6 +2288,8 @@
       <x:c r="C208" s="9"/>
       <x:c r="D208" s="9"/>
       <x:c r="E208" s="9"/>
+      <x:c r="F208" s="25"/>
+      <x:c r="G208" s="25"/>
     </x:row>
     <x:row r="209">
       <x:c r="A209" s="8"/>
@@ -1807,6 +2297,8 @@
       <x:c r="C209" s="9"/>
       <x:c r="D209" s="9"/>
       <x:c r="E209" s="9"/>
+      <x:c r="F209" s="29"/>
+      <x:c r="G209" s="29"/>
     </x:row>
     <x:row r="210">
       <x:c r="A210" s="8"/>
@@ -1814,6 +2306,8 @@
       <x:c r="C210" s="9"/>
       <x:c r="D210" s="9"/>
       <x:c r="E210" s="9"/>
+      <x:c r="F210" s="25"/>
+      <x:c r="G210" s="25"/>
     </x:row>
     <x:row r="211">
       <x:c r="A211" s="8"/>
@@ -1821,6 +2315,8 @@
       <x:c r="C211" s="9"/>
       <x:c r="D211" s="9"/>
       <x:c r="E211" s="9"/>
+      <x:c r="F211" s="29"/>
+      <x:c r="G211" s="29"/>
     </x:row>
     <x:row r="212">
       <x:c r="A212" s="8"/>
@@ -1828,6 +2324,8 @@
       <x:c r="C212" s="9"/>
       <x:c r="D212" s="9"/>
       <x:c r="E212" s="9"/>
+      <x:c r="F212" s="25"/>
+      <x:c r="G212" s="25"/>
     </x:row>
     <x:row r="213">
       <x:c r="A213" s="8"/>
@@ -1835,6 +2333,8 @@
       <x:c r="C213" s="9"/>
       <x:c r="D213" s="9"/>
       <x:c r="E213" s="9"/>
+      <x:c r="F213" s="29"/>
+      <x:c r="G213" s="29"/>
     </x:row>
     <x:row r="214">
       <x:c r="A214" s="8"/>
@@ -1842,6 +2342,8 @@
       <x:c r="C214" s="9"/>
       <x:c r="D214" s="9"/>
       <x:c r="E214" s="9"/>
+      <x:c r="F214" s="25"/>
+      <x:c r="G214" s="25"/>
     </x:row>
     <x:row r="215">
       <x:c r="A215" s="8"/>
@@ -1849,6 +2351,8 @@
       <x:c r="C215" s="9"/>
       <x:c r="D215" s="9"/>
       <x:c r="E215" s="9"/>
+      <x:c r="F215" s="29"/>
+      <x:c r="G215" s="29"/>
     </x:row>
     <x:row r="216">
       <x:c r="A216" s="8"/>
@@ -1856,6 +2360,8 @@
       <x:c r="C216" s="9"/>
       <x:c r="D216" s="9"/>
       <x:c r="E216" s="9"/>
+      <x:c r="F216" s="25"/>
+      <x:c r="G216" s="25"/>
     </x:row>
     <x:row r="217">
       <x:c r="A217" s="8"/>
@@ -1863,6 +2369,8 @@
       <x:c r="C217" s="9"/>
       <x:c r="D217" s="9"/>
       <x:c r="E217" s="9"/>
+      <x:c r="F217" s="29"/>
+      <x:c r="G217" s="29"/>
     </x:row>
     <x:row r="218">
       <x:c r="A218" s="8"/>
@@ -1870,6 +2378,8 @@
       <x:c r="C218" s="9"/>
       <x:c r="D218" s="9"/>
       <x:c r="E218" s="9"/>
+      <x:c r="F218" s="25"/>
+      <x:c r="G218" s="25"/>
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="8"/>
@@ -1877,6 +2387,8 @@
       <x:c r="C219" s="9"/>
       <x:c r="D219" s="9"/>
       <x:c r="E219" s="9"/>
+      <x:c r="F219" s="29"/>
+      <x:c r="G219" s="29"/>
     </x:row>
     <x:row r="220">
       <x:c r="A220" s="8"/>
@@ -1884,6 +2396,8 @@
       <x:c r="C220" s="9"/>
       <x:c r="D220" s="9"/>
       <x:c r="E220" s="9"/>
+      <x:c r="F220" s="25"/>
+      <x:c r="G220" s="25"/>
     </x:row>
     <x:row r="221">
       <x:c r="A221" s="8"/>
@@ -1891,6 +2405,8 @@
       <x:c r="C221" s="9"/>
       <x:c r="D221" s="9"/>
       <x:c r="E221" s="9"/>
+      <x:c r="F221" s="29"/>
+      <x:c r="G221" s="29"/>
     </x:row>
     <x:row r="222">
       <x:c r="A222" s="8"/>
@@ -1898,6 +2414,8 @@
       <x:c r="C222" s="9"/>
       <x:c r="D222" s="9"/>
       <x:c r="E222" s="9"/>
+      <x:c r="F222" s="25"/>
+      <x:c r="G222" s="25"/>
     </x:row>
     <x:row r="223">
       <x:c r="A223" s="8"/>
@@ -1905,6 +2423,8 @@
       <x:c r="C223" s="9"/>
       <x:c r="D223" s="9"/>
       <x:c r="E223" s="9"/>
+      <x:c r="F223" s="29"/>
+      <x:c r="G223" s="29"/>
     </x:row>
     <x:row r="224">
       <x:c r="A224" s="8"/>
@@ -1912,6 +2432,8 @@
       <x:c r="C224" s="9"/>
       <x:c r="D224" s="9"/>
       <x:c r="E224" s="9"/>
+      <x:c r="F224" s="25"/>
+      <x:c r="G224" s="25"/>
     </x:row>
     <x:row r="225">
       <x:c r="A225" s="8"/>
@@ -1919,6 +2441,8 @@
       <x:c r="C225" s="9"/>
       <x:c r="D225" s="9"/>
       <x:c r="E225" s="9"/>
+      <x:c r="F225" s="29"/>
+      <x:c r="G225" s="29"/>
     </x:row>
     <x:row r="226">
       <x:c r="A226" s="8"/>
@@ -1926,6 +2450,8 @@
       <x:c r="C226" s="9"/>
       <x:c r="D226" s="9"/>
       <x:c r="E226" s="9"/>
+      <x:c r="F226" s="25"/>
+      <x:c r="G226" s="25"/>
     </x:row>
     <x:row r="227">
       <x:c r="A227" s="8"/>
@@ -1933,6 +2459,8 @@
       <x:c r="C227" s="9"/>
       <x:c r="D227" s="9"/>
       <x:c r="E227" s="9"/>
+      <x:c r="F227" s="29"/>
+      <x:c r="G227" s="29"/>
     </x:row>
     <x:row r="228">
       <x:c r="A228" s="8"/>
@@ -1940,6 +2468,8 @@
       <x:c r="C228" s="9"/>
       <x:c r="D228" s="9"/>
       <x:c r="E228" s="9"/>
+      <x:c r="F228" s="25"/>
+      <x:c r="G228" s="25"/>
     </x:row>
     <x:row r="229">
       <x:c r="A229" s="8"/>
@@ -1947,6 +2477,8 @@
       <x:c r="C229" s="9"/>
       <x:c r="D229" s="9"/>
       <x:c r="E229" s="9"/>
+      <x:c r="F229" s="29"/>
+      <x:c r="G229" s="29"/>
     </x:row>
     <x:row r="230">
       <x:c r="A230" s="8"/>
@@ -1954,6 +2486,8 @@
       <x:c r="C230" s="9"/>
       <x:c r="D230" s="9"/>
       <x:c r="E230" s="9"/>
+      <x:c r="F230" s="25"/>
+      <x:c r="G230" s="25"/>
     </x:row>
     <x:row r="231">
       <x:c r="A231" s="8"/>
@@ -1961,6 +2495,8 @@
       <x:c r="C231" s="9"/>
       <x:c r="D231" s="9"/>
       <x:c r="E231" s="9"/>
+      <x:c r="F231" s="29"/>
+      <x:c r="G231" s="29"/>
     </x:row>
     <x:row r="232">
       <x:c r="A232" s="8"/>
@@ -1968,6 +2504,8 @@
       <x:c r="C232" s="9"/>
       <x:c r="D232" s="9"/>
       <x:c r="E232" s="9"/>
+      <x:c r="F232" s="25"/>
+      <x:c r="G232" s="25"/>
     </x:row>
     <x:row r="233">
       <x:c r="A233" s="8"/>
@@ -1975,6 +2513,8 @@
       <x:c r="C233" s="9"/>
       <x:c r="D233" s="9"/>
       <x:c r="E233" s="9"/>
+      <x:c r="F233" s="29"/>
+      <x:c r="G233" s="29"/>
     </x:row>
     <x:row r="234">
       <x:c r="A234" s="8"/>
@@ -1982,6 +2522,8 @@
       <x:c r="C234" s="9"/>
       <x:c r="D234" s="9"/>
       <x:c r="E234" s="9"/>
+      <x:c r="F234" s="25"/>
+      <x:c r="G234" s="25"/>
     </x:row>
     <x:row r="235">
       <x:c r="A235" s="8"/>
@@ -1989,6 +2531,8 @@
       <x:c r="C235" s="9"/>
       <x:c r="D235" s="9"/>
       <x:c r="E235" s="9"/>
+      <x:c r="F235" s="29"/>
+      <x:c r="G235" s="29"/>
     </x:row>
     <x:row r="236">
       <x:c r="A236" s="8"/>
@@ -1996,6 +2540,8 @@
       <x:c r="C236" s="9"/>
       <x:c r="D236" s="9"/>
       <x:c r="E236" s="9"/>
+      <x:c r="F236" s="25"/>
+      <x:c r="G236" s="25"/>
     </x:row>
     <x:row r="237">
       <x:c r="A237" s="8"/>
@@ -2003,6 +2549,8 @@
       <x:c r="C237" s="9"/>
       <x:c r="D237" s="9"/>
       <x:c r="E237" s="9"/>
+      <x:c r="F237" s="29"/>
+      <x:c r="G237" s="29"/>
     </x:row>
     <x:row r="238">
       <x:c r="A238" s="8"/>
@@ -2010,6 +2558,8 @@
       <x:c r="C238" s="9"/>
       <x:c r="D238" s="9"/>
       <x:c r="E238" s="9"/>
+      <x:c r="F238" s="25"/>
+      <x:c r="G238" s="25"/>
     </x:row>
     <x:row r="239">
       <x:c r="A239" s="8"/>
@@ -2017,6 +2567,8 @@
       <x:c r="C239" s="9"/>
       <x:c r="D239" s="9"/>
       <x:c r="E239" s="9"/>
+      <x:c r="F239" s="29"/>
+      <x:c r="G239" s="29"/>
     </x:row>
     <x:row r="240">
       <x:c r="A240" s="8"/>
@@ -2024,6 +2576,8 @@
       <x:c r="C240" s="9"/>
       <x:c r="D240" s="9"/>
       <x:c r="E240" s="9"/>
+      <x:c r="F240" s="25"/>
+      <x:c r="G240" s="25"/>
     </x:row>
     <x:row r="241">
       <x:c r="A241" s="8"/>
@@ -2031,6 +2585,8 @@
       <x:c r="C241" s="9"/>
       <x:c r="D241" s="9"/>
       <x:c r="E241" s="9"/>
+      <x:c r="F241" s="29"/>
+      <x:c r="G241" s="29"/>
     </x:row>
     <x:row r="242">
       <x:c r="A242" s="8"/>
@@ -2038,6 +2594,8 @@
       <x:c r="C242" s="9"/>
       <x:c r="D242" s="9"/>
       <x:c r="E242" s="9"/>
+      <x:c r="F242" s="25"/>
+      <x:c r="G242" s="25"/>
     </x:row>
     <x:row r="243">
       <x:c r="A243" s="8"/>
@@ -2045,6 +2603,8 @@
       <x:c r="C243" s="9"/>
       <x:c r="D243" s="9"/>
       <x:c r="E243" s="9"/>
+      <x:c r="F243" s="29"/>
+      <x:c r="G243" s="29"/>
     </x:row>
     <x:row r="244">
       <x:c r="A244" s="8"/>
@@ -2052,6 +2612,8 @@
       <x:c r="C244" s="9"/>
       <x:c r="D244" s="9"/>
       <x:c r="E244" s="9"/>
+      <x:c r="F244" s="25"/>
+      <x:c r="G244" s="25"/>
     </x:row>
     <x:row r="245">
       <x:c r="A245" s="8"/>
@@ -2059,6 +2621,8 @@
       <x:c r="C245" s="9"/>
       <x:c r="D245" s="9"/>
       <x:c r="E245" s="9"/>
+      <x:c r="F245" s="29"/>
+      <x:c r="G245" s="29"/>
     </x:row>
     <x:row r="246">
       <x:c r="A246" s="8"/>
@@ -2066,6 +2630,8 @@
       <x:c r="C246" s="9"/>
       <x:c r="D246" s="9"/>
       <x:c r="E246" s="9"/>
+      <x:c r="F246" s="25"/>
+      <x:c r="G246" s="25"/>
     </x:row>
     <x:row r="247">
       <x:c r="A247" s="8"/>
@@ -2073,6 +2639,8 @@
       <x:c r="C247" s="9"/>
       <x:c r="D247" s="9"/>
       <x:c r="E247" s="9"/>
+      <x:c r="F247" s="29"/>
+      <x:c r="G247" s="29"/>
     </x:row>
     <x:row r="248">
       <x:c r="A248" s="8"/>
@@ -2080,6 +2648,8 @@
       <x:c r="C248" s="9"/>
       <x:c r="D248" s="9"/>
       <x:c r="E248" s="9"/>
+      <x:c r="F248" s="25"/>
+      <x:c r="G248" s="25"/>
     </x:row>
     <x:row r="249">
       <x:c r="A249" s="8"/>
@@ -2087,6 +2657,8 @@
       <x:c r="C249" s="9"/>
       <x:c r="D249" s="9"/>
       <x:c r="E249" s="9"/>
+      <x:c r="F249" s="29"/>
+      <x:c r="G249" s="29"/>
     </x:row>
     <x:row r="250">
       <x:c r="A250" s="8"/>
@@ -2094,6 +2666,8 @@
       <x:c r="C250" s="9"/>
       <x:c r="D250" s="9"/>
       <x:c r="E250" s="9"/>
+      <x:c r="F250" s="25"/>
+      <x:c r="G250" s="25"/>
     </x:row>
     <x:row r="251">
       <x:c r="A251" s="8"/>
@@ -2101,6 +2675,8 @@
       <x:c r="C251" s="9"/>
       <x:c r="D251" s="9"/>
       <x:c r="E251" s="9"/>
+      <x:c r="F251" s="29"/>
+      <x:c r="G251" s="29"/>
     </x:row>
     <x:row r="252">
       <x:c r="A252" s="8"/>
@@ -2108,6 +2684,8 @@
       <x:c r="C252" s="9"/>
       <x:c r="D252" s="9"/>
       <x:c r="E252" s="9"/>
+      <x:c r="F252" s="25"/>
+      <x:c r="G252" s="25"/>
     </x:row>
     <x:row r="253">
       <x:c r="A253" s="8"/>
@@ -2115,6 +2693,8 @@
       <x:c r="C253" s="9"/>
       <x:c r="D253" s="9"/>
       <x:c r="E253" s="9"/>
+      <x:c r="F253" s="29"/>
+      <x:c r="G253" s="29"/>
     </x:row>
     <x:row r="254">
       <x:c r="A254" s="8"/>
@@ -2122,6 +2702,8 @@
       <x:c r="C254" s="9"/>
       <x:c r="D254" s="9"/>
       <x:c r="E254" s="9"/>
+      <x:c r="F254" s="25"/>
+      <x:c r="G254" s="25"/>
     </x:row>
     <x:row r="255">
       <x:c r="A255" s="8"/>
@@ -2129,6 +2711,8 @@
       <x:c r="C255" s="9"/>
       <x:c r="D255" s="9"/>
       <x:c r="E255" s="9"/>
+      <x:c r="F255" s="29"/>
+      <x:c r="G255" s="29"/>
     </x:row>
     <x:row r="256">
       <x:c r="A256" s="8"/>
@@ -2136,6 +2720,8 @@
       <x:c r="C256" s="9"/>
       <x:c r="D256" s="9"/>
       <x:c r="E256" s="9"/>
+      <x:c r="F256" s="25"/>
+      <x:c r="G256" s="25"/>
     </x:row>
     <x:row r="257">
       <x:c r="A257" s="8"/>
@@ -2143,6 +2729,8 @@
       <x:c r="C257" s="9"/>
       <x:c r="D257" s="9"/>
       <x:c r="E257" s="9"/>
+      <x:c r="F257" s="29"/>
+      <x:c r="G257" s="29"/>
     </x:row>
     <x:row r="258">
       <x:c r="A258" s="8"/>
@@ -2150,6 +2738,8 @@
       <x:c r="C258" s="9"/>
       <x:c r="D258" s="9"/>
       <x:c r="E258" s="9"/>
+      <x:c r="F258" s="25"/>
+      <x:c r="G258" s="25"/>
     </x:row>
     <x:row r="259">
       <x:c r="A259" s="8"/>
@@ -2157,6 +2747,8 @@
       <x:c r="C259" s="9"/>
       <x:c r="D259" s="9"/>
       <x:c r="E259" s="9"/>
+      <x:c r="F259" s="29"/>
+      <x:c r="G259" s="29"/>
     </x:row>
     <x:row r="260">
       <x:c r="A260" s="8"/>
@@ -2164,6 +2756,8 @@
       <x:c r="C260" s="9"/>
       <x:c r="D260" s="9"/>
       <x:c r="E260" s="9"/>
+      <x:c r="F260" s="25"/>
+      <x:c r="G260" s="25"/>
     </x:row>
     <x:row r="261">
       <x:c r="A261" s="8"/>
@@ -2171,6 +2765,8 @@
       <x:c r="C261" s="9"/>
       <x:c r="D261" s="9"/>
       <x:c r="E261" s="9"/>
+      <x:c r="F261" s="29"/>
+      <x:c r="G261" s="29"/>
     </x:row>
     <x:row r="262">
       <x:c r="A262" s="8"/>
@@ -2178,6 +2774,8 @@
       <x:c r="C262" s="9"/>
       <x:c r="D262" s="9"/>
       <x:c r="E262" s="9"/>
+      <x:c r="F262" s="25"/>
+      <x:c r="G262" s="25"/>
     </x:row>
     <x:row r="263">
       <x:c r="A263" s="8"/>
@@ -2185,6 +2783,8 @@
       <x:c r="C263" s="9"/>
       <x:c r="D263" s="9"/>
       <x:c r="E263" s="9"/>
+      <x:c r="F263" s="29"/>
+      <x:c r="G263" s="29"/>
     </x:row>
     <x:row r="264">
       <x:c r="A264" s="8"/>
@@ -2192,6 +2792,8 @@
       <x:c r="C264" s="9"/>
       <x:c r="D264" s="9"/>
       <x:c r="E264" s="9"/>
+      <x:c r="F264" s="25"/>
+      <x:c r="G264" s="25"/>
     </x:row>
     <x:row r="265">
       <x:c r="A265" s="8"/>
@@ -2199,6 +2801,8 @@
       <x:c r="C265" s="9"/>
       <x:c r="D265" s="9"/>
       <x:c r="E265" s="9"/>
+      <x:c r="F265" s="29"/>
+      <x:c r="G265" s="29"/>
     </x:row>
     <x:row r="266">
       <x:c r="A266" s="8"/>
@@ -2206,6 +2810,8 @@
       <x:c r="C266" s="9"/>
       <x:c r="D266" s="9"/>
       <x:c r="E266" s="9"/>
+      <x:c r="F266" s="25"/>
+      <x:c r="G266" s="25"/>
     </x:row>
     <x:row r="267">
       <x:c r="A267" s="8"/>
@@ -2213,6 +2819,8 @@
       <x:c r="C267" s="9"/>
       <x:c r="D267" s="9"/>
       <x:c r="E267" s="9"/>
+      <x:c r="F267" s="29"/>
+      <x:c r="G267" s="29"/>
     </x:row>
     <x:row r="268">
       <x:c r="A268" s="8"/>
@@ -2220,6 +2828,8 @@
       <x:c r="C268" s="9"/>
       <x:c r="D268" s="9"/>
       <x:c r="E268" s="9"/>
+      <x:c r="F268" s="25"/>
+      <x:c r="G268" s="25"/>
     </x:row>
     <x:row r="269">
       <x:c r="A269" s="8"/>
@@ -2227,6 +2837,8 @@
       <x:c r="C269" s="9"/>
       <x:c r="D269" s="9"/>
       <x:c r="E269" s="9"/>
+      <x:c r="F269" s="29"/>
+      <x:c r="G269" s="29"/>
     </x:row>
     <x:row r="270">
       <x:c r="A270" s="8"/>
@@ -2234,6 +2846,8 @@
       <x:c r="C270" s="9"/>
       <x:c r="D270" s="9"/>
       <x:c r="E270" s="9"/>
+      <x:c r="F270" s="25"/>
+      <x:c r="G270" s="25"/>
     </x:row>
     <x:row r="271">
       <x:c r="A271" s="8"/>
@@ -2241,6 +2855,8 @@
       <x:c r="C271" s="9"/>
       <x:c r="D271" s="9"/>
       <x:c r="E271" s="9"/>
+      <x:c r="F271" s="29"/>
+      <x:c r="G271" s="29"/>
     </x:row>
     <x:row r="272">
       <x:c r="A272" s="8"/>
@@ -2248,6 +2864,8 @@
       <x:c r="C272" s="9"/>
       <x:c r="D272" s="9"/>
       <x:c r="E272" s="9"/>
+      <x:c r="F272" s="25"/>
+      <x:c r="G272" s="25"/>
     </x:row>
     <x:row r="273">
       <x:c r="A273" s="8"/>
@@ -2255,6 +2873,8 @@
       <x:c r="C273" s="9"/>
       <x:c r="D273" s="9"/>
       <x:c r="E273" s="9"/>
+      <x:c r="F273" s="29"/>
+      <x:c r="G273" s="29"/>
     </x:row>
     <x:row r="274">
       <x:c r="A274" s="8"/>
@@ -2262,6 +2882,8 @@
       <x:c r="C274" s="9"/>
       <x:c r="D274" s="9"/>
       <x:c r="E274" s="9"/>
+      <x:c r="F274" s="25"/>
+      <x:c r="G274" s="25"/>
     </x:row>
     <x:row r="275">
       <x:c r="A275" s="8"/>
@@ -2269,6 +2891,8 @@
       <x:c r="C275" s="9"/>
       <x:c r="D275" s="9"/>
       <x:c r="E275" s="9"/>
+      <x:c r="F275" s="29"/>
+      <x:c r="G275" s="29"/>
     </x:row>
     <x:row r="276">
       <x:c r="A276" s="8"/>
@@ -2276,6 +2900,8 @@
       <x:c r="C276" s="9"/>
       <x:c r="D276" s="9"/>
       <x:c r="E276" s="9"/>
+      <x:c r="F276" s="25"/>
+      <x:c r="G276" s="25"/>
     </x:row>
     <x:row r="277">
       <x:c r="A277" s="8"/>
@@ -2283,6 +2909,8 @@
       <x:c r="C277" s="9"/>
       <x:c r="D277" s="9"/>
       <x:c r="E277" s="9"/>
+      <x:c r="F277" s="29"/>
+      <x:c r="G277" s="29"/>
     </x:row>
     <x:row r="278">
       <x:c r="A278" s="8"/>
@@ -2290,6 +2918,8 @@
       <x:c r="C278" s="9"/>
       <x:c r="D278" s="9"/>
       <x:c r="E278" s="9"/>
+      <x:c r="F278" s="25"/>
+      <x:c r="G278" s="25"/>
     </x:row>
     <x:row r="279">
       <x:c r="A279" s="8"/>
@@ -2297,6 +2927,8 @@
       <x:c r="C279" s="9"/>
       <x:c r="D279" s="9"/>
       <x:c r="E279" s="9"/>
+      <x:c r="F279" s="29"/>
+      <x:c r="G279" s="29"/>
     </x:row>
     <x:row r="280">
       <x:c r="A280" s="8"/>
@@ -2304,6 +2936,8 @@
       <x:c r="C280" s="9"/>
       <x:c r="D280" s="9"/>
       <x:c r="E280" s="9"/>
+      <x:c r="F280" s="25"/>
+      <x:c r="G280" s="25"/>
     </x:row>
     <x:row r="281">
       <x:c r="A281" s="8"/>
@@ -2311,6 +2945,8 @@
       <x:c r="C281" s="9"/>
       <x:c r="D281" s="9"/>
       <x:c r="E281" s="9"/>
+      <x:c r="F281" s="29"/>
+      <x:c r="G281" s="29"/>
     </x:row>
     <x:row r="282">
       <x:c r="A282" s="8"/>
@@ -2318,6 +2954,8 @@
       <x:c r="C282" s="9"/>
       <x:c r="D282" s="9"/>
       <x:c r="E282" s="9"/>
+      <x:c r="F282" s="25"/>
+      <x:c r="G282" s="25"/>
     </x:row>
     <x:row r="283">
       <x:c r="A283" s="8"/>
@@ -2325,6 +2963,8 @@
       <x:c r="C283" s="9"/>
       <x:c r="D283" s="9"/>
       <x:c r="E283" s="9"/>
+      <x:c r="F283" s="29"/>
+      <x:c r="G283" s="29"/>
     </x:row>
     <x:row r="284">
       <x:c r="A284" s="8"/>
@@ -2332,6 +2972,8 @@
       <x:c r="C284" s="9"/>
       <x:c r="D284" s="9"/>
       <x:c r="E284" s="9"/>
+      <x:c r="F284" s="25"/>
+      <x:c r="G284" s="25"/>
     </x:row>
     <x:row r="285">
       <x:c r="A285" s="8"/>
@@ -2339,6 +2981,8 @@
       <x:c r="C285" s="9"/>
       <x:c r="D285" s="9"/>
       <x:c r="E285" s="9"/>
+      <x:c r="F285" s="29"/>
+      <x:c r="G285" s="29"/>
     </x:row>
     <x:row r="286">
       <x:c r="A286" s="8"/>
@@ -2346,6 +2990,8 @@
       <x:c r="C286" s="9"/>
       <x:c r="D286" s="9"/>
       <x:c r="E286" s="9"/>
+      <x:c r="F286" s="25"/>
+      <x:c r="G286" s="25"/>
     </x:row>
     <x:row r="287">
       <x:c r="A287" s="8"/>
@@ -2353,6 +2999,8 @@
       <x:c r="C287" s="9"/>
       <x:c r="D287" s="9"/>
       <x:c r="E287" s="9"/>
+      <x:c r="F287" s="29"/>
+      <x:c r="G287" s="29"/>
     </x:row>
     <x:row r="288">
       <x:c r="A288" s="8"/>
@@ -2360,6 +3008,8 @@
       <x:c r="C288" s="9"/>
       <x:c r="D288" s="9"/>
       <x:c r="E288" s="9"/>
+      <x:c r="F288" s="25"/>
+      <x:c r="G288" s="25"/>
     </x:row>
     <x:row r="289">
       <x:c r="A289" s="8"/>
@@ -2367,6 +3017,8 @@
       <x:c r="C289" s="9"/>
       <x:c r="D289" s="9"/>
       <x:c r="E289" s="9"/>
+      <x:c r="F289" s="29"/>
+      <x:c r="G289" s="29"/>
     </x:row>
     <x:row r="290">
       <x:c r="A290" s="8"/>
@@ -2374,6 +3026,8 @@
       <x:c r="C290" s="9"/>
       <x:c r="D290" s="9"/>
       <x:c r="E290" s="9"/>
+      <x:c r="F290" s="25"/>
+      <x:c r="G290" s="25"/>
     </x:row>
     <x:row r="291">
       <x:c r="A291" s="8"/>
@@ -2381,6 +3035,8 @@
       <x:c r="C291" s="9"/>
       <x:c r="D291" s="9"/>
       <x:c r="E291" s="9"/>
+      <x:c r="F291" s="29"/>
+      <x:c r="G291" s="29"/>
     </x:row>
     <x:row r="292">
       <x:c r="A292" s="8"/>
@@ -2388,6 +3044,8 @@
       <x:c r="C292" s="9"/>
       <x:c r="D292" s="9"/>
       <x:c r="E292" s="9"/>
+      <x:c r="F292" s="25"/>
+      <x:c r="G292" s="25"/>
     </x:row>
     <x:row r="293">
       <x:c r="A293" s="8"/>
@@ -2395,6 +3053,8 @@
       <x:c r="C293" s="9"/>
       <x:c r="D293" s="9"/>
       <x:c r="E293" s="9"/>
+      <x:c r="F293" s="29"/>
+      <x:c r="G293" s="29"/>
     </x:row>
     <x:row r="294">
       <x:c r="A294" s="8"/>
@@ -2402,6 +3062,8 @@
       <x:c r="C294" s="9"/>
       <x:c r="D294" s="9"/>
       <x:c r="E294" s="9"/>
+      <x:c r="F294" s="25"/>
+      <x:c r="G294" s="25"/>
     </x:row>
     <x:row r="295">
       <x:c r="A295" s="8"/>
@@ -2409,6 +3071,8 @@
       <x:c r="C295" s="9"/>
       <x:c r="D295" s="9"/>
       <x:c r="E295" s="9"/>
+      <x:c r="F295" s="29"/>
+      <x:c r="G295" s="29"/>
     </x:row>
     <x:row r="296">
       <x:c r="A296" s="8"/>
@@ -2416,6 +3080,8 @@
       <x:c r="C296" s="9"/>
       <x:c r="D296" s="9"/>
       <x:c r="E296" s="9"/>
+      <x:c r="F296" s="25"/>
+      <x:c r="G296" s="25"/>
     </x:row>
     <x:row r="297">
       <x:c r="A297" s="8"/>
@@ -2423,6 +3089,8 @@
       <x:c r="C297" s="9"/>
       <x:c r="D297" s="9"/>
       <x:c r="E297" s="9"/>
+      <x:c r="F297" s="29"/>
+      <x:c r="G297" s="29"/>
     </x:row>
     <x:row r="298">
       <x:c r="A298" s="8"/>
@@ -2430,6 +3098,8 @@
       <x:c r="C298" s="9"/>
       <x:c r="D298" s="9"/>
       <x:c r="E298" s="9"/>
+      <x:c r="F298" s="25"/>
+      <x:c r="G298" s="25"/>
     </x:row>
     <x:row r="299">
       <x:c r="A299" s="8"/>
@@ -2437,6 +3107,8 @@
       <x:c r="C299" s="9"/>
       <x:c r="D299" s="9"/>
       <x:c r="E299" s="9"/>
+      <x:c r="F299" s="29"/>
+      <x:c r="G299" s="29"/>
     </x:row>
     <x:row r="300">
       <x:c r="A300" s="8"/>
@@ -2444,6 +3116,8 @@
       <x:c r="C300" s="9"/>
       <x:c r="D300" s="9"/>
       <x:c r="E300" s="9"/>
+      <x:c r="F300" s="25"/>
+      <x:c r="G300" s="25"/>
     </x:row>
     <x:row r="301">
       <x:c r="A301" s="8"/>
@@ -2451,6 +3125,8 @@
       <x:c r="C301" s="9"/>
       <x:c r="D301" s="9"/>
       <x:c r="E301" s="9"/>
+      <x:c r="F301" s="29"/>
+      <x:c r="G301" s="29"/>
     </x:row>
     <x:row r="302">
       <x:c r="A302" s="8"/>
@@ -2458,6 +3134,8 @@
       <x:c r="C302" s="9"/>
       <x:c r="D302" s="9"/>
       <x:c r="E302" s="9"/>
+      <x:c r="F302" s="25"/>
+      <x:c r="G302" s="25"/>
     </x:row>
     <x:row r="303">
       <x:c r="A303" s="8"/>
@@ -2465,6 +3143,8 @@
       <x:c r="C303" s="9"/>
       <x:c r="D303" s="9"/>
       <x:c r="E303" s="9"/>
+      <x:c r="F303" s="29"/>
+      <x:c r="G303" s="29"/>
     </x:row>
     <x:row r="304">
       <x:c r="A304" s="8"/>
@@ -2472,6 +3152,8 @@
       <x:c r="C304" s="9"/>
       <x:c r="D304" s="9"/>
       <x:c r="E304" s="9"/>
+      <x:c r="F304" s="25"/>
+      <x:c r="G304" s="25"/>
     </x:row>
     <x:row r="305">
       <x:c r="A305" s="8"/>
@@ -2479,6 +3161,8 @@
       <x:c r="C305" s="9"/>
       <x:c r="D305" s="9"/>
       <x:c r="E305" s="9"/>
+      <x:c r="F305" s="29"/>
+      <x:c r="G305" s="29"/>
     </x:row>
     <x:row r="306">
       <x:c r="A306" s="8"/>
@@ -2486,6 +3170,8 @@
       <x:c r="C306" s="9"/>
       <x:c r="D306" s="9"/>
       <x:c r="E306" s="9"/>
+      <x:c r="F306" s="25"/>
+      <x:c r="G306" s="25"/>
     </x:row>
     <x:row r="307">
       <x:c r="A307" s="8"/>
@@ -2493,6 +3179,8 @@
       <x:c r="C307" s="9"/>
       <x:c r="D307" s="9"/>
       <x:c r="E307" s="9"/>
+      <x:c r="F307" s="29"/>
+      <x:c r="G307" s="29"/>
     </x:row>
     <x:row r="308">
       <x:c r="A308" s="8"/>
@@ -2500,6 +3188,8 @@
       <x:c r="C308" s="9"/>
       <x:c r="D308" s="9"/>
       <x:c r="E308" s="9"/>
+      <x:c r="F308" s="25"/>
+      <x:c r="G308" s="25"/>
     </x:row>
     <x:row r="309">
       <x:c r="A309" s="8"/>
@@ -2507,6 +3197,8 @@
       <x:c r="C309" s="9"/>
       <x:c r="D309" s="9"/>
       <x:c r="E309" s="9"/>
+      <x:c r="F309" s="29"/>
+      <x:c r="G309" s="29"/>
     </x:row>
     <x:row r="310">
       <x:c r="A310" s="8"/>
@@ -2514,6 +3206,8 @@
       <x:c r="C310" s="9"/>
       <x:c r="D310" s="9"/>
       <x:c r="E310" s="9"/>
+      <x:c r="F310" s="25"/>
+      <x:c r="G310" s="25"/>
     </x:row>
     <x:row r="311">
       <x:c r="A311" s="8"/>
@@ -2521,6 +3215,8 @@
       <x:c r="C311" s="9"/>
       <x:c r="D311" s="9"/>
       <x:c r="E311" s="9"/>
+      <x:c r="F311" s="29"/>
+      <x:c r="G311" s="29"/>
     </x:row>
     <x:row r="312">
       <x:c r="A312" s="8"/>
@@ -2528,6 +3224,8 @@
       <x:c r="C312" s="9"/>
       <x:c r="D312" s="9"/>
       <x:c r="E312" s="9"/>
+      <x:c r="F312" s="25"/>
+      <x:c r="G312" s="25"/>
     </x:row>
     <x:row r="313">
       <x:c r="A313" s="8"/>
@@ -2535,6 +3233,8 @@
       <x:c r="C313" s="9"/>
       <x:c r="D313" s="9"/>
       <x:c r="E313" s="9"/>
+      <x:c r="F313" s="29"/>
+      <x:c r="G313" s="29"/>
     </x:row>
     <x:row r="314">
       <x:c r="A314" s="8"/>
@@ -2542,6 +3242,8 @@
       <x:c r="C314" s="9"/>
       <x:c r="D314" s="9"/>
       <x:c r="E314" s="9"/>
+      <x:c r="F314" s="25"/>
+      <x:c r="G314" s="25"/>
     </x:row>
     <x:row r="315">
       <x:c r="A315" s="8"/>
@@ -2549,6 +3251,8 @@
       <x:c r="C315" s="9"/>
       <x:c r="D315" s="9"/>
       <x:c r="E315" s="9"/>
+      <x:c r="F315" s="29"/>
+      <x:c r="G315" s="29"/>
     </x:row>
     <x:row r="316">
       <x:c r="A316" s="8"/>
@@ -2556,6 +3260,8 @@
       <x:c r="C316" s="9"/>
       <x:c r="D316" s="9"/>
       <x:c r="E316" s="9"/>
+      <x:c r="F316" s="25"/>
+      <x:c r="G316" s="25"/>
     </x:row>
     <x:row r="317">
       <x:c r="A317" s="8"/>
@@ -2563,6 +3269,8 @@
       <x:c r="C317" s="9"/>
       <x:c r="D317" s="9"/>
       <x:c r="E317" s="9"/>
+      <x:c r="F317" s="29"/>
+      <x:c r="G317" s="29"/>
     </x:row>
     <x:row r="318">
       <x:c r="A318" s="8"/>
@@ -2570,6 +3278,8 @@
       <x:c r="C318" s="9"/>
       <x:c r="D318" s="9"/>
       <x:c r="E318" s="9"/>
+      <x:c r="F318" s="25"/>
+      <x:c r="G318" s="25"/>
     </x:row>
     <x:row r="319">
       <x:c r="A319" s="8"/>
@@ -2577,6 +3287,8 @@
       <x:c r="C319" s="9"/>
       <x:c r="D319" s="9"/>
       <x:c r="E319" s="9"/>
+      <x:c r="F319" s="29"/>
+      <x:c r="G319" s="29"/>
     </x:row>
     <x:row r="320">
       <x:c r="A320" s="8"/>
@@ -2584,6 +3296,8 @@
       <x:c r="C320" s="9"/>
       <x:c r="D320" s="9"/>
       <x:c r="E320" s="9"/>
+      <x:c r="F320" s="25"/>
+      <x:c r="G320" s="25"/>
     </x:row>
     <x:row r="321">
       <x:c r="A321" s="8"/>
@@ -2591,6 +3305,8 @@
       <x:c r="C321" s="9"/>
       <x:c r="D321" s="9"/>
       <x:c r="E321" s="9"/>
+      <x:c r="F321" s="29"/>
+      <x:c r="G321" s="29"/>
     </x:row>
     <x:row r="322">
       <x:c r="A322" s="8"/>
@@ -2598,6 +3314,8 @@
       <x:c r="C322" s="9"/>
       <x:c r="D322" s="9"/>
       <x:c r="E322" s="9"/>
+      <x:c r="F322" s="25"/>
+      <x:c r="G322" s="25"/>
     </x:row>
     <x:row r="323">
       <x:c r="A323" s="8"/>
@@ -2605,6 +3323,8 @@
       <x:c r="C323" s="9"/>
       <x:c r="D323" s="9"/>
       <x:c r="E323" s="9"/>
+      <x:c r="F323" s="29"/>
+      <x:c r="G323" s="29"/>
     </x:row>
     <x:row r="324">
       <x:c r="A324" s="8"/>
@@ -2612,6 +3332,8 @@
       <x:c r="C324" s="9"/>
       <x:c r="D324" s="9"/>
       <x:c r="E324" s="9"/>
+      <x:c r="F324" s="25"/>
+      <x:c r="G324" s="25"/>
     </x:row>
     <x:row r="325">
       <x:c r="A325" s="8"/>
@@ -2619,6 +3341,8 @@
       <x:c r="C325" s="9"/>
       <x:c r="D325" s="9"/>
       <x:c r="E325" s="9"/>
+      <x:c r="F325" s="29"/>
+      <x:c r="G325" s="29"/>
     </x:row>
     <x:row r="326">
       <x:c r="A326" s="8"/>
@@ -2626,6 +3350,8 @@
       <x:c r="C326" s="9"/>
       <x:c r="D326" s="9"/>
       <x:c r="E326" s="9"/>
+      <x:c r="F326" s="25"/>
+      <x:c r="G326" s="25"/>
     </x:row>
     <x:row r="327">
       <x:c r="A327" s="8"/>
@@ -2633,6 +3359,8 @@
       <x:c r="C327" s="9"/>
       <x:c r="D327" s="9"/>
       <x:c r="E327" s="9"/>
+      <x:c r="F327" s="29"/>
+      <x:c r="G327" s="29"/>
     </x:row>
     <x:row r="328">
       <x:c r="A328" s="8"/>
@@ -2640,6 +3368,8 @@
       <x:c r="C328" s="9"/>
       <x:c r="D328" s="9"/>
       <x:c r="E328" s="9"/>
+      <x:c r="F328" s="25"/>
+      <x:c r="G328" s="25"/>
     </x:row>
     <x:row r="329">
       <x:c r="A329" s="8"/>
@@ -2647,6 +3377,8 @@
       <x:c r="C329" s="9"/>
       <x:c r="D329" s="9"/>
       <x:c r="E329" s="9"/>
+      <x:c r="F329" s="29"/>
+      <x:c r="G329" s="29"/>
     </x:row>
     <x:row r="330">
       <x:c r="A330" s="8"/>
@@ -2654,6 +3386,8 @@
       <x:c r="C330" s="9"/>
       <x:c r="D330" s="9"/>
       <x:c r="E330" s="9"/>
+      <x:c r="F330" s="25"/>
+      <x:c r="G330" s="25"/>
     </x:row>
     <x:row r="331">
       <x:c r="A331" s="8"/>
@@ -2661,6 +3395,8 @@
       <x:c r="C331" s="9"/>
       <x:c r="D331" s="9"/>
       <x:c r="E331" s="9"/>
+      <x:c r="F331" s="29"/>
+      <x:c r="G331" s="29"/>
     </x:row>
     <x:row r="332">
       <x:c r="A332" s="8"/>
@@ -2668,6 +3404,8 @@
       <x:c r="C332" s="9"/>
       <x:c r="D332" s="9"/>
       <x:c r="E332" s="9"/>
+      <x:c r="F332" s="25"/>
+      <x:c r="G332" s="25"/>
     </x:row>
     <x:row r="333">
       <x:c r="A333" s="8"/>
@@ -2675,6 +3413,8 @@
       <x:c r="C333" s="9"/>
       <x:c r="D333" s="9"/>
       <x:c r="E333" s="9"/>
+      <x:c r="F333" s="29"/>
+      <x:c r="G333" s="29"/>
     </x:row>
     <x:row r="334">
       <x:c r="A334" s="8"/>
@@ -2682,6 +3422,8 @@
       <x:c r="C334" s="9"/>
       <x:c r="D334" s="9"/>
       <x:c r="E334" s="9"/>
+      <x:c r="F334" s="25"/>
+      <x:c r="G334" s="25"/>
     </x:row>
     <x:row r="335">
       <x:c r="A335" s="8"/>
@@ -2689,6 +3431,8 @@
       <x:c r="C335" s="9"/>
       <x:c r="D335" s="9"/>
       <x:c r="E335" s="9"/>
+      <x:c r="F335" s="29"/>
+      <x:c r="G335" s="29"/>
     </x:row>
     <x:row r="336">
       <x:c r="A336" s="8"/>
@@ -2696,6 +3440,8 @@
       <x:c r="C336" s="9"/>
       <x:c r="D336" s="9"/>
       <x:c r="E336" s="9"/>
+      <x:c r="F336" s="25"/>
+      <x:c r="G336" s="25"/>
     </x:row>
     <x:row r="337">
       <x:c r="A337" s="8"/>
@@ -2703,6 +3449,8 @@
       <x:c r="C337" s="9"/>
       <x:c r="D337" s="9"/>
       <x:c r="E337" s="9"/>
+      <x:c r="F337" s="29"/>
+      <x:c r="G337" s="29"/>
     </x:row>
     <x:row r="338">
       <x:c r="A338" s="8"/>
@@ -2710,6 +3458,8 @@
       <x:c r="C338" s="9"/>
       <x:c r="D338" s="9"/>
       <x:c r="E338" s="9"/>
+      <x:c r="F338" s="25"/>
+      <x:c r="G338" s="25"/>
     </x:row>
     <x:row r="339">
       <x:c r="A339" s="8"/>
@@ -2717,6 +3467,8 @@
       <x:c r="C339" s="9"/>
       <x:c r="D339" s="9"/>
       <x:c r="E339" s="9"/>
+      <x:c r="F339" s="29"/>
+      <x:c r="G339" s="29"/>
     </x:row>
     <x:row r="340">
       <x:c r="A340" s="8"/>
@@ -2724,6 +3476,8 @@
       <x:c r="C340" s="9"/>
       <x:c r="D340" s="9"/>
       <x:c r="E340" s="9"/>
+      <x:c r="F340" s="25"/>
+      <x:c r="G340" s="25"/>
     </x:row>
     <x:row r="341">
       <x:c r="A341" s="8"/>
@@ -2731,6 +3485,8 @@
       <x:c r="C341" s="9"/>
       <x:c r="D341" s="9"/>
       <x:c r="E341" s="9"/>
+      <x:c r="F341" s="29"/>
+      <x:c r="G341" s="29"/>
     </x:row>
     <x:row r="342">
       <x:c r="A342" s="8"/>
@@ -2738,6 +3494,8 @@
       <x:c r="C342" s="9"/>
       <x:c r="D342" s="9"/>
       <x:c r="E342" s="9"/>
+      <x:c r="F342" s="25"/>
+      <x:c r="G342" s="25"/>
     </x:row>
     <x:row r="343">
       <x:c r="A343" s="8"/>
@@ -2745,6 +3503,8 @@
       <x:c r="C343" s="9"/>
       <x:c r="D343" s="9"/>
       <x:c r="E343" s="9"/>
+      <x:c r="F343" s="29"/>
+      <x:c r="G343" s="29"/>
     </x:row>
     <x:row r="344">
       <x:c r="A344" s="8"/>
@@ -2752,6 +3512,8 @@
       <x:c r="C344" s="9"/>
       <x:c r="D344" s="9"/>
       <x:c r="E344" s="9"/>
+      <x:c r="F344" s="25"/>
+      <x:c r="G344" s="25"/>
     </x:row>
     <x:row r="345">
       <x:c r="A345" s="8"/>
@@ -2759,6 +3521,8 @@
       <x:c r="C345" s="9"/>
       <x:c r="D345" s="9"/>
       <x:c r="E345" s="9"/>
+      <x:c r="F345" s="29"/>
+      <x:c r="G345" s="29"/>
     </x:row>
     <x:row r="346">
       <x:c r="A346" s="8"/>
@@ -2766,6 +3530,8 @@
       <x:c r="C346" s="9"/>
       <x:c r="D346" s="9"/>
       <x:c r="E346" s="9"/>
+      <x:c r="F346" s="25"/>
+      <x:c r="G346" s="25"/>
     </x:row>
     <x:row r="347">
       <x:c r="A347" s="8"/>
@@ -2773,6 +3539,8 @@
       <x:c r="C347" s="9"/>
       <x:c r="D347" s="9"/>
       <x:c r="E347" s="9"/>
+      <x:c r="F347" s="29"/>
+      <x:c r="G347" s="29"/>
     </x:row>
     <x:row r="348">
       <x:c r="A348" s="8"/>
@@ -2780,6 +3548,8 @@
       <x:c r="C348" s="9"/>
       <x:c r="D348" s="9"/>
       <x:c r="E348" s="9"/>
+      <x:c r="F348" s="25"/>
+      <x:c r="G348" s="25"/>
     </x:row>
     <x:row r="349">
       <x:c r="A349" s="8"/>
@@ -2787,6 +3557,8 @@
       <x:c r="C349" s="9"/>
       <x:c r="D349" s="9"/>
       <x:c r="E349" s="9"/>
+      <x:c r="F349" s="29"/>
+      <x:c r="G349" s="29"/>
     </x:row>
     <x:row r="350">
       <x:c r="A350" s="8"/>
@@ -2794,6 +3566,8 @@
       <x:c r="C350" s="9"/>
       <x:c r="D350" s="9"/>
       <x:c r="E350" s="9"/>
+      <x:c r="F350" s="25"/>
+      <x:c r="G350" s="25"/>
     </x:row>
     <x:row r="351">
       <x:c r="A351" s="8"/>
@@ -2801,6 +3575,8 @@
       <x:c r="C351" s="9"/>
       <x:c r="D351" s="9"/>
       <x:c r="E351" s="9"/>
+      <x:c r="F351" s="29"/>
+      <x:c r="G351" s="29"/>
     </x:row>
     <x:row r="352">
       <x:c r="A352" s="8"/>
@@ -2808,6 +3584,8 @@
       <x:c r="C352" s="9"/>
       <x:c r="D352" s="9"/>
       <x:c r="E352" s="9"/>
+      <x:c r="F352" s="25"/>
+      <x:c r="G352" s="25"/>
     </x:row>
     <x:row r="353">
       <x:c r="A353" s="8"/>
@@ -2815,6 +3593,8 @@
       <x:c r="C353" s="9"/>
       <x:c r="D353" s="9"/>
       <x:c r="E353" s="9"/>
+      <x:c r="F353" s="29"/>
+      <x:c r="G353" s="29"/>
     </x:row>
     <x:row r="354">
       <x:c r="A354" s="8"/>
@@ -2822,6 +3602,8 @@
       <x:c r="C354" s="9"/>
       <x:c r="D354" s="9"/>
       <x:c r="E354" s="9"/>
+      <x:c r="F354" s="25"/>
+      <x:c r="G354" s="25"/>
     </x:row>
     <x:row r="355">
       <x:c r="A355" s="8"/>
@@ -2829,6 +3611,8 @@
       <x:c r="C355" s="9"/>
       <x:c r="D355" s="9"/>
       <x:c r="E355" s="9"/>
+      <x:c r="F355" s="29"/>
+      <x:c r="G355" s="29"/>
     </x:row>
     <x:row r="356">
       <x:c r="A356" s="8"/>
@@ -2836,6 +3620,8 @@
       <x:c r="C356" s="9"/>
       <x:c r="D356" s="9"/>
       <x:c r="E356" s="9"/>
+      <x:c r="F356" s="25"/>
+      <x:c r="G356" s="25"/>
     </x:row>
     <x:row r="357">
       <x:c r="A357" s="8"/>
@@ -2843,6 +3629,8 @@
       <x:c r="C357" s="9"/>
       <x:c r="D357" s="9"/>
       <x:c r="E357" s="9"/>
+      <x:c r="F357" s="29"/>
+      <x:c r="G357" s="29"/>
     </x:row>
     <x:row r="358">
       <x:c r="A358" s="8"/>
@@ -2850,6 +3638,8 @@
       <x:c r="C358" s="9"/>
       <x:c r="D358" s="9"/>
       <x:c r="E358" s="9"/>
+      <x:c r="F358" s="25"/>
+      <x:c r="G358" s="25"/>
     </x:row>
     <x:row r="359">
       <x:c r="A359" s="8"/>
@@ -2857,6 +3647,8 @@
       <x:c r="C359" s="9"/>
       <x:c r="D359" s="9"/>
       <x:c r="E359" s="9"/>
+      <x:c r="F359" s="29"/>
+      <x:c r="G359" s="29"/>
     </x:row>
     <x:row r="360">
       <x:c r="A360" s="8"/>
@@ -2864,6 +3656,8 @@
       <x:c r="C360" s="9"/>
       <x:c r="D360" s="9"/>
       <x:c r="E360" s="9"/>
+      <x:c r="F360" s="25"/>
+      <x:c r="G360" s="25"/>
     </x:row>
     <x:row r="361">
       <x:c r="A361" s="8"/>
@@ -2871,6 +3665,8 @@
       <x:c r="C361" s="9"/>
       <x:c r="D361" s="9"/>
       <x:c r="E361" s="9"/>
+      <x:c r="F361" s="29"/>
+      <x:c r="G361" s="29"/>
     </x:row>
     <x:row r="362">
       <x:c r="A362" s="8"/>
@@ -2878,6 +3674,8 @@
       <x:c r="C362" s="9"/>
       <x:c r="D362" s="9"/>
       <x:c r="E362" s="9"/>
+      <x:c r="F362" s="25"/>
+      <x:c r="G362" s="25"/>
     </x:row>
     <x:row r="363">
       <x:c r="A363" s="8"/>
@@ -2885,6 +3683,8 @@
       <x:c r="C363" s="9"/>
       <x:c r="D363" s="9"/>
       <x:c r="E363" s="9"/>
+      <x:c r="F363" s="29"/>
+      <x:c r="G363" s="29"/>
     </x:row>
     <x:row r="364">
       <x:c r="A364" s="8"/>
@@ -2892,6 +3692,8 @@
       <x:c r="C364" s="9"/>
       <x:c r="D364" s="9"/>
       <x:c r="E364" s="9"/>
+      <x:c r="F364" s="25"/>
+      <x:c r="G364" s="25"/>
     </x:row>
     <x:row r="365">
       <x:c r="A365" s="8"/>
@@ -2899,6 +3701,8 @@
       <x:c r="C365" s="9"/>
       <x:c r="D365" s="9"/>
       <x:c r="E365" s="9"/>
+      <x:c r="F365" s="29"/>
+      <x:c r="G365" s="29"/>
     </x:row>
     <x:row r="366">
       <x:c r="A366" s="8"/>
@@ -2906,6 +3710,8 @@
       <x:c r="C366" s="9"/>
       <x:c r="D366" s="9"/>
       <x:c r="E366" s="9"/>
+      <x:c r="F366" s="25"/>
+      <x:c r="G366" s="25"/>
     </x:row>
     <x:row r="367">
       <x:c r="A367" s="8"/>
@@ -2913,6 +3719,8 @@
       <x:c r="C367" s="9"/>
       <x:c r="D367" s="9"/>
       <x:c r="E367" s="9"/>
+      <x:c r="F367" s="29"/>
+      <x:c r="G367" s="29"/>
     </x:row>
     <x:row r="368">
       <x:c r="A368" s="8"/>
@@ -2920,6 +3728,8 @@
       <x:c r="C368" s="9"/>
       <x:c r="D368" s="9"/>
       <x:c r="E368" s="9"/>
+      <x:c r="F368" s="25"/>
+      <x:c r="G368" s="25"/>
     </x:row>
     <x:row r="369">
       <x:c r="A369" s="8"/>
@@ -2927,6 +3737,8 @@
       <x:c r="C369" s="9"/>
       <x:c r="D369" s="9"/>
       <x:c r="E369" s="9"/>
+      <x:c r="F369" s="29"/>
+      <x:c r="G369" s="29"/>
     </x:row>
     <x:row r="370">
       <x:c r="A370" s="8"/>
@@ -2934,6 +3746,8 @@
       <x:c r="C370" s="9"/>
       <x:c r="D370" s="9"/>
       <x:c r="E370" s="9"/>
+      <x:c r="F370" s="25"/>
+      <x:c r="G370" s="25"/>
     </x:row>
     <x:row r="371">
       <x:c r="A371" s="8"/>
@@ -2941,6 +3755,8 @@
       <x:c r="C371" s="9"/>
       <x:c r="D371" s="9"/>
       <x:c r="E371" s="9"/>
+      <x:c r="F371" s="29"/>
+      <x:c r="G371" s="29"/>
     </x:row>
     <x:row r="372">
       <x:c r="A372" s="8"/>
@@ -2948,6 +3764,8 @@
       <x:c r="C372" s="9"/>
       <x:c r="D372" s="9"/>
       <x:c r="E372" s="9"/>
+      <x:c r="F372" s="25"/>
+      <x:c r="G372" s="25"/>
     </x:row>
     <x:row r="373">
       <x:c r="A373" s="8"/>
@@ -2955,6 +3773,8 @@
       <x:c r="C373" s="9"/>
       <x:c r="D373" s="9"/>
       <x:c r="E373" s="9"/>
+      <x:c r="F373" s="29"/>
+      <x:c r="G373" s="29"/>
     </x:row>
     <x:row r="374">
       <x:c r="A374" s="8"/>
@@ -2962,6 +3782,8 @@
       <x:c r="C374" s="9"/>
       <x:c r="D374" s="9"/>
       <x:c r="E374" s="9"/>
+      <x:c r="F374" s="25"/>
+      <x:c r="G374" s="25"/>
     </x:row>
     <x:row r="375">
       <x:c r="A375" s="8"/>
@@ -2969,6 +3791,8 @@
       <x:c r="C375" s="9"/>
       <x:c r="D375" s="9"/>
       <x:c r="E375" s="9"/>
+      <x:c r="F375" s="29"/>
+      <x:c r="G375" s="29"/>
     </x:row>
     <x:row r="376">
       <x:c r="A376" s="8"/>
@@ -2976,6 +3800,8 @@
       <x:c r="C376" s="9"/>
       <x:c r="D376" s="9"/>
       <x:c r="E376" s="9"/>
+      <x:c r="F376" s="25"/>
+      <x:c r="G376" s="25"/>
     </x:row>
     <x:row r="377">
       <x:c r="A377" s="8"/>
@@ -2983,6 +3809,8 @@
       <x:c r="C377" s="9"/>
       <x:c r="D377" s="9"/>
       <x:c r="E377" s="9"/>
+      <x:c r="F377" s="29"/>
+      <x:c r="G377" s="29"/>
     </x:row>
     <x:row r="378">
       <x:c r="A378" s="8"/>
@@ -2990,6 +3818,8 @@
       <x:c r="C378" s="9"/>
       <x:c r="D378" s="9"/>
       <x:c r="E378" s="9"/>
+      <x:c r="F378" s="25"/>
+      <x:c r="G378" s="25"/>
     </x:row>
     <x:row r="379">
       <x:c r="A379" s="8"/>
@@ -2997,6 +3827,8 @@
       <x:c r="C379" s="9"/>
       <x:c r="D379" s="9"/>
       <x:c r="E379" s="9"/>
+      <x:c r="F379" s="29"/>
+      <x:c r="G379" s="29"/>
     </x:row>
     <x:row r="380">
       <x:c r="A380" s="8"/>
@@ -3004,6 +3836,8 @@
       <x:c r="C380" s="9"/>
       <x:c r="D380" s="9"/>
       <x:c r="E380" s="9"/>
+      <x:c r="F380" s="25"/>
+      <x:c r="G380" s="25"/>
     </x:row>
     <x:row r="381">
       <x:c r="A381" s="8"/>
@@ -3011,6 +3845,8 @@
       <x:c r="C381" s="9"/>
       <x:c r="D381" s="9"/>
       <x:c r="E381" s="9"/>
+      <x:c r="F381" s="29"/>
+      <x:c r="G381" s="29"/>
     </x:row>
     <x:row r="382">
       <x:c r="A382" s="8"/>
@@ -3018,6 +3854,8 @@
       <x:c r="C382" s="9"/>
       <x:c r="D382" s="9"/>
       <x:c r="E382" s="9"/>
+      <x:c r="F382" s="25"/>
+      <x:c r="G382" s="25"/>
     </x:row>
     <x:row r="383">
       <x:c r="A383" s="8"/>
@@ -3025,6 +3863,8 @@
       <x:c r="C383" s="9"/>
       <x:c r="D383" s="9"/>
       <x:c r="E383" s="9"/>
+      <x:c r="F383" s="29"/>
+      <x:c r="G383" s="29"/>
     </x:row>
     <x:row r="384">
       <x:c r="A384" s="8"/>
@@ -3032,6 +3872,8 @@
       <x:c r="C384" s="9"/>
       <x:c r="D384" s="9"/>
       <x:c r="E384" s="9"/>
+      <x:c r="F384" s="25"/>
+      <x:c r="G384" s="25"/>
     </x:row>
     <x:row r="385">
       <x:c r="A385" s="8"/>
@@ -3039,6 +3881,8 @@
       <x:c r="C385" s="9"/>
       <x:c r="D385" s="9"/>
       <x:c r="E385" s="9"/>
+      <x:c r="F385" s="29"/>
+      <x:c r="G385" s="29"/>
     </x:row>
     <x:row r="386">
       <x:c r="A386" s="8"/>
@@ -3046,6 +3890,8 @@
       <x:c r="C386" s="9"/>
       <x:c r="D386" s="9"/>
       <x:c r="E386" s="9"/>
+      <x:c r="F386" s="25"/>
+      <x:c r="G386" s="25"/>
     </x:row>
     <x:row r="387">
       <x:c r="A387" s="8"/>
@@ -3053,6 +3899,8 @@
       <x:c r="C387" s="9"/>
       <x:c r="D387" s="9"/>
       <x:c r="E387" s="9"/>
+      <x:c r="F387" s="29"/>
+      <x:c r="G387" s="29"/>
     </x:row>
     <x:row r="388">
       <x:c r="A388" s="8"/>
@@ -3060,6 +3908,8 @@
       <x:c r="C388" s="9"/>
       <x:c r="D388" s="9"/>
       <x:c r="E388" s="9"/>
+      <x:c r="F388" s="25"/>
+      <x:c r="G388" s="25"/>
     </x:row>
     <x:row r="389">
       <x:c r="A389" s="8"/>
@@ -3067,6 +3917,8 @@
       <x:c r="C389" s="9"/>
       <x:c r="D389" s="9"/>
       <x:c r="E389" s="9"/>
+      <x:c r="F389" s="29"/>
+      <x:c r="G389" s="29"/>
     </x:row>
     <x:row r="390">
       <x:c r="A390" s="8"/>
@@ -3074,6 +3926,8 @@
       <x:c r="C390" s="9"/>
       <x:c r="D390" s="9"/>
       <x:c r="E390" s="9"/>
+      <x:c r="F390" s="25"/>
+      <x:c r="G390" s="25"/>
     </x:row>
     <x:row r="391">
       <x:c r="A391" s="8"/>
@@ -3081,6 +3935,8 @@
       <x:c r="C391" s="9"/>
       <x:c r="D391" s="9"/>
       <x:c r="E391" s="9"/>
+      <x:c r="F391" s="29"/>
+      <x:c r="G391" s="29"/>
     </x:row>
     <x:row r="392">
       <x:c r="A392" s="8"/>
@@ -3088,6 +3944,8 @@
       <x:c r="C392" s="9"/>
       <x:c r="D392" s="9"/>
       <x:c r="E392" s="9"/>
+      <x:c r="F392" s="25"/>
+      <x:c r="G392" s="25"/>
     </x:row>
     <x:row r="393">
       <x:c r="A393" s="8"/>
@@ -3095,6 +3953,8 @@
       <x:c r="C393" s="9"/>
       <x:c r="D393" s="9"/>
       <x:c r="E393" s="9"/>
+      <x:c r="F393" s="29"/>
+      <x:c r="G393" s="29"/>
     </x:row>
     <x:row r="394">
       <x:c r="A394" s="8"/>
@@ -3102,6 +3962,8 @@
       <x:c r="C394" s="9"/>
       <x:c r="D394" s="9"/>
       <x:c r="E394" s="9"/>
+      <x:c r="F394" s="25"/>
+      <x:c r="G394" s="25"/>
     </x:row>
     <x:row r="395">
       <x:c r="A395" s="8"/>
@@ -3109,6 +3971,8 @@
       <x:c r="C395" s="9"/>
       <x:c r="D395" s="9"/>
       <x:c r="E395" s="9"/>
+      <x:c r="F395" s="29"/>
+      <x:c r="G395" s="29"/>
     </x:row>
     <x:row r="396">
       <x:c r="A396" s="8"/>
@@ -3116,6 +3980,8 @@
       <x:c r="C396" s="9"/>
       <x:c r="D396" s="9"/>
       <x:c r="E396" s="9"/>
+      <x:c r="F396" s="25"/>
+      <x:c r="G396" s="25"/>
     </x:row>
     <x:row r="397">
       <x:c r="A397" s="8"/>
@@ -3123,6 +3989,8 @@
       <x:c r="C397" s="9"/>
       <x:c r="D397" s="9"/>
       <x:c r="E397" s="9"/>
+      <x:c r="F397" s="29"/>
+      <x:c r="G397" s="29"/>
     </x:row>
     <x:row r="398">
       <x:c r="A398" s="8"/>
@@ -3130,6 +3998,8 @@
       <x:c r="C398" s="9"/>
       <x:c r="D398" s="9"/>
       <x:c r="E398" s="9"/>
+      <x:c r="F398" s="25"/>
+      <x:c r="G398" s="25"/>
     </x:row>
     <x:row r="399">
       <x:c r="A399" s="8"/>
@@ -3137,6 +4007,8 @@
       <x:c r="C399" s="9"/>
       <x:c r="D399" s="9"/>
       <x:c r="E399" s="9"/>
+      <x:c r="F399" s="29"/>
+      <x:c r="G399" s="29"/>
     </x:row>
     <x:row r="400">
       <x:c r="A400" s="8"/>
@@ -3144,6 +4016,8 @@
       <x:c r="C400" s="9"/>
       <x:c r="D400" s="9"/>
       <x:c r="E400" s="9"/>
+      <x:c r="F400" s="25"/>
+      <x:c r="G400" s="25"/>
     </x:row>
     <x:row r="401">
       <x:c r="A401" s="8"/>
@@ -3151,6 +4025,8 @@
       <x:c r="C401" s="9"/>
       <x:c r="D401" s="9"/>
       <x:c r="E401" s="9"/>
+      <x:c r="F401" s="29"/>
+      <x:c r="G401" s="29"/>
     </x:row>
     <x:row r="402">
       <x:c r="A402" s="8"/>
@@ -3158,6 +4034,8 @@
       <x:c r="C402" s="9"/>
       <x:c r="D402" s="9"/>
       <x:c r="E402" s="9"/>
+      <x:c r="F402" s="25"/>
+      <x:c r="G402" s="25"/>
     </x:row>
     <x:row r="403">
       <x:c r="A403" s="8"/>
@@ -3165,6 +4043,8 @@
       <x:c r="C403" s="9"/>
       <x:c r="D403" s="9"/>
       <x:c r="E403" s="9"/>
+      <x:c r="F403" s="29"/>
+      <x:c r="G403" s="29"/>
     </x:row>
     <x:row r="404">
       <x:c r="A404" s="8"/>
@@ -3172,6 +4052,8 @@
       <x:c r="C404" s="9"/>
       <x:c r="D404" s="9"/>
       <x:c r="E404" s="9"/>
+      <x:c r="F404" s="25"/>
+      <x:c r="G404" s="25"/>
     </x:row>
     <x:row r="405">
       <x:c r="A405" s="8"/>
@@ -3179,6 +4061,8 @@
       <x:c r="C405" s="9"/>
       <x:c r="D405" s="9"/>
       <x:c r="E405" s="9"/>
+      <x:c r="F405" s="29"/>
+      <x:c r="G405" s="29"/>
     </x:row>
     <x:row r="406">
       <x:c r="A406" s="8"/>
@@ -3186,6 +4070,8 @@
       <x:c r="C406" s="9"/>
       <x:c r="D406" s="9"/>
       <x:c r="E406" s="9"/>
+      <x:c r="F406" s="25"/>
+      <x:c r="G406" s="25"/>
     </x:row>
     <x:row r="407">
       <x:c r="A407" s="8"/>
@@ -3193,6 +4079,8 @@
       <x:c r="C407" s="9"/>
       <x:c r="D407" s="9"/>
       <x:c r="E407" s="9"/>
+      <x:c r="F407" s="29"/>
+      <x:c r="G407" s="29"/>
     </x:row>
     <x:row r="408">
       <x:c r="A408" s="8"/>
@@ -3200,6 +4088,8 @@
       <x:c r="C408" s="9"/>
       <x:c r="D408" s="9"/>
       <x:c r="E408" s="9"/>
+      <x:c r="F408" s="25"/>
+      <x:c r="G408" s="25"/>
     </x:row>
     <x:row r="409">
       <x:c r="A409" s="8"/>
@@ -3207,6 +4097,8 @@
       <x:c r="C409" s="9"/>
       <x:c r="D409" s="9"/>
       <x:c r="E409" s="9"/>
+      <x:c r="F409" s="29"/>
+      <x:c r="G409" s="29"/>
     </x:row>
     <x:row r="410">
       <x:c r="A410" s="8"/>
@@ -3214,6 +4106,8 @@
       <x:c r="C410" s="9"/>
       <x:c r="D410" s="9"/>
       <x:c r="E410" s="9"/>
+      <x:c r="F410" s="25"/>
+      <x:c r="G410" s="25"/>
     </x:row>
     <x:row r="411">
       <x:c r="A411" s="8"/>
@@ -3221,6 +4115,8 @@
       <x:c r="C411" s="9"/>
       <x:c r="D411" s="9"/>
       <x:c r="E411" s="9"/>
+      <x:c r="F411" s="29"/>
+      <x:c r="G411" s="29"/>
     </x:row>
     <x:row r="412">
       <x:c r="A412" s="8"/>
@@ -3228,6 +4124,8 @@
       <x:c r="C412" s="9"/>
       <x:c r="D412" s="9"/>
       <x:c r="E412" s="9"/>
+      <x:c r="F412" s="25"/>
+      <x:c r="G412" s="25"/>
     </x:row>
     <x:row r="413">
       <x:c r="A413" s="8"/>
@@ -3235,6 +4133,8 @@
       <x:c r="C413" s="9"/>
       <x:c r="D413" s="9"/>
       <x:c r="E413" s="9"/>
+      <x:c r="F413" s="29"/>
+      <x:c r="G413" s="29"/>
     </x:row>
     <x:row r="414">
       <x:c r="A414" s="8"/>
@@ -3242,6 +4142,8 @@
       <x:c r="C414" s="9"/>
       <x:c r="D414" s="9"/>
       <x:c r="E414" s="9"/>
+      <x:c r="F414" s="25"/>
+      <x:c r="G414" s="25"/>
     </x:row>
     <x:row r="415">
       <x:c r="A415" s="8"/>
@@ -3249,6 +4151,8 @@
       <x:c r="C415" s="9"/>
       <x:c r="D415" s="9"/>
       <x:c r="E415" s="9"/>
+      <x:c r="F415" s="29"/>
+      <x:c r="G415" s="29"/>
     </x:row>
     <x:row r="416">
       <x:c r="A416" s="8"/>
@@ -3256,6 +4160,8 @@
       <x:c r="C416" s="9"/>
       <x:c r="D416" s="9"/>
       <x:c r="E416" s="9"/>
+      <x:c r="F416" s="25"/>
+      <x:c r="G416" s="25"/>
     </x:row>
     <x:row r="417">
       <x:c r="A417" s="8"/>
@@ -3263,6 +4169,8 @@
       <x:c r="C417" s="9"/>
       <x:c r="D417" s="9"/>
       <x:c r="E417" s="9"/>
+      <x:c r="F417" s="29"/>
+      <x:c r="G417" s="29"/>
     </x:row>
     <x:row r="418">
       <x:c r="A418" s="8"/>
@@ -3270,6 +4178,8 @@
       <x:c r="C418" s="9"/>
       <x:c r="D418" s="9"/>
       <x:c r="E418" s="9"/>
+      <x:c r="F418" s="25"/>
+      <x:c r="G418" s="25"/>
     </x:row>
     <x:row r="419">
       <x:c r="A419" s="8"/>
@@ -3277,6 +4187,8 @@
       <x:c r="C419" s="9"/>
       <x:c r="D419" s="9"/>
       <x:c r="E419" s="9"/>
+      <x:c r="F419" s="29"/>
+      <x:c r="G419" s="29"/>
     </x:row>
     <x:row r="420">
       <x:c r="A420" s="8"/>
@@ -3284,6 +4196,8 @@
       <x:c r="C420" s="9"/>
       <x:c r="D420" s="9"/>
       <x:c r="E420" s="9"/>
+      <x:c r="F420" s="25"/>
+      <x:c r="G420" s="25"/>
     </x:row>
     <x:row r="421">
       <x:c r="A421" s="8"/>
@@ -3291,6 +4205,8 @@
       <x:c r="C421" s="9"/>
       <x:c r="D421" s="9"/>
       <x:c r="E421" s="9"/>
+      <x:c r="F421" s="29"/>
+      <x:c r="G421" s="29"/>
     </x:row>
     <x:row r="422">
       <x:c r="A422" s="8"/>
@@ -3298,6 +4214,8 @@
       <x:c r="C422" s="9"/>
       <x:c r="D422" s="9"/>
       <x:c r="E422" s="9"/>
+      <x:c r="F422" s="25"/>
+      <x:c r="G422" s="25"/>
     </x:row>
     <x:row r="423">
       <x:c r="A423" s="8"/>
@@ -3305,6 +4223,8 @@
       <x:c r="C423" s="9"/>
       <x:c r="D423" s="9"/>
       <x:c r="E423" s="9"/>
+      <x:c r="F423" s="29"/>
+      <x:c r="G423" s="29"/>
     </x:row>
     <x:row r="424">
       <x:c r="A424" s="8"/>
@@ -3312,6 +4232,8 @@
       <x:c r="C424" s="9"/>
       <x:c r="D424" s="9"/>
       <x:c r="E424" s="9"/>
+      <x:c r="F424" s="25"/>
+      <x:c r="G424" s="25"/>
     </x:row>
     <x:row r="425">
       <x:c r="A425" s="8"/>
@@ -3319,6 +4241,8 @@
       <x:c r="C425" s="9"/>
       <x:c r="D425" s="9"/>
       <x:c r="E425" s="9"/>
+      <x:c r="F425" s="29"/>
+      <x:c r="G425" s="29"/>
     </x:row>
     <x:row r="426">
       <x:c r="A426" s="8"/>
@@ -3326,6 +4250,8 @@
       <x:c r="C426" s="9"/>
       <x:c r="D426" s="9"/>
       <x:c r="E426" s="9"/>
+      <x:c r="F426" s="25"/>
+      <x:c r="G426" s="25"/>
     </x:row>
     <x:row r="427">
       <x:c r="A427" s="8"/>
@@ -3333,6 +4259,8 @@
       <x:c r="C427" s="9"/>
       <x:c r="D427" s="9"/>
       <x:c r="E427" s="9"/>
+      <x:c r="F427" s="29"/>
+      <x:c r="G427" s="29"/>
     </x:row>
     <x:row r="428">
       <x:c r="A428" s="8"/>
@@ -3340,6 +4268,8 @@
       <x:c r="C428" s="9"/>
       <x:c r="D428" s="9"/>
       <x:c r="E428" s="9"/>
+      <x:c r="F428" s="25"/>
+      <x:c r="G428" s="25"/>
     </x:row>
     <x:row r="429">
       <x:c r="A429" s="8"/>
@@ -3347,6 +4277,8 @@
       <x:c r="C429" s="9"/>
       <x:c r="D429" s="9"/>
       <x:c r="E429" s="9"/>
+      <x:c r="F429" s="29"/>
+      <x:c r="G429" s="29"/>
     </x:row>
     <x:row r="430">
       <x:c r="A430" s="8"/>
@@ -3354,6 +4286,8 @@
       <x:c r="C430" s="9"/>
       <x:c r="D430" s="9"/>
       <x:c r="E430" s="9"/>
+      <x:c r="F430" s="25"/>
+      <x:c r="G430" s="25"/>
     </x:row>
     <x:row r="431">
       <x:c r="A431" s="8"/>
@@ -3361,6 +4295,8 @@
       <x:c r="C431" s="9"/>
       <x:c r="D431" s="9"/>
       <x:c r="E431" s="9"/>
+      <x:c r="F431" s="29"/>
+      <x:c r="G431" s="29"/>
     </x:row>
     <x:row r="432">
       <x:c r="A432" s="8"/>
@@ -3368,6 +4304,8 @@
       <x:c r="C432" s="9"/>
       <x:c r="D432" s="9"/>
       <x:c r="E432" s="9"/>
+      <x:c r="F432" s="25"/>
+      <x:c r="G432" s="25"/>
     </x:row>
     <x:row r="433">
       <x:c r="A433" s="8"/>
@@ -3375,6 +4313,8 @@
       <x:c r="C433" s="9"/>
       <x:c r="D433" s="9"/>
       <x:c r="E433" s="9"/>
+      <x:c r="F433" s="29"/>
+      <x:c r="G433" s="29"/>
     </x:row>
     <x:row r="434">
       <x:c r="A434" s="8"/>
@@ -3382,6 +4322,8 @@
       <x:c r="C434" s="9"/>
       <x:c r="D434" s="9"/>
       <x:c r="E434" s="9"/>
+      <x:c r="F434" s="25"/>
+      <x:c r="G434" s="25"/>
     </x:row>
     <x:row r="435">
       <x:c r="A435" s="8"/>
@@ -3389,6 +4331,8 @@
       <x:c r="C435" s="9"/>
       <x:c r="D435" s="9"/>
       <x:c r="E435" s="9"/>
+      <x:c r="F435" s="29"/>
+      <x:c r="G435" s="29"/>
     </x:row>
     <x:row r="436">
       <x:c r="A436" s="8"/>
@@ -3396,6 +4340,8 @@
       <x:c r="C436" s="9"/>
       <x:c r="D436" s="9"/>
       <x:c r="E436" s="9"/>
+      <x:c r="F436" s="25"/>
+      <x:c r="G436" s="25"/>
     </x:row>
     <x:row r="437">
       <x:c r="A437" s="8"/>
@@ -3403,6 +4349,8 @@
       <x:c r="C437" s="9"/>
       <x:c r="D437" s="9"/>
       <x:c r="E437" s="9"/>
+      <x:c r="F437" s="29"/>
+      <x:c r="G437" s="29"/>
     </x:row>
     <x:row r="438">
       <x:c r="A438" s="8"/>
@@ -3410,6 +4358,8 @@
       <x:c r="C438" s="9"/>
       <x:c r="D438" s="9"/>
       <x:c r="E438" s="9"/>
+      <x:c r="F438" s="25"/>
+      <x:c r="G438" s="25"/>
     </x:row>
     <x:row r="439">
       <x:c r="A439" s="8"/>
@@ -3417,6 +4367,8 @@
       <x:c r="C439" s="9"/>
       <x:c r="D439" s="9"/>
       <x:c r="E439" s="9"/>
+      <x:c r="F439" s="29"/>
+      <x:c r="G439" s="29"/>
     </x:row>
     <x:row r="440">
       <x:c r="A440" s="8"/>
@@ -3424,6 +4376,8 @@
       <x:c r="C440" s="9"/>
       <x:c r="D440" s="9"/>
       <x:c r="E440" s="9"/>
+      <x:c r="F440" s="25"/>
+      <x:c r="G440" s="25"/>
     </x:row>
     <x:row r="441">
       <x:c r="A441" s="8"/>
@@ -3431,6 +4385,8 @@
       <x:c r="C441" s="9"/>
       <x:c r="D441" s="9"/>
       <x:c r="E441" s="9"/>
+      <x:c r="F441" s="29"/>
+      <x:c r="G441" s="29"/>
     </x:row>
     <x:row r="442">
       <x:c r="A442" s="8"/>
@@ -3438,6 +4394,8 @@
       <x:c r="C442" s="9"/>
       <x:c r="D442" s="9"/>
       <x:c r="E442" s="9"/>
+      <x:c r="F442" s="25"/>
+      <x:c r="G442" s="25"/>
     </x:row>
     <x:row r="443">
       <x:c r="A443" s="8"/>
@@ -3445,6 +4403,8 @@
       <x:c r="C443" s="9"/>
       <x:c r="D443" s="9"/>
       <x:c r="E443" s="9"/>
+      <x:c r="F443" s="29"/>
+      <x:c r="G443" s="29"/>
     </x:row>
     <x:row r="444">
       <x:c r="A444" s="8"/>
@@ -3452,6 +4412,8 @@
       <x:c r="C444" s="9"/>
       <x:c r="D444" s="9"/>
       <x:c r="E444" s="9"/>
+      <x:c r="F444" s="25"/>
+      <x:c r="G444" s="25"/>
     </x:row>
     <x:row r="445">
       <x:c r="A445" s="8"/>
@@ -3459,6 +4421,8 @@
       <x:c r="C445" s="9"/>
       <x:c r="D445" s="9"/>
       <x:c r="E445" s="9"/>
+      <x:c r="F445" s="29"/>
+      <x:c r="G445" s="29"/>
     </x:row>
     <x:row r="446">
       <x:c r="A446" s="8"/>
@@ -3466,6 +4430,8 @@
       <x:c r="C446" s="9"/>
       <x:c r="D446" s="9"/>
       <x:c r="E446" s="9"/>
+      <x:c r="F446" s="25"/>
+      <x:c r="G446" s="25"/>
     </x:row>
     <x:row r="447">
       <x:c r="A447" s="8"/>
@@ -3473,6 +4439,8 @@
       <x:c r="C447" s="9"/>
       <x:c r="D447" s="9"/>
       <x:c r="E447" s="9"/>
+      <x:c r="F447" s="29"/>
+      <x:c r="G447" s="29"/>
     </x:row>
     <x:row r="448">
       <x:c r="A448" s="8"/>
@@ -3480,6 +4448,8 @@
       <x:c r="C448" s="9"/>
       <x:c r="D448" s="9"/>
       <x:c r="E448" s="9"/>
+      <x:c r="F448" s="25"/>
+      <x:c r="G448" s="25"/>
     </x:row>
     <x:row r="449">
       <x:c r="A449" s="8"/>
@@ -3487,6 +4457,8 @@
       <x:c r="C449" s="9"/>
       <x:c r="D449" s="9"/>
       <x:c r="E449" s="9"/>
+      <x:c r="F449" s="29"/>
+      <x:c r="G449" s="29"/>
     </x:row>
     <x:row r="450">
       <x:c r="A450" s="8"/>
@@ -3494,6 +4466,8 @@
       <x:c r="C450" s="9"/>
       <x:c r="D450" s="9"/>
       <x:c r="E450" s="9"/>
+      <x:c r="F450" s="25"/>
+      <x:c r="G450" s="25"/>
     </x:row>
     <x:row r="451">
       <x:c r="A451" s="8"/>
@@ -3501,6 +4475,8 @@
       <x:c r="C451" s="9"/>
       <x:c r="D451" s="9"/>
       <x:c r="E451" s="9"/>
+      <x:c r="F451" s="29"/>
+      <x:c r="G451" s="29"/>
     </x:row>
     <x:row r="452">
       <x:c r="A452" s="8"/>
@@ -3508,6 +4484,8 @@
       <x:c r="C452" s="9"/>
       <x:c r="D452" s="9"/>
       <x:c r="E452" s="9"/>
+      <x:c r="F452" s="25"/>
+      <x:c r="G452" s="25"/>
     </x:row>
     <x:row r="453">
       <x:c r="A453" s="8"/>
@@ -3515,6 +4493,8 @@
       <x:c r="C453" s="9"/>
       <x:c r="D453" s="9"/>
       <x:c r="E453" s="9"/>
+      <x:c r="F453" s="29"/>
+      <x:c r="G453" s="29"/>
     </x:row>
     <x:row r="454">
       <x:c r="A454" s="8"/>
@@ -3522,6 +4502,8 @@
       <x:c r="C454" s="9"/>
       <x:c r="D454" s="9"/>
       <x:c r="E454" s="9"/>
+      <x:c r="F454" s="25"/>
+      <x:c r="G454" s="25"/>
     </x:row>
     <x:row r="455">
       <x:c r="A455" s="8"/>
@@ -3529,6 +4511,8 @@
       <x:c r="C455" s="9"/>
       <x:c r="D455" s="9"/>
       <x:c r="E455" s="9"/>
+      <x:c r="F455" s="29"/>
+      <x:c r="G455" s="29"/>
     </x:row>
     <x:row r="456">
       <x:c r="A456" s="8"/>
@@ -3536,6 +4520,8 @@
       <x:c r="C456" s="9"/>
       <x:c r="D456" s="9"/>
       <x:c r="E456" s="9"/>
+      <x:c r="F456" s="25"/>
+      <x:c r="G456" s="25"/>
     </x:row>
     <x:row r="457">
       <x:c r="A457" s="8"/>
@@ -3543,6 +4529,8 @@
       <x:c r="C457" s="9"/>
       <x:c r="D457" s="9"/>
       <x:c r="E457" s="9"/>
+      <x:c r="F457" s="29"/>
+      <x:c r="G457" s="29"/>
     </x:row>
     <x:row r="458">
       <x:c r="A458" s="8"/>
@@ -3550,6 +4538,8 @@
       <x:c r="C458" s="9"/>
       <x:c r="D458" s="9"/>
       <x:c r="E458" s="9"/>
+      <x:c r="F458" s="25"/>
+      <x:c r="G458" s="25"/>
     </x:row>
     <x:row r="459">
       <x:c r="A459" s="8"/>
@@ -3557,6 +4547,8 @@
       <x:c r="C459" s="9"/>
       <x:c r="D459" s="9"/>
       <x:c r="E459" s="9"/>
+      <x:c r="F459" s="29"/>
+      <x:c r="G459" s="29"/>
     </x:row>
     <x:row r="460">
       <x:c r="A460" s="8"/>
@@ -3564,6 +4556,8 @@
       <x:c r="C460" s="9"/>
       <x:c r="D460" s="9"/>
       <x:c r="E460" s="9"/>
+      <x:c r="F460" s="25"/>
+      <x:c r="G460" s="25"/>
     </x:row>
     <x:row r="461">
       <x:c r="A461" s="8"/>
@@ -3571,6 +4565,8 @@
       <x:c r="C461" s="9"/>
       <x:c r="D461" s="9"/>
       <x:c r="E461" s="9"/>
+      <x:c r="F461" s="29"/>
+      <x:c r="G461" s="29"/>
     </x:row>
     <x:row r="462">
       <x:c r="A462" s="8"/>
@@ -3578,6 +4574,8 @@
       <x:c r="C462" s="9"/>
       <x:c r="D462" s="9"/>
       <x:c r="E462" s="9"/>
+      <x:c r="F462" s="25"/>
+      <x:c r="G462" s="25"/>
     </x:row>
     <x:row r="463">
       <x:c r="A463" s="8"/>
@@ -3585,6 +4583,8 @@
       <x:c r="C463" s="9"/>
       <x:c r="D463" s="9"/>
       <x:c r="E463" s="9"/>
+      <x:c r="F463" s="29"/>
+      <x:c r="G463" s="29"/>
     </x:row>
     <x:row r="464">
       <x:c r="A464" s="8"/>
@@ -3592,6 +4592,8 @@
       <x:c r="C464" s="9"/>
       <x:c r="D464" s="9"/>
       <x:c r="E464" s="9"/>
+      <x:c r="F464" s="25"/>
+      <x:c r="G464" s="25"/>
     </x:row>
     <x:row r="465">
       <x:c r="A465" s="8"/>
@@ -3599,6 +4601,8 @@
       <x:c r="C465" s="9"/>
       <x:c r="D465" s="9"/>
       <x:c r="E465" s="9"/>
+      <x:c r="F465" s="29"/>
+      <x:c r="G465" s="29"/>
     </x:row>
     <x:row r="466">
       <x:c r="A466" s="8"/>
@@ -3606,6 +4610,8 @@
       <x:c r="C466" s="9"/>
       <x:c r="D466" s="9"/>
       <x:c r="E466" s="9"/>
+      <x:c r="F466" s="25"/>
+      <x:c r="G466" s="25"/>
     </x:row>
     <x:row r="467">
       <x:c r="A467" s="8"/>
@@ -3613,6 +4619,8 @@
       <x:c r="C467" s="9"/>
       <x:c r="D467" s="9"/>
       <x:c r="E467" s="9"/>
+      <x:c r="F467" s="29"/>
+      <x:c r="G467" s="29"/>
     </x:row>
     <x:row r="468">
       <x:c r="A468" s="8"/>
@@ -3620,6 +4628,8 @@
       <x:c r="C468" s="9"/>
       <x:c r="D468" s="9"/>
       <x:c r="E468" s="9"/>
+      <x:c r="F468" s="25"/>
+      <x:c r="G468" s="25"/>
     </x:row>
     <x:row r="469">
       <x:c r="A469" s="8"/>
@@ -3627,6 +4637,8 @@
       <x:c r="C469" s="9"/>
       <x:c r="D469" s="9"/>
       <x:c r="E469" s="9"/>
+      <x:c r="F469" s="29"/>
+      <x:c r="G469" s="29"/>
     </x:row>
     <x:row r="470">
       <x:c r="A470" s="8"/>
@@ -3634,6 +4646,8 @@
       <x:c r="C470" s="9"/>
       <x:c r="D470" s="9"/>
       <x:c r="E470" s="9"/>
+      <x:c r="F470" s="25"/>
+      <x:c r="G470" s="25"/>
     </x:row>
     <x:row r="471">
       <x:c r="A471" s="8"/>
@@ -3641,6 +4655,8 @@
       <x:c r="C471" s="9"/>
       <x:c r="D471" s="9"/>
       <x:c r="E471" s="9"/>
+      <x:c r="F471" s="29"/>
+      <x:c r="G471" s="29"/>
     </x:row>
     <x:row r="472">
       <x:c r="A472" s="8"/>
@@ -3648,6 +4664,8 @@
       <x:c r="C472" s="9"/>
       <x:c r="D472" s="9"/>
       <x:c r="E472" s="9"/>
+      <x:c r="F472" s="25"/>
+      <x:c r="G472" s="25"/>
     </x:row>
     <x:row r="473">
       <x:c r="A473" s="8"/>
@@ -3655,6 +4673,8 @@
       <x:c r="C473" s="9"/>
       <x:c r="D473" s="9"/>
       <x:c r="E473" s="9"/>
+      <x:c r="F473" s="29"/>
+      <x:c r="G473" s="29"/>
     </x:row>
     <x:row r="474">
       <x:c r="A474" s="8"/>
@@ -3662,6 +4682,8 @@
       <x:c r="C474" s="9"/>
       <x:c r="D474" s="9"/>
       <x:c r="E474" s="9"/>
+      <x:c r="F474" s="25"/>
+      <x:c r="G474" s="25"/>
     </x:row>
     <x:row r="475">
       <x:c r="A475" s="8"/>
@@ -3669,6 +4691,8 @@
       <x:c r="C475" s="9"/>
       <x:c r="D475" s="9"/>
       <x:c r="E475" s="9"/>
+      <x:c r="F475" s="29"/>
+      <x:c r="G475" s="29"/>
     </x:row>
     <x:row r="476">
       <x:c r="A476" s="8"/>
@@ -3676,6 +4700,8 @@
       <x:c r="C476" s="9"/>
       <x:c r="D476" s="9"/>
       <x:c r="E476" s="9"/>
+      <x:c r="F476" s="25"/>
+      <x:c r="G476" s="25"/>
     </x:row>
     <x:row r="477">
       <x:c r="A477" s="8"/>
@@ -3683,6 +4709,8 @@
       <x:c r="C477" s="9"/>
       <x:c r="D477" s="9"/>
       <x:c r="E477" s="9"/>
+      <x:c r="F477" s="29"/>
+      <x:c r="G477" s="29"/>
     </x:row>
     <x:row r="478">
       <x:c r="A478" s="8"/>
@@ -3690,6 +4718,8 @@
       <x:c r="C478" s="9"/>
       <x:c r="D478" s="9"/>
       <x:c r="E478" s="9"/>
+      <x:c r="F478" s="25"/>
+      <x:c r="G478" s="25"/>
     </x:row>
     <x:row r="479">
       <x:c r="A479" s="8"/>
@@ -3697,6 +4727,8 @@
       <x:c r="C479" s="9"/>
       <x:c r="D479" s="9"/>
       <x:c r="E479" s="9"/>
+      <x:c r="F479" s="29"/>
+      <x:c r="G479" s="29"/>
     </x:row>
     <x:row r="480">
       <x:c r="A480" s="8"/>
@@ -3704,6 +4736,8 @@
       <x:c r="C480" s="9"/>
       <x:c r="D480" s="9"/>
       <x:c r="E480" s="9"/>
+      <x:c r="F480" s="25"/>
+      <x:c r="G480" s="25"/>
     </x:row>
     <x:row r="481">
       <x:c r="A481" s="8"/>
@@ -3711,6 +4745,8 @@
       <x:c r="C481" s="9"/>
       <x:c r="D481" s="9"/>
       <x:c r="E481" s="9"/>
+      <x:c r="F481" s="29"/>
+      <x:c r="G481" s="29"/>
     </x:row>
     <x:row r="482">
       <x:c r="A482" s="8"/>
@@ -3718,6 +4754,8 @@
       <x:c r="C482" s="9"/>
       <x:c r="D482" s="9"/>
       <x:c r="E482" s="9"/>
+      <x:c r="F482" s="25"/>
+      <x:c r="G482" s="25"/>
     </x:row>
     <x:row r="483">
       <x:c r="A483" s="8"/>
@@ -3725,6 +4763,8 @@
       <x:c r="C483" s="9"/>
       <x:c r="D483" s="9"/>
       <x:c r="E483" s="9"/>
+      <x:c r="F483" s="29"/>
+      <x:c r="G483" s="29"/>
     </x:row>
     <x:row r="484">
       <x:c r="A484" s="8"/>
@@ -3732,6 +4772,8 @@
       <x:c r="C484" s="9"/>
       <x:c r="D484" s="9"/>
       <x:c r="E484" s="9"/>
+      <x:c r="F484" s="25"/>
+      <x:c r="G484" s="25"/>
     </x:row>
     <x:row r="485">
       <x:c r="A485" s="8"/>
@@ -3739,6 +4781,8 @@
       <x:c r="C485" s="9"/>
       <x:c r="D485" s="9"/>
       <x:c r="E485" s="9"/>
+      <x:c r="F485" s="29"/>
+      <x:c r="G485" s="29"/>
     </x:row>
     <x:row r="486">
       <x:c r="A486" s="8"/>
@@ -3746,6 +4790,8 @@
       <x:c r="C486" s="9"/>
       <x:c r="D486" s="9"/>
       <x:c r="E486" s="9"/>
+      <x:c r="F486" s="25"/>
+      <x:c r="G486" s="25"/>
     </x:row>
     <x:row r="487">
       <x:c r="A487" s="8"/>
@@ -3753,6 +4799,8 @@
       <x:c r="C487" s="9"/>
       <x:c r="D487" s="9"/>
       <x:c r="E487" s="9"/>
+      <x:c r="F487" s="29"/>
+      <x:c r="G487" s="29"/>
     </x:row>
     <x:row r="488">
       <x:c r="A488" s="8"/>
@@ -3760,6 +4808,8 @@
       <x:c r="C488" s="9"/>
       <x:c r="D488" s="9"/>
       <x:c r="E488" s="9"/>
+      <x:c r="F488" s="25"/>
+      <x:c r="G488" s="25"/>
     </x:row>
     <x:row r="489">
       <x:c r="A489" s="8"/>
@@ -3767,6 +4817,8 @@
       <x:c r="C489" s="9"/>
       <x:c r="D489" s="9"/>
       <x:c r="E489" s="9"/>
+      <x:c r="F489" s="29"/>
+      <x:c r="G489" s="29"/>
     </x:row>
     <x:row r="490">
       <x:c r="A490" s="8"/>
@@ -3774,6 +4826,8 @@
       <x:c r="C490" s="9"/>
       <x:c r="D490" s="9"/>
       <x:c r="E490" s="9"/>
+      <x:c r="F490" s="25"/>
+      <x:c r="G490" s="25"/>
     </x:row>
     <x:row r="491">
       <x:c r="A491" s="8"/>
@@ -3781,6 +4835,8 @@
       <x:c r="C491" s="9"/>
       <x:c r="D491" s="9"/>
       <x:c r="E491" s="9"/>
+      <x:c r="F491" s="29"/>
+      <x:c r="G491" s="29"/>
     </x:row>
     <x:row r="492">
       <x:c r="A492" s="8"/>
@@ -3788,6 +4844,8 @@
       <x:c r="C492" s="9"/>
       <x:c r="D492" s="9"/>
       <x:c r="E492" s="9"/>
+      <x:c r="F492" s="25"/>
+      <x:c r="G492" s="25"/>
     </x:row>
     <x:row r="493">
       <x:c r="A493" s="8"/>
@@ -3795,6 +4853,8 @@
       <x:c r="C493" s="9"/>
       <x:c r="D493" s="9"/>
       <x:c r="E493" s="9"/>
+      <x:c r="F493" s="29"/>
+      <x:c r="G493" s="29"/>
     </x:row>
     <x:row r="494">
       <x:c r="A494" s="8"/>
@@ -3802,6 +4862,8 @@
       <x:c r="C494" s="9"/>
       <x:c r="D494" s="9"/>
       <x:c r="E494" s="9"/>
+      <x:c r="F494" s="25"/>
+      <x:c r="G494" s="25"/>
     </x:row>
     <x:row r="495">
       <x:c r="A495" s="8"/>
@@ -3809,6 +4871,8 @@
       <x:c r="C495" s="9"/>
       <x:c r="D495" s="9"/>
       <x:c r="E495" s="9"/>
+      <x:c r="F495" s="29"/>
+      <x:c r="G495" s="29"/>
     </x:row>
     <x:row r="496">
       <x:c r="A496" s="8"/>
@@ -3816,6 +4880,8 @@
       <x:c r="C496" s="9"/>
       <x:c r="D496" s="9"/>
       <x:c r="E496" s="9"/>
+      <x:c r="F496" s="25"/>
+      <x:c r="G496" s="25"/>
     </x:row>
     <x:row r="497">
       <x:c r="A497" s="8"/>
@@ -3823,6 +4889,8 @@
       <x:c r="C497" s="9"/>
       <x:c r="D497" s="9"/>
       <x:c r="E497" s="9"/>
+      <x:c r="F497" s="29"/>
+      <x:c r="G497" s="29"/>
     </x:row>
     <x:row r="498">
       <x:c r="A498" s="8"/>
@@ -3830,6 +4898,8 @@
       <x:c r="C498" s="9"/>
       <x:c r="D498" s="9"/>
       <x:c r="E498" s="9"/>
+      <x:c r="F498" s="25"/>
+      <x:c r="G498" s="25"/>
     </x:row>
     <x:row r="499">
       <x:c r="A499" s="8"/>
@@ -3837,6 +4907,8 @@
       <x:c r="C499" s="9"/>
       <x:c r="D499" s="9"/>
       <x:c r="E499" s="9"/>
+      <x:c r="F499" s="29"/>
+      <x:c r="G499" s="29"/>
     </x:row>
     <x:row r="500">
       <x:c r="A500" s="8"/>
@@ -3844,11 +4916,21 @@
       <x:c r="C500" s="9"/>
       <x:c r="D500" s="9"/>
       <x:c r="E500" s="9"/>
+      <x:c r="F500" s="25"/>
+      <x:c r="G500" s="25"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="D2:D500">
+      <x:formula1>"AUTO,FCO,FNO,OGU"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E2:E500">
+      <x:formula1>"Pronaf B,Pronaf B para mulheres,Pronaf B agroecológico/orgânico,Pronaf B quintais produtivos"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re564b99b99b84191"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdf2a2a93db34ddc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3861,79 +4943,95 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="85" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="86" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A1" s="14" t="str">
+      <x:c r="A1" s="31" t="str">
         <x:v>MODELO DE CONSULTA EM LISTA</x:v>
       </x:c>
-      <x:c r="B1" s="14" t="str">
+      <x:c r="B1" s="31" t="str">
         <x:v>Preencha somente a aba Consultas</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="15" t="str">
+      <x:c r="A2" s="35" t="str">
         <x:v>CPF_CNPJ</x:v>
       </x:c>
-      <x:c r="B2" s="16" t="str">
+      <x:c r="B2" s="37" t="str">
         <x:v>Obrigatório. Pode ser digitado com ou sem pontos, barra e traço.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="15" t="str">
+      <x:c r="A3" s="35" t="str">
         <x:v>CAR</x:v>
       </x:c>
-      <x:c r="B3" s="16" t="str">
+      <x:c r="B3" s="37" t="str">
         <x:v>Opcional. Se ficar vazio, todos os CARs distintos encontrados para o CPF/CNPJ serão analisados.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="15" t="str">
+      <x:c r="A4" s="35" t="str">
         <x:v>PROPRIETARIO_POSSUIDOR</x:v>
       </x:c>
-      <x:c r="B4" s="16" t="str">
+      <x:c r="B4" s="37" t="str">
         <x:v>Opcional. Use quando o proprietário/possuidor for diferente do CPF/CNPJ consultado.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="15" t="str">
+      <x:c r="A5" s="35" t="str">
+        <x:v>FONTE_RECURSOS</x:v>
+      </x:c>
+      <x:c r="B5" s="37" t="str">
+        <x:v>Obrigatório. Escolha AUTO para sugestão pela UF do CAR ou informe FCO, FNO ou OGU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="35" t="str">
+        <x:v>LINHA_CREDITO</x:v>
+      </x:c>
+      <x:c r="B6" s="37" t="str">
+        <x:v>Obrigatório. Selecione uma das linhas Pronaf B disponíveis na lista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="35" t="str">
         <x:v>REFERENCIA_INTERNA</x:v>
       </x:c>
-      <x:c r="B5" s="16" t="str">
+      <x:c r="B7" s="37" t="str">
         <x:v>Opcional. Número da proposta, contrato ou outro código usado pela instituição.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="15" t="str">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="35" t="str">
         <x:v>OBSERVACAO</x:v>
       </x:c>
-      <x:c r="B6" s="16" t="str">
+      <x:c r="B8" s="37" t="str">
         <x:v>Opcional. Texto que deverá acompanhar o item no relatório consolidado.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="15" t="str">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="35" t="str">
         <x:v>Exemplo CPF</x:v>
       </x:c>
-      <x:c r="B7" s="16" t="str">
+      <x:c r="B9" s="37" t="str">
         <x:v>123.456.789-00</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="15" t="str">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="35" t="str">
         <x:v>Exemplo CAR</x:v>
       </x:c>
-      <x:c r="B8" s="16" t="str">
+      <x:c r="B10" s="37" t="str">
         <x:v>RO-1101500-XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="15" t="str">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="35" t="str">
         <x:v>Saída</x:v>
       </x:c>
-      <x:c r="B9" s="16" t="str">
-        <x:v>Um PDF consolidado, agrupado por CPF/CNPJ, e um JSON de auditoria.</x:v>
+      <x:c r="B11" s="37" t="str">
+        <x:v>Um PDF consolidado de pré-análise, agrupado por CPF/CNPJ, e um JSON de auditoria.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>